<commit_message>
chore: update currency rates for 2026-09-14
</commit_message>
<xml_diff>
--- a/data/rates.xlsx
+++ b/data/rates.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3221"/>
+  <dimension ref="A1:E3247"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -80943,6 +80943,656 @@
         </is>
       </c>
     </row>
+    <row r="3222">
+      <c r="A3222" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B3222" t="inlineStr">
+        <is>
+          <t>CNY/SGD</t>
+        </is>
+      </c>
+      <c r="C3222" t="n">
+        <v>0.189395</v>
+      </c>
+      <c r="D3222" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3222" t="inlineStr">
+        <is>
+          <t>2026-09-14 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3223">
+      <c r="A3223" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B3223" t="inlineStr">
+        <is>
+          <t>CNY/USD</t>
+        </is>
+      </c>
+      <c r="C3223" t="n">
+        <v>0.149066</v>
+      </c>
+      <c r="D3223" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3223" t="inlineStr">
+        <is>
+          <t>2026-09-14 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3224">
+      <c r="A3224" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B3224" t="inlineStr">
+        <is>
+          <t>EUR/AED</t>
+        </is>
+      </c>
+      <c r="C3224" t="n">
+        <v>4.258835</v>
+      </c>
+      <c r="D3224" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3224" t="inlineStr">
+        <is>
+          <t>2026-09-14 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3225">
+      <c r="A3225" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B3225" t="inlineStr">
+        <is>
+          <t>EUR/ARS</t>
+        </is>
+      </c>
+      <c r="C3225" t="n">
+        <v>1750.972424</v>
+      </c>
+      <c r="D3225" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3225" t="inlineStr">
+        <is>
+          <t>2026-09-14 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3226">
+      <c r="A3226" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B3226" t="inlineStr">
+        <is>
+          <t>EUR/BRL</t>
+        </is>
+      </c>
+      <c r="C3226" t="n">
+        <v>5.9564</v>
+      </c>
+      <c r="D3226" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3226" t="inlineStr">
+        <is>
+          <t>2026-09-14 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3227">
+      <c r="A3227" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B3227" t="inlineStr">
+        <is>
+          <t>EUR/CHF</t>
+        </is>
+      </c>
+      <c r="C3227" t="n">
+        <v>0.9431</v>
+      </c>
+      <c r="D3227" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3227" t="inlineStr">
+        <is>
+          <t>2026-09-14 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3228">
+      <c r="A3228" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B3228" t="inlineStr">
+        <is>
+          <t>EUR/CLP</t>
+        </is>
+      </c>
+      <c r="C3228" t="n">
+        <v>1091.066415</v>
+      </c>
+      <c r="D3228" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3228" t="inlineStr">
+        <is>
+          <t>2026-09-14 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3229">
+      <c r="A3229" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B3229" t="inlineStr">
+        <is>
+          <t>EUR/CNY</t>
+        </is>
+      </c>
+      <c r="C3229" t="n">
+        <v>7.7489</v>
+      </c>
+      <c r="D3229" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3229" t="inlineStr">
+        <is>
+          <t>2026-09-14 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3230">
+      <c r="A3230" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B3230" t="inlineStr">
+        <is>
+          <t>EUR/COP</t>
+        </is>
+      </c>
+      <c r="C3230" t="n">
+        <v>3576.54701</v>
+      </c>
+      <c r="D3230" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3230" t="inlineStr">
+        <is>
+          <t>2026-09-14 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3231">
+      <c r="A3231" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B3231" t="inlineStr">
+        <is>
+          <t>EUR/DKK</t>
+        </is>
+      </c>
+      <c r="C3231" t="n">
+        <v>7.4753</v>
+      </c>
+      <c r="D3231" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3231" t="inlineStr">
+        <is>
+          <t>2026-09-14 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3232">
+      <c r="A3232" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B3232" t="inlineStr">
+        <is>
+          <t>EUR/GBP</t>
+        </is>
+      </c>
+      <c r="C3232" t="n">
+        <v>0.85598</v>
+      </c>
+      <c r="D3232" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3232" t="inlineStr">
+        <is>
+          <t>2026-09-14 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3233">
+      <c r="A3233" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B3233" t="inlineStr">
+        <is>
+          <t>EUR/HKD</t>
+        </is>
+      </c>
+      <c r="C3233" t="n">
+        <v>9.059900000000001</v>
+      </c>
+      <c r="D3233" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3233" t="inlineStr">
+        <is>
+          <t>2026-09-14 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3234">
+      <c r="A3234" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B3234" t="inlineStr">
+        <is>
+          <t>EUR/IDR</t>
+        </is>
+      </c>
+      <c r="C3234" t="n">
+        <v>20398.66</v>
+      </c>
+      <c r="D3234" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3234" t="inlineStr">
+        <is>
+          <t>2026-09-14 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3235">
+      <c r="A3235" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B3235" t="inlineStr">
+        <is>
+          <t>EUR/ILS</t>
+        </is>
+      </c>
+      <c r="C3235" t="n">
+        <v>3.527</v>
+      </c>
+      <c r="D3235" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3235" t="inlineStr">
+        <is>
+          <t>2026-09-14 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3236">
+      <c r="A3236" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B3236" t="inlineStr">
+        <is>
+          <t>EUR/JPY</t>
+        </is>
+      </c>
+      <c r="C3236" t="n">
+        <v>178.52</v>
+      </c>
+      <c r="D3236" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3236" t="inlineStr">
+        <is>
+          <t>2026-09-14 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3237">
+      <c r="A3237" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B3237" t="inlineStr">
+        <is>
+          <t>EUR/KRW</t>
+        </is>
+      </c>
+      <c r="C3237" t="n">
+        <v>1555.04</v>
+      </c>
+      <c r="D3237" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3237" t="inlineStr">
+        <is>
+          <t>2026-09-14 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3238">
+      <c r="A3238" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B3238" t="inlineStr">
+        <is>
+          <t>EUR/MAD</t>
+        </is>
+      </c>
+      <c r="C3238" t="n">
+        <v>10.90371</v>
+      </c>
+      <c r="D3238" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3238" t="inlineStr">
+        <is>
+          <t>2026-09-14 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3239">
+      <c r="A3239" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B3239" t="inlineStr">
+        <is>
+          <t>EUR/PEN</t>
+        </is>
+      </c>
+      <c r="C3239" t="n">
+        <v>3.891723</v>
+      </c>
+      <c r="D3239" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3239" t="inlineStr">
+        <is>
+          <t>2026-09-14 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3240">
+      <c r="A3240" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B3240" t="inlineStr">
+        <is>
+          <t>EUR/PHP</t>
+        </is>
+      </c>
+      <c r="C3240" t="n">
+        <v>72.619</v>
+      </c>
+      <c r="D3240" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3240" t="inlineStr">
+        <is>
+          <t>2026-09-14 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3241">
+      <c r="A3241" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B3241" t="inlineStr">
+        <is>
+          <t>EUR/RUB</t>
+        </is>
+      </c>
+      <c r="C3241" t="n">
+        <v>97.648713</v>
+      </c>
+      <c r="D3241" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3241" t="inlineStr">
+        <is>
+          <t>2026-09-14 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3242">
+      <c r="A3242" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B3242" t="inlineStr">
+        <is>
+          <t>EUR/SAR</t>
+        </is>
+      </c>
+      <c r="C3242" t="n">
+        <v>4.348708</v>
+      </c>
+      <c r="D3242" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3242" t="inlineStr">
+        <is>
+          <t>2026-09-14 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3243">
+      <c r="A3243" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B3243" t="inlineStr">
+        <is>
+          <t>EUR/SEK</t>
+        </is>
+      </c>
+      <c r="C3243" t="n">
+        <v>11.281</v>
+      </c>
+      <c r="D3243" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3243" t="inlineStr">
+        <is>
+          <t>2026-09-14 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3244">
+      <c r="A3244" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B3244" t="inlineStr">
+        <is>
+          <t>EUR/SGD</t>
+        </is>
+      </c>
+      <c r="C3244" t="n">
+        <v>1.4676</v>
+      </c>
+      <c r="D3244" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3244" t="inlineStr">
+        <is>
+          <t>2026-09-14 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3245">
+      <c r="A3245" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B3245" t="inlineStr">
+        <is>
+          <t>EUR/THB</t>
+        </is>
+      </c>
+      <c r="C3245" t="n">
+        <v>38.407</v>
+      </c>
+      <c r="D3245" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3245" t="inlineStr">
+        <is>
+          <t>2026-09-14 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3246">
+      <c r="A3246" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B3246" t="inlineStr">
+        <is>
+          <t>EUR/TRY</t>
+        </is>
+      </c>
+      <c r="C3246" t="n">
+        <v>56.1636</v>
+      </c>
+      <c r="D3246" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3246" t="inlineStr">
+        <is>
+          <t>2026-09-14 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3247">
+      <c r="A3247" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B3247" t="inlineStr">
+        <is>
+          <t>EUR/USD</t>
+        </is>
+      </c>
+      <c r="C3247" t="n">
+        <v>1.1551</v>
+      </c>
+      <c r="D3247" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3247" t="inlineStr">
+        <is>
+          <t>2026-09-14 07:30 CET</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update currency rates for 2026-09-15
</commit_message>
<xml_diff>
--- a/data/rates.xlsx
+++ b/data/rates.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3247"/>
+  <dimension ref="A1:E3273"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -81593,6 +81593,656 @@
         </is>
       </c>
     </row>
+    <row r="3248">
+      <c r="A3248" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B3248" t="inlineStr">
+        <is>
+          <t>CNY/SGD</t>
+        </is>
+      </c>
+      <c r="C3248" t="n">
+        <v>0.189595</v>
+      </c>
+      <c r="D3248" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3248" t="inlineStr">
+        <is>
+          <t>2026-09-15 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3249">
+      <c r="A3249" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B3249" t="inlineStr">
+        <is>
+          <t>CNY/USD</t>
+        </is>
+      </c>
+      <c r="C3249" t="n">
+        <v>0.148998</v>
+      </c>
+      <c r="D3249" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3249" t="inlineStr">
+        <is>
+          <t>2026-09-15 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3250">
+      <c r="A3250" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B3250" t="inlineStr">
+        <is>
+          <t>EUR/AED</t>
+        </is>
+      </c>
+      <c r="C3250" t="n">
+        <v>4.243878</v>
+      </c>
+      <c r="D3250" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3250" t="inlineStr">
+        <is>
+          <t>2026-09-15 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3251">
+      <c r="A3251" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B3251" t="inlineStr">
+        <is>
+          <t>EUR/ARS</t>
+        </is>
+      </c>
+      <c r="C3251" t="n">
+        <v>1745.301482</v>
+      </c>
+      <c r="D3251" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3251" t="inlineStr">
+        <is>
+          <t>2026-09-15 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3252">
+      <c r="A3252" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B3252" t="inlineStr">
+        <is>
+          <t>EUR/BRL</t>
+        </is>
+      </c>
+      <c r="C3252" t="n">
+        <v>5.944</v>
+      </c>
+      <c r="D3252" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3252" t="inlineStr">
+        <is>
+          <t>2026-09-15 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3253">
+      <c r="A3253" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B3253" t="inlineStr">
+        <is>
+          <t>EUR/CHF</t>
+        </is>
+      </c>
+      <c r="C3253" t="n">
+        <v>0.9441000000000001</v>
+      </c>
+      <c r="D3253" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3253" t="inlineStr">
+        <is>
+          <t>2026-09-15 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3254">
+      <c r="A3254" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B3254" t="inlineStr">
+        <is>
+          <t>EUR/CLP</t>
+        </is>
+      </c>
+      <c r="C3254" t="n">
+        <v>1087.055258</v>
+      </c>
+      <c r="D3254" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3254" t="inlineStr">
+        <is>
+          <t>2026-09-15 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3255">
+      <c r="A3255" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B3255" t="inlineStr">
+        <is>
+          <t>EUR/CNY</t>
+        </is>
+      </c>
+      <c r="C3255" t="n">
+        <v>7.7444</v>
+      </c>
+      <c r="D3255" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3255" t="inlineStr">
+        <is>
+          <t>2026-09-15 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3256">
+      <c r="A3256" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B3256" t="inlineStr">
+        <is>
+          <t>EUR/COP</t>
+        </is>
+      </c>
+      <c r="C3256" t="n">
+        <v>3557.366489</v>
+      </c>
+      <c r="D3256" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3256" t="inlineStr">
+        <is>
+          <t>2026-09-15 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3257">
+      <c r="A3257" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B3257" t="inlineStr">
+        <is>
+          <t>EUR/DKK</t>
+        </is>
+      </c>
+      <c r="C3257" t="n">
+        <v>7.4752</v>
+      </c>
+      <c r="D3257" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3257" t="inlineStr">
+        <is>
+          <t>2026-09-15 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3258">
+      <c r="A3258" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B3258" t="inlineStr">
+        <is>
+          <t>EUR/GBP</t>
+        </is>
+      </c>
+      <c r="C3258" t="n">
+        <v>0.8558</v>
+      </c>
+      <c r="D3258" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3258" t="inlineStr">
+        <is>
+          <t>2026-09-15 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3259">
+      <c r="A3259" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B3259" t="inlineStr">
+        <is>
+          <t>EUR/HKD</t>
+        </is>
+      </c>
+      <c r="C3259" t="n">
+        <v>9.0518</v>
+      </c>
+      <c r="D3259" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3259" t="inlineStr">
+        <is>
+          <t>2026-09-15 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3260">
+      <c r="A3260" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B3260" t="inlineStr">
+        <is>
+          <t>EUR/IDR</t>
+        </is>
+      </c>
+      <c r="C3260" t="n">
+        <v>20420.4</v>
+      </c>
+      <c r="D3260" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3260" t="inlineStr">
+        <is>
+          <t>2026-09-15 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3261">
+      <c r="A3261" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B3261" t="inlineStr">
+        <is>
+          <t>EUR/ILS</t>
+        </is>
+      </c>
+      <c r="C3261" t="n">
+        <v>3.5093</v>
+      </c>
+      <c r="D3261" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3261" t="inlineStr">
+        <is>
+          <t>2026-09-15 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3262">
+      <c r="A3262" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B3262" t="inlineStr">
+        <is>
+          <t>EUR/JPY</t>
+        </is>
+      </c>
+      <c r="C3262" t="n">
+        <v>178.86</v>
+      </c>
+      <c r="D3262" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3262" t="inlineStr">
+        <is>
+          <t>2026-09-15 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3263">
+      <c r="A3263" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B3263" t="inlineStr">
+        <is>
+          <t>EUR/KRW</t>
+        </is>
+      </c>
+      <c r="C3263" t="n">
+        <v>1568.32</v>
+      </c>
+      <c r="D3263" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3263" t="inlineStr">
+        <is>
+          <t>2026-09-15 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3264">
+      <c r="A3264" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B3264" t="inlineStr">
+        <is>
+          <t>EUR/MAD</t>
+        </is>
+      </c>
+      <c r="C3264" t="n">
+        <v>10.9218</v>
+      </c>
+      <c r="D3264" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3264" t="inlineStr">
+        <is>
+          <t>2026-09-15 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3265">
+      <c r="A3265" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B3265" t="inlineStr">
+        <is>
+          <t>EUR/PEN</t>
+        </is>
+      </c>
+      <c r="C3265" t="n">
+        <v>3.889873</v>
+      </c>
+      <c r="D3265" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3265" t="inlineStr">
+        <is>
+          <t>2026-09-15 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3266">
+      <c r="A3266" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B3266" t="inlineStr">
+        <is>
+          <t>EUR/PHP</t>
+        </is>
+      </c>
+      <c r="C3266" t="n">
+        <v>72.467</v>
+      </c>
+      <c r="D3266" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3266" t="inlineStr">
+        <is>
+          <t>2026-09-15 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3267">
+      <c r="A3267" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B3267" t="inlineStr">
+        <is>
+          <t>EUR/RUB</t>
+        </is>
+      </c>
+      <c r="C3267" t="n">
+        <v>97.25535000000001</v>
+      </c>
+      <c r="D3267" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3267" t="inlineStr">
+        <is>
+          <t>2026-09-15 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3268">
+      <c r="A3268" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B3268" t="inlineStr">
+        <is>
+          <t>EUR/SAR</t>
+        </is>
+      </c>
+      <c r="C3268" t="n">
+        <v>4.333435</v>
+      </c>
+      <c r="D3268" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3268" t="inlineStr">
+        <is>
+          <t>2026-09-15 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3269">
+      <c r="A3269" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B3269" t="inlineStr">
+        <is>
+          <t>EUR/SEK</t>
+        </is>
+      </c>
+      <c r="C3269" t="n">
+        <v>11.274</v>
+      </c>
+      <c r="D3269" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3269" t="inlineStr">
+        <is>
+          <t>2026-09-15 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3270">
+      <c r="A3270" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B3270" t="inlineStr">
+        <is>
+          <t>EUR/SGD</t>
+        </is>
+      </c>
+      <c r="C3270" t="n">
+        <v>1.4683</v>
+      </c>
+      <c r="D3270" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3270" t="inlineStr">
+        <is>
+          <t>2026-09-15 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3271">
+      <c r="A3271" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B3271" t="inlineStr">
+        <is>
+          <t>EUR/THB</t>
+        </is>
+      </c>
+      <c r="C3271" t="n">
+        <v>38.419</v>
+      </c>
+      <c r="D3271" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3271" t="inlineStr">
+        <is>
+          <t>2026-09-15 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3272">
+      <c r="A3272" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B3272" t="inlineStr">
+        <is>
+          <t>EUR/TRY</t>
+        </is>
+      </c>
+      <c r="C3272" t="n">
+        <v>56.1255</v>
+      </c>
+      <c r="D3272" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3272" t="inlineStr">
+        <is>
+          <t>2026-09-15 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3273">
+      <c r="A3273" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B3273" t="inlineStr">
+        <is>
+          <t>EUR/USD</t>
+        </is>
+      </c>
+      <c r="C3273" t="n">
+        <v>1.1539</v>
+      </c>
+      <c r="D3273" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3273" t="inlineStr">
+        <is>
+          <t>2026-09-15 07:30 CET</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update currency rates for 2026-09-16
</commit_message>
<xml_diff>
--- a/data/rates.xlsx
+++ b/data/rates.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3273"/>
+  <dimension ref="A1:E3299"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -82243,6 +82243,656 @@
         </is>
       </c>
     </row>
+    <row r="3274">
+      <c r="A3274" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B3274" t="inlineStr">
+        <is>
+          <t>CNY/SGD</t>
+        </is>
+      </c>
+      <c r="C3274" t="n">
+        <v>0.189842</v>
+      </c>
+      <c r="D3274" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3274" t="inlineStr">
+        <is>
+          <t>2026-09-16 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3275">
+      <c r="A3275" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B3275" t="inlineStr">
+        <is>
+          <t>CNY/USD</t>
+        </is>
+      </c>
+      <c r="C3275" t="n">
+        <v>0.149095</v>
+      </c>
+      <c r="D3275" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3275" t="inlineStr">
+        <is>
+          <t>2026-09-16 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3276">
+      <c r="A3276" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B3276" t="inlineStr">
+        <is>
+          <t>EUR/AED</t>
+        </is>
+      </c>
+      <c r="C3276" t="n">
+        <v>4.23724</v>
+      </c>
+      <c r="D3276" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3276" t="inlineStr">
+        <is>
+          <t>2026-09-16 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3277">
+      <c r="A3277" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B3277" t="inlineStr">
+        <is>
+          <t>EUR/ARS</t>
+        </is>
+      </c>
+      <c r="C3277" t="n">
+        <v>1738.374521</v>
+      </c>
+      <c r="D3277" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3277" t="inlineStr">
+        <is>
+          <t>2026-09-16 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3278">
+      <c r="A3278" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B3278" t="inlineStr">
+        <is>
+          <t>EUR/BRL</t>
+        </is>
+      </c>
+      <c r="C3278" t="n">
+        <v>5.9368</v>
+      </c>
+      <c r="D3278" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3278" t="inlineStr">
+        <is>
+          <t>2026-09-16 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3279">
+      <c r="A3279" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B3279" t="inlineStr">
+        <is>
+          <t>EUR/CHF</t>
+        </is>
+      </c>
+      <c r="C3279" t="n">
+        <v>0.9449</v>
+      </c>
+      <c r="D3279" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3279" t="inlineStr">
+        <is>
+          <t>2026-09-16 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3280">
+      <c r="A3280" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B3280" t="inlineStr">
+        <is>
+          <t>EUR/CLP</t>
+        </is>
+      </c>
+      <c r="C3280" t="n">
+        <v>1104.232785</v>
+      </c>
+      <c r="D3280" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3280" t="inlineStr">
+        <is>
+          <t>2026-09-16 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3281">
+      <c r="A3281" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B3281" t="inlineStr">
+        <is>
+          <t>EUR/CNY</t>
+        </is>
+      </c>
+      <c r="C3281" t="n">
+        <v>7.738</v>
+      </c>
+      <c r="D3281" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3281" t="inlineStr">
+        <is>
+          <t>2026-09-16 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3282">
+      <c r="A3282" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B3282" t="inlineStr">
+        <is>
+          <t>EUR/COP</t>
+        </is>
+      </c>
+      <c r="C3282" t="n">
+        <v>3581.327122</v>
+      </c>
+      <c r="D3282" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3282" t="inlineStr">
+        <is>
+          <t>2026-09-16 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3283">
+      <c r="A3283" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B3283" t="inlineStr">
+        <is>
+          <t>EUR/DKK</t>
+        </is>
+      </c>
+      <c r="C3283" t="n">
+        <v>7.4755</v>
+      </c>
+      <c r="D3283" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3283" t="inlineStr">
+        <is>
+          <t>2026-09-16 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3284">
+      <c r="A3284" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B3284" t="inlineStr">
+        <is>
+          <t>EUR/GBP</t>
+        </is>
+      </c>
+      <c r="C3284" t="n">
+        <v>0.8574000000000001</v>
+      </c>
+      <c r="D3284" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3284" t="inlineStr">
+        <is>
+          <t>2026-09-16 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3285">
+      <c r="A3285" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B3285" t="inlineStr">
+        <is>
+          <t>EUR/HKD</t>
+        </is>
+      </c>
+      <c r="C3285" t="n">
+        <v>9.050700000000001</v>
+      </c>
+      <c r="D3285" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3285" t="inlineStr">
+        <is>
+          <t>2026-09-16 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3286">
+      <c r="A3286" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B3286" t="inlineStr">
+        <is>
+          <t>EUR/IDR</t>
+        </is>
+      </c>
+      <c r="C3286" t="n">
+        <v>20386.17</v>
+      </c>
+      <c r="D3286" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3286" t="inlineStr">
+        <is>
+          <t>2026-09-16 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3287">
+      <c r="A3287" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B3287" t="inlineStr">
+        <is>
+          <t>EUR/ILS</t>
+        </is>
+      </c>
+      <c r="C3287" t="n">
+        <v>3.4971</v>
+      </c>
+      <c r="D3287" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3287" t="inlineStr">
+        <is>
+          <t>2026-09-16 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3288">
+      <c r="A3288" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B3288" t="inlineStr">
+        <is>
+          <t>EUR/JPY</t>
+        </is>
+      </c>
+      <c r="C3288" t="n">
+        <v>178.88</v>
+      </c>
+      <c r="D3288" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3288" t="inlineStr">
+        <is>
+          <t>2026-09-16 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3289">
+      <c r="A3289" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B3289" t="inlineStr">
+        <is>
+          <t>EUR/KRW</t>
+        </is>
+      </c>
+      <c r="C3289" t="n">
+        <v>1578.03</v>
+      </c>
+      <c r="D3289" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3289" t="inlineStr">
+        <is>
+          <t>2026-09-16 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3290">
+      <c r="A3290" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B3290" t="inlineStr">
+        <is>
+          <t>EUR/MAD</t>
+        </is>
+      </c>
+      <c r="C3290" t="n">
+        <v>10.938862</v>
+      </c>
+      <c r="D3290" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3290" t="inlineStr">
+        <is>
+          <t>2026-09-16 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3291">
+      <c r="A3291" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B3291" t="inlineStr">
+        <is>
+          <t>EUR/PEN</t>
+        </is>
+      </c>
+      <c r="C3291" t="n">
+        <v>3.883754</v>
+      </c>
+      <c r="D3291" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3291" t="inlineStr">
+        <is>
+          <t>2026-09-16 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3292">
+      <c r="A3292" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B3292" t="inlineStr">
+        <is>
+          <t>EUR/PHP</t>
+        </is>
+      </c>
+      <c r="C3292" t="n">
+        <v>72.37</v>
+      </c>
+      <c r="D3292" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3292" t="inlineStr">
+        <is>
+          <t>2026-09-16 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3293">
+      <c r="A3293" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B3293" t="inlineStr">
+        <is>
+          <t>EUR/RUB</t>
+        </is>
+      </c>
+      <c r="C3293" t="n">
+        <v>97.28895900000001</v>
+      </c>
+      <c r="D3293" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3293" t="inlineStr">
+        <is>
+          <t>2026-09-16 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3294">
+      <c r="A3294" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B3294" t="inlineStr">
+        <is>
+          <t>EUR/SAR</t>
+        </is>
+      </c>
+      <c r="C3294" t="n">
+        <v>4.326658</v>
+      </c>
+      <c r="D3294" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3294" t="inlineStr">
+        <is>
+          <t>2026-09-16 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3295">
+      <c r="A3295" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B3295" t="inlineStr">
+        <is>
+          <t>EUR/SEK</t>
+        </is>
+      </c>
+      <c r="C3295" t="n">
+        <v>11.2875</v>
+      </c>
+      <c r="D3295" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3295" t="inlineStr">
+        <is>
+          <t>2026-09-16 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3296">
+      <c r="A3296" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B3296" t="inlineStr">
+        <is>
+          <t>EUR/SGD</t>
+        </is>
+      </c>
+      <c r="C3296" t="n">
+        <v>1.469</v>
+      </c>
+      <c r="D3296" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3296" t="inlineStr">
+        <is>
+          <t>2026-09-16 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3297">
+      <c r="A3297" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B3297" t="inlineStr">
+        <is>
+          <t>EUR/THB</t>
+        </is>
+      </c>
+      <c r="C3297" t="n">
+        <v>38.361</v>
+      </c>
+      <c r="D3297" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3297" t="inlineStr">
+        <is>
+          <t>2026-09-16 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3298">
+      <c r="A3298" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B3298" t="inlineStr">
+        <is>
+          <t>EUR/TRY</t>
+        </is>
+      </c>
+      <c r="C3298" t="n">
+        <v>56.136</v>
+      </c>
+      <c r="D3298" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3298" t="inlineStr">
+        <is>
+          <t>2026-09-16 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3299">
+      <c r="A3299" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B3299" t="inlineStr">
+        <is>
+          <t>EUR/USD</t>
+        </is>
+      </c>
+      <c r="C3299" t="n">
+        <v>1.1537</v>
+      </c>
+      <c r="D3299" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3299" t="inlineStr">
+        <is>
+          <t>2026-09-16 07:30 CET</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update currency rates for 2026-09-17
</commit_message>
<xml_diff>
--- a/data/rates.xlsx
+++ b/data/rates.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3299"/>
+  <dimension ref="A1:E3325"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -82893,6 +82893,656 @@
         </is>
       </c>
     </row>
+    <row r="3300">
+      <c r="A3300" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B3300" t="inlineStr">
+        <is>
+          <t>CNY/SGD</t>
+        </is>
+      </c>
+      <c r="C3300" t="n">
+        <v>0.190134</v>
+      </c>
+      <c r="D3300" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3300" t="inlineStr">
+        <is>
+          <t>2026-09-17 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3301">
+      <c r="A3301" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B3301" t="inlineStr">
+        <is>
+          <t>CNY/USD</t>
+        </is>
+      </c>
+      <c r="C3301" t="n">
+        <v>0.149086</v>
+      </c>
+      <c r="D3301" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3301" t="inlineStr">
+        <is>
+          <t>2026-09-17 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3302">
+      <c r="A3302" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B3302" t="inlineStr">
+        <is>
+          <t>EUR/AED</t>
+        </is>
+      </c>
+      <c r="C3302" t="n">
+        <v>4.224639</v>
+      </c>
+      <c r="D3302" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3302" t="inlineStr">
+        <is>
+          <t>2026-09-17 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3303">
+      <c r="A3303" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B3303" t="inlineStr">
+        <is>
+          <t>EUR/ARS</t>
+        </is>
+      </c>
+      <c r="C3303" t="n">
+        <v>1735.990723</v>
+      </c>
+      <c r="D3303" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3303" t="inlineStr">
+        <is>
+          <t>2026-09-17 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3304">
+      <c r="A3304" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B3304" t="inlineStr">
+        <is>
+          <t>EUR/BRL</t>
+        </is>
+      </c>
+      <c r="C3304" t="n">
+        <v>5.8905</v>
+      </c>
+      <c r="D3304" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3304" t="inlineStr">
+        <is>
+          <t>2026-09-17 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3305">
+      <c r="A3305" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B3305" t="inlineStr">
+        <is>
+          <t>EUR/CHF</t>
+        </is>
+      </c>
+      <c r="C3305" t="n">
+        <v>0.9466</v>
+      </c>
+      <c r="D3305" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3305" t="inlineStr">
+        <is>
+          <t>2026-09-17 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3306">
+      <c r="A3306" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B3306" t="inlineStr">
+        <is>
+          <t>EUR/CLP</t>
+        </is>
+      </c>
+      <c r="C3306" t="n">
+        <v>1102.918507</v>
+      </c>
+      <c r="D3306" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3306" t="inlineStr">
+        <is>
+          <t>2026-09-17 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3307">
+      <c r="A3307" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B3307" t="inlineStr">
+        <is>
+          <t>EUR/CNY</t>
+        </is>
+      </c>
+      <c r="C3307" t="n">
+        <v>7.7009</v>
+      </c>
+      <c r="D3307" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3307" t="inlineStr">
+        <is>
+          <t>2026-09-17 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3308">
+      <c r="A3308" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B3308" t="inlineStr">
+        <is>
+          <t>EUR/COP</t>
+        </is>
+      </c>
+      <c r="C3308" t="n">
+        <v>3595.507721</v>
+      </c>
+      <c r="D3308" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3308" t="inlineStr">
+        <is>
+          <t>2026-09-17 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3309">
+      <c r="A3309" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B3309" t="inlineStr">
+        <is>
+          <t>EUR/DKK</t>
+        </is>
+      </c>
+      <c r="C3309" t="n">
+        <v>7.4753</v>
+      </c>
+      <c r="D3309" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3309" t="inlineStr">
+        <is>
+          <t>2026-09-17 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3310">
+      <c r="A3310" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B3310" t="inlineStr">
+        <is>
+          <t>EUR/GBP</t>
+        </is>
+      </c>
+      <c r="C3310" t="n">
+        <v>0.8583</v>
+      </c>
+      <c r="D3310" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3310" t="inlineStr">
+        <is>
+          <t>2026-09-17 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3311">
+      <c r="A3311" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B3311" t="inlineStr">
+        <is>
+          <t>EUR/HKD</t>
+        </is>
+      </c>
+      <c r="C3311" t="n">
+        <v>9.007099999999999</v>
+      </c>
+      <c r="D3311" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3311" t="inlineStr">
+        <is>
+          <t>2026-09-17 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3312">
+      <c r="A3312" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B3312" t="inlineStr">
+        <is>
+          <t>EUR/IDR</t>
+        </is>
+      </c>
+      <c r="C3312" t="n">
+        <v>20352.48</v>
+      </c>
+      <c r="D3312" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3312" t="inlineStr">
+        <is>
+          <t>2026-09-17 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3313">
+      <c r="A3313" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B3313" t="inlineStr">
+        <is>
+          <t>EUR/ILS</t>
+        </is>
+      </c>
+      <c r="C3313" t="n">
+        <v>3.4825</v>
+      </c>
+      <c r="D3313" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3313" t="inlineStr">
+        <is>
+          <t>2026-09-17 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3314">
+      <c r="A3314" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B3314" t="inlineStr">
+        <is>
+          <t>EUR/JPY</t>
+        </is>
+      </c>
+      <c r="C3314" t="n">
+        <v>178.75</v>
+      </c>
+      <c r="D3314" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3314" t="inlineStr">
+        <is>
+          <t>2026-09-17 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3315">
+      <c r="A3315" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B3315" t="inlineStr">
+        <is>
+          <t>EUR/KRW</t>
+        </is>
+      </c>
+      <c r="C3315" t="n">
+        <v>1587.31</v>
+      </c>
+      <c r="D3315" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3315" t="inlineStr">
+        <is>
+          <t>2026-09-17 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3316">
+      <c r="A3316" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B3316" t="inlineStr">
+        <is>
+          <t>EUR/MAD</t>
+        </is>
+      </c>
+      <c r="C3316" t="n">
+        <v>10.911141</v>
+      </c>
+      <c r="D3316" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3316" t="inlineStr">
+        <is>
+          <t>2026-09-17 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3317">
+      <c r="A3317" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B3317" t="inlineStr">
+        <is>
+          <t>EUR/PEN</t>
+        </is>
+      </c>
+      <c r="C3317" t="n">
+        <v>3.873588</v>
+      </c>
+      <c r="D3317" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3317" t="inlineStr">
+        <is>
+          <t>2026-09-17 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3318">
+      <c r="A3318" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B3318" t="inlineStr">
+        <is>
+          <t>EUR/PHP</t>
+        </is>
+      </c>
+      <c r="C3318" t="n">
+        <v>72.006</v>
+      </c>
+      <c r="D3318" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3318" t="inlineStr">
+        <is>
+          <t>2026-09-17 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3319">
+      <c r="A3319" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B3319" t="inlineStr">
+        <is>
+          <t>EUR/RUB</t>
+        </is>
+      </c>
+      <c r="C3319" t="n">
+        <v>97.11441499999999</v>
+      </c>
+      <c r="D3319" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3319" t="inlineStr">
+        <is>
+          <t>2026-09-17 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3320">
+      <c r="A3320" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B3320" t="inlineStr">
+        <is>
+          <t>EUR/SAR</t>
+        </is>
+      </c>
+      <c r="C3320" t="n">
+        <v>4.313791</v>
+      </c>
+      <c r="D3320" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3320" t="inlineStr">
+        <is>
+          <t>2026-09-17 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3321">
+      <c r="A3321" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B3321" t="inlineStr">
+        <is>
+          <t>EUR/SEK</t>
+        </is>
+      </c>
+      <c r="C3321" t="n">
+        <v>11.2715</v>
+      </c>
+      <c r="D3321" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3321" t="inlineStr">
+        <is>
+          <t>2026-09-17 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3322">
+      <c r="A3322" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B3322" t="inlineStr">
+        <is>
+          <t>EUR/SGD</t>
+        </is>
+      </c>
+      <c r="C3322" t="n">
+        <v>1.4642</v>
+      </c>
+      <c r="D3322" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3322" t="inlineStr">
+        <is>
+          <t>2026-09-17 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3323">
+      <c r="A3323" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B3323" t="inlineStr">
+        <is>
+          <t>EUR/THB</t>
+        </is>
+      </c>
+      <c r="C3323" t="n">
+        <v>38.237</v>
+      </c>
+      <c r="D3323" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3323" t="inlineStr">
+        <is>
+          <t>2026-09-17 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3324">
+      <c r="A3324" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B3324" t="inlineStr">
+        <is>
+          <t>EUR/TRY</t>
+        </is>
+      </c>
+      <c r="C3324" t="n">
+        <v>55.8841</v>
+      </c>
+      <c r="D3324" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3324" t="inlineStr">
+        <is>
+          <t>2026-09-17 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3325">
+      <c r="A3325" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B3325" t="inlineStr">
+        <is>
+          <t>EUR/USD</t>
+        </is>
+      </c>
+      <c r="C3325" t="n">
+        <v>1.1481</v>
+      </c>
+      <c r="D3325" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3325" t="inlineStr">
+        <is>
+          <t>2026-09-17 07:30 CET</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update currency rates for 2026-09-18
</commit_message>
<xml_diff>
--- a/data/rates.xlsx
+++ b/data/rates.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3325"/>
+  <dimension ref="A1:E3351"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -83543,6 +83543,656 @@
         </is>
       </c>
     </row>
+    <row r="3326">
+      <c r="A3326" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B3326" t="inlineStr">
+        <is>
+          <t>CNY/SGD</t>
+        </is>
+      </c>
+      <c r="C3326" t="n">
+        <v>0.19088</v>
+      </c>
+      <c r="D3326" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3326" t="inlineStr">
+        <is>
+          <t>2026-09-18 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3327">
+      <c r="A3327" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B3327" t="inlineStr">
+        <is>
+          <t>CNY/USD</t>
+        </is>
+      </c>
+      <c r="C3327" t="n">
+        <v>0.149306</v>
+      </c>
+      <c r="D3327" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3327" t="inlineStr">
+        <is>
+          <t>2026-09-18 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3328">
+      <c r="A3328" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B3328" t="inlineStr">
+        <is>
+          <t>EUR/AED</t>
+        </is>
+      </c>
+      <c r="C3328" t="n">
+        <v>4.218208</v>
+      </c>
+      <c r="D3328" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3328" t="inlineStr">
+        <is>
+          <t>2026-09-18 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3329">
+      <c r="A3329" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B3329" t="inlineStr">
+        <is>
+          <t>EUR/ARS</t>
+        </is>
+      </c>
+      <c r="C3329" t="n">
+        <v>1734.378107</v>
+      </c>
+      <c r="D3329" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3329" t="inlineStr">
+        <is>
+          <t>2026-09-18 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3330">
+      <c r="A3330" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B3330" t="inlineStr">
+        <is>
+          <t>EUR/BRL</t>
+        </is>
+      </c>
+      <c r="C3330" t="n">
+        <v>5.8857</v>
+      </c>
+      <c r="D3330" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3330" t="inlineStr">
+        <is>
+          <t>2026-09-18 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3331">
+      <c r="A3331" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B3331" t="inlineStr">
+        <is>
+          <t>EUR/CHF</t>
+        </is>
+      </c>
+      <c r="C3331" t="n">
+        <v>0.9462</v>
+      </c>
+      <c r="D3331" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3331" t="inlineStr">
+        <is>
+          <t>2026-09-18 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3332">
+      <c r="A3332" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B3332" t="inlineStr">
+        <is>
+          <t>EUR/CLP</t>
+        </is>
+      </c>
+      <c r="C3332" t="n">
+        <v>1093.951975</v>
+      </c>
+      <c r="D3332" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3332" t="inlineStr">
+        <is>
+          <t>2026-09-18 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3333">
+      <c r="A3333" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B3333" t="inlineStr">
+        <is>
+          <t>EUR/CNY</t>
+        </is>
+      </c>
+      <c r="C3333" t="n">
+        <v>7.6755</v>
+      </c>
+      <c r="D3333" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3333" t="inlineStr">
+        <is>
+          <t>2026-09-18 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3334">
+      <c r="A3334" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B3334" t="inlineStr">
+        <is>
+          <t>EUR/COP</t>
+        </is>
+      </c>
+      <c r="C3334" t="n">
+        <v>3595.345846</v>
+      </c>
+      <c r="D3334" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3334" t="inlineStr">
+        <is>
+          <t>2026-09-18 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3335">
+      <c r="A3335" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B3335" t="inlineStr">
+        <is>
+          <t>EUR/DKK</t>
+        </is>
+      </c>
+      <c r="C3335" t="n">
+        <v>7.4754</v>
+      </c>
+      <c r="D3335" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3335" t="inlineStr">
+        <is>
+          <t>2026-09-18 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3336">
+      <c r="A3336" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B3336" t="inlineStr">
+        <is>
+          <t>EUR/GBP</t>
+        </is>
+      </c>
+      <c r="C3336" t="n">
+        <v>0.8588</v>
+      </c>
+      <c r="D3336" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3336" t="inlineStr">
+        <is>
+          <t>2026-09-18 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3337">
+      <c r="A3337" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B3337" t="inlineStr">
+        <is>
+          <t>EUR/HKD</t>
+        </is>
+      </c>
+      <c r="C3337" t="n">
+        <v>8.9903</v>
+      </c>
+      <c r="D3337" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3337" t="inlineStr">
+        <is>
+          <t>2026-09-18 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3338">
+      <c r="A3338" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B3338" t="inlineStr">
+        <is>
+          <t>EUR/IDR</t>
+        </is>
+      </c>
+      <c r="C3338" t="n">
+        <v>20424.81</v>
+      </c>
+      <c r="D3338" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3338" t="inlineStr">
+        <is>
+          <t>2026-09-18 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3339">
+      <c r="A3339" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B3339" t="inlineStr">
+        <is>
+          <t>EUR/ILS</t>
+        </is>
+      </c>
+      <c r="C3339" t="n">
+        <v>3.4812</v>
+      </c>
+      <c r="D3339" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3339" t="inlineStr">
+        <is>
+          <t>2026-09-18 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3340">
+      <c r="A3340" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B3340" t="inlineStr">
+        <is>
+          <t>EUR/JPY</t>
+        </is>
+      </c>
+      <c r="C3340" t="n">
+        <v>180.94</v>
+      </c>
+      <c r="D3340" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3340" t="inlineStr">
+        <is>
+          <t>2026-09-18 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3341">
+      <c r="A3341" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B3341" t="inlineStr">
+        <is>
+          <t>EUR/KRW</t>
+        </is>
+      </c>
+      <c r="C3341" t="n">
+        <v>1590.76</v>
+      </c>
+      <c r="D3341" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3341" t="inlineStr">
+        <is>
+          <t>2026-09-18 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3342">
+      <c r="A3342" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B3342" t="inlineStr">
+        <is>
+          <t>EUR/MAD</t>
+        </is>
+      </c>
+      <c r="C3342" t="n">
+        <v>10.901707</v>
+      </c>
+      <c r="D3342" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3342" t="inlineStr">
+        <is>
+          <t>2026-09-18 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3343">
+      <c r="A3343" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B3343" t="inlineStr">
+        <is>
+          <t>EUR/PEN</t>
+        </is>
+      </c>
+      <c r="C3343" t="n">
+        <v>3.867149</v>
+      </c>
+      <c r="D3343" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3343" t="inlineStr">
+        <is>
+          <t>2026-09-18 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3344">
+      <c r="A3344" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B3344" t="inlineStr">
+        <is>
+          <t>EUR/PHP</t>
+        </is>
+      </c>
+      <c r="C3344" t="n">
+        <v>71.97199999999999</v>
+      </c>
+      <c r="D3344" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3344" t="inlineStr">
+        <is>
+          <t>2026-09-18 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3345">
+      <c r="A3345" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B3345" t="inlineStr">
+        <is>
+          <t>EUR/RUB</t>
+        </is>
+      </c>
+      <c r="C3345" t="n">
+        <v>96.985207</v>
+      </c>
+      <c r="D3345" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3345" t="inlineStr">
+        <is>
+          <t>2026-09-18 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3346">
+      <c r="A3346" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B3346" t="inlineStr">
+        <is>
+          <t>EUR/SAR</t>
+        </is>
+      </c>
+      <c r="C3346" t="n">
+        <v>4.307224</v>
+      </c>
+      <c r="D3346" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3346" t="inlineStr">
+        <is>
+          <t>2026-09-18 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3347">
+      <c r="A3347" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B3347" t="inlineStr">
+        <is>
+          <t>EUR/SEK</t>
+        </is>
+      </c>
+      <c r="C3347" t="n">
+        <v>11.2915</v>
+      </c>
+      <c r="D3347" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3347" t="inlineStr">
+        <is>
+          <t>2026-09-18 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3348">
+      <c r="A3348" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B3348" t="inlineStr">
+        <is>
+          <t>EUR/SGD</t>
+        </is>
+      </c>
+      <c r="C3348" t="n">
+        <v>1.4651</v>
+      </c>
+      <c r="D3348" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3348" t="inlineStr">
+        <is>
+          <t>2026-09-18 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3349">
+      <c r="A3349" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B3349" t="inlineStr">
+        <is>
+          <t>EUR/THB</t>
+        </is>
+      </c>
+      <c r="C3349" t="n">
+        <v>38.225</v>
+      </c>
+      <c r="D3349" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3349" t="inlineStr">
+        <is>
+          <t>2026-09-18 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3350">
+      <c r="A3350" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B3350" t="inlineStr">
+        <is>
+          <t>EUR/TRY</t>
+        </is>
+      </c>
+      <c r="C3350" t="n">
+        <v>55.9077</v>
+      </c>
+      <c r="D3350" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3350" t="inlineStr">
+        <is>
+          <t>2026-09-18 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3351">
+      <c r="A3351" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B3351" t="inlineStr">
+        <is>
+          <t>EUR/USD</t>
+        </is>
+      </c>
+      <c r="C3351" t="n">
+        <v>1.146</v>
+      </c>
+      <c r="D3351" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3351" t="inlineStr">
+        <is>
+          <t>2026-09-18 07:30 CET</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update currency rates for 2026-09-21
</commit_message>
<xml_diff>
--- a/data/rates.xlsx
+++ b/data/rates.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3351"/>
+  <dimension ref="A1:E3377"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -84193,6 +84193,656 @@
         </is>
       </c>
     </row>
+    <row r="3352">
+      <c r="A3352" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B3352" t="inlineStr">
+        <is>
+          <t>CNY/SGD</t>
+        </is>
+      </c>
+      <c r="C3352" t="n">
+        <v>0.190394</v>
+      </c>
+      <c r="D3352" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3352" t="inlineStr">
+        <is>
+          <t>2026-09-21 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3353">
+      <c r="A3353" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B3353" t="inlineStr">
+        <is>
+          <t>CNY/USD</t>
+        </is>
+      </c>
+      <c r="C3353" t="n">
+        <v>0.149357</v>
+      </c>
+      <c r="D3353" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3353" t="inlineStr">
+        <is>
+          <t>2026-09-21 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3354">
+      <c r="A3354" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B3354" t="inlineStr">
+        <is>
+          <t>EUR/AED</t>
+        </is>
+      </c>
+      <c r="C3354" t="n">
+        <v>4.2145</v>
+      </c>
+      <c r="D3354" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3354" t="inlineStr">
+        <is>
+          <t>2026-09-21 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3355">
+      <c r="A3355" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B3355" t="inlineStr">
+        <is>
+          <t>EUR/ARS</t>
+        </is>
+      </c>
+      <c r="C3355" t="n">
+        <v>1735.528441</v>
+      </c>
+      <c r="D3355" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3355" t="inlineStr">
+        <is>
+          <t>2026-09-21 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3356">
+      <c r="A3356" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B3356" t="inlineStr">
+        <is>
+          <t>EUR/BRL</t>
+        </is>
+      </c>
+      <c r="C3356" t="n">
+        <v>5.892</v>
+      </c>
+      <c r="D3356" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3356" t="inlineStr">
+        <is>
+          <t>2026-09-21 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3357">
+      <c r="A3357" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B3357" t="inlineStr">
+        <is>
+          <t>EUR/CHF</t>
+        </is>
+      </c>
+      <c r="C3357" t="n">
+        <v>0.9438</v>
+      </c>
+      <c r="D3357" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3357" t="inlineStr">
+        <is>
+          <t>2026-09-21 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3358">
+      <c r="A3358" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B3358" t="inlineStr">
+        <is>
+          <t>EUR/CLP</t>
+        </is>
+      </c>
+      <c r="C3358" t="n">
+        <v>1103.376185</v>
+      </c>
+      <c r="D3358" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3358" t="inlineStr">
+        <is>
+          <t>2026-09-21 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3359">
+      <c r="A3359" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B3359" t="inlineStr">
+        <is>
+          <t>EUR/CNY</t>
+        </is>
+      </c>
+      <c r="C3359" t="n">
+        <v>7.693</v>
+      </c>
+      <c r="D3359" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3359" t="inlineStr">
+        <is>
+          <t>2026-09-21 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3360">
+      <c r="A3360" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B3360" t="inlineStr">
+        <is>
+          <t>EUR/COP</t>
+        </is>
+      </c>
+      <c r="C3360" t="n">
+        <v>3637.593026</v>
+      </c>
+      <c r="D3360" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3360" t="inlineStr">
+        <is>
+          <t>2026-09-21 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3361">
+      <c r="A3361" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B3361" t="inlineStr">
+        <is>
+          <t>EUR/DKK</t>
+        </is>
+      </c>
+      <c r="C3361" t="n">
+        <v>7.4755</v>
+      </c>
+      <c r="D3361" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3361" t="inlineStr">
+        <is>
+          <t>2026-09-21 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3362">
+      <c r="A3362" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B3362" t="inlineStr">
+        <is>
+          <t>EUR/GBP</t>
+        </is>
+      </c>
+      <c r="C3362" t="n">
+        <v>0.8578</v>
+      </c>
+      <c r="D3362" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3362" t="inlineStr">
+        <is>
+          <t>2026-09-21 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3363">
+      <c r="A3363" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B3363" t="inlineStr">
+        <is>
+          <t>EUR/HKD</t>
+        </is>
+      </c>
+      <c r="C3363" t="n">
+        <v>9.0144</v>
+      </c>
+      <c r="D3363" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3363" t="inlineStr">
+        <is>
+          <t>2026-09-21 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3364">
+      <c r="A3364" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B3364" t="inlineStr">
+        <is>
+          <t>EUR/IDR</t>
+        </is>
+      </c>
+      <c r="C3364" t="n">
+        <v>20532.06</v>
+      </c>
+      <c r="D3364" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3364" t="inlineStr">
+        <is>
+          <t>2026-09-21 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3365">
+      <c r="A3365" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B3365" t="inlineStr">
+        <is>
+          <t>EUR/ILS</t>
+        </is>
+      </c>
+      <c r="C3365" t="n">
+        <v>3.4602</v>
+      </c>
+      <c r="D3365" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3365" t="inlineStr">
+        <is>
+          <t>2026-09-21 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3366">
+      <c r="A3366" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B3366" t="inlineStr">
+        <is>
+          <t>EUR/JPY</t>
+        </is>
+      </c>
+      <c r="C3366" t="n">
+        <v>180.7</v>
+      </c>
+      <c r="D3366" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3366" t="inlineStr">
+        <is>
+          <t>2026-09-21 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3367">
+      <c r="A3367" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B3367" t="inlineStr">
+        <is>
+          <t>EUR/KRW</t>
+        </is>
+      </c>
+      <c r="C3367" t="n">
+        <v>1576.63</v>
+      </c>
+      <c r="D3367" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3367" t="inlineStr">
+        <is>
+          <t>2026-09-21 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3368">
+      <c r="A3368" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B3368" t="inlineStr">
+        <is>
+          <t>EUR/MAD</t>
+        </is>
+      </c>
+      <c r="C3368" t="n">
+        <v>10.93028</v>
+      </c>
+      <c r="D3368" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3368" t="inlineStr">
+        <is>
+          <t>2026-09-21 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3369">
+      <c r="A3369" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B3369" t="inlineStr">
+        <is>
+          <t>EUR/PEN</t>
+        </is>
+      </c>
+      <c r="C3369" t="n">
+        <v>3.873735</v>
+      </c>
+      <c r="D3369" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3369" t="inlineStr">
+        <is>
+          <t>2026-09-21 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3370">
+      <c r="A3370" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B3370" t="inlineStr">
+        <is>
+          <t>EUR/PHP</t>
+        </is>
+      </c>
+      <c r="C3370" t="n">
+        <v>72.151</v>
+      </c>
+      <c r="D3370" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3370" t="inlineStr">
+        <is>
+          <t>2026-09-21 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3371">
+      <c r="A3371" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B3371" t="inlineStr">
+        <is>
+          <t>EUR/RUB</t>
+        </is>
+      </c>
+      <c r="C3371" t="n">
+        <v>96.628974</v>
+      </c>
+      <c r="D3371" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3371" t="inlineStr">
+        <is>
+          <t>2026-09-21 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3372">
+      <c r="A3372" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B3372" t="inlineStr">
+        <is>
+          <t>EUR/SAR</t>
+        </is>
+      </c>
+      <c r="C3372" t="n">
+        <v>4.303438</v>
+      </c>
+      <c r="D3372" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3372" t="inlineStr">
+        <is>
+          <t>2026-09-21 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3373">
+      <c r="A3373" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B3373" t="inlineStr">
+        <is>
+          <t>EUR/SEK</t>
+        </is>
+      </c>
+      <c r="C3373" t="n">
+        <v>11.275</v>
+      </c>
+      <c r="D3373" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3373" t="inlineStr">
+        <is>
+          <t>2026-09-21 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3374">
+      <c r="A3374" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B3374" t="inlineStr">
+        <is>
+          <t>EUR/SGD</t>
+        </is>
+      </c>
+      <c r="C3374" t="n">
+        <v>1.4647</v>
+      </c>
+      <c r="D3374" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3374" t="inlineStr">
+        <is>
+          <t>2026-09-21 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3375">
+      <c r="A3375" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B3375" t="inlineStr">
+        <is>
+          <t>EUR/THB</t>
+        </is>
+      </c>
+      <c r="C3375" t="n">
+        <v>38.187</v>
+      </c>
+      <c r="D3375" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3375" t="inlineStr">
+        <is>
+          <t>2026-09-21 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3376">
+      <c r="A3376" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B3376" t="inlineStr">
+        <is>
+          <t>EUR/TRY</t>
+        </is>
+      </c>
+      <c r="C3376" t="n">
+        <v>56.0701</v>
+      </c>
+      <c r="D3376" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3376" t="inlineStr">
+        <is>
+          <t>2026-09-21 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3377">
+      <c r="A3377" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B3377" t="inlineStr">
+        <is>
+          <t>EUR/USD</t>
+        </is>
+      </c>
+      <c r="C3377" t="n">
+        <v>1.149</v>
+      </c>
+      <c r="D3377" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3377" t="inlineStr">
+        <is>
+          <t>2026-09-21 07:30 CET</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update currency rates for 2026-09-22
</commit_message>
<xml_diff>
--- a/data/rates.xlsx
+++ b/data/rates.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3377"/>
+  <dimension ref="A1:E3403"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -84843,6 +84843,656 @@
         </is>
       </c>
     </row>
+    <row r="3378">
+      <c r="A3378" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B3378" t="inlineStr">
+        <is>
+          <t>CNY/SGD</t>
+        </is>
+      </c>
+      <c r="C3378" t="n">
+        <v>0.190253</v>
+      </c>
+      <c r="D3378" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3378" t="inlineStr">
+        <is>
+          <t>2026-09-22 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3379">
+      <c r="A3379" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B3379" t="inlineStr">
+        <is>
+          <t>CNY/USD</t>
+        </is>
+      </c>
+      <c r="C3379" t="n">
+        <v>0.149252</v>
+      </c>
+      <c r="D3379" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3379" t="inlineStr">
+        <is>
+          <t>2026-09-22 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3380">
+      <c r="A3380" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B3380" t="inlineStr">
+        <is>
+          <t>EUR/AED</t>
+        </is>
+      </c>
+      <c r="C3380" t="n">
+        <v>4.21291</v>
+      </c>
+      <c r="D3380" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3380" t="inlineStr">
+        <is>
+          <t>2026-09-22 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3381">
+      <c r="A3381" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B3381" t="inlineStr">
+        <is>
+          <t>EUR/ARS</t>
+        </is>
+      </c>
+      <c r="C3381" t="n">
+        <v>1737.833713</v>
+      </c>
+      <c r="D3381" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3381" t="inlineStr">
+        <is>
+          <t>2026-09-22 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3382">
+      <c r="A3382" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B3382" t="inlineStr">
+        <is>
+          <t>EUR/BRL</t>
+        </is>
+      </c>
+      <c r="C3382" t="n">
+        <v>5.8726</v>
+      </c>
+      <c r="D3382" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3382" t="inlineStr">
+        <is>
+          <t>2026-09-22 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3383">
+      <c r="A3383" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B3383" t="inlineStr">
+        <is>
+          <t>EUR/CHF</t>
+        </is>
+      </c>
+      <c r="C3383" t="n">
+        <v>0.9393</v>
+      </c>
+      <c r="D3383" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3383" t="inlineStr">
+        <is>
+          <t>2026-09-22 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3384">
+      <c r="A3384" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B3384" t="inlineStr">
+        <is>
+          <t>EUR/CLP</t>
+        </is>
+      </c>
+      <c r="C3384" t="n">
+        <v>1101.707785</v>
+      </c>
+      <c r="D3384" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3384" t="inlineStr">
+        <is>
+          <t>2026-09-22 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3385">
+      <c r="A3385" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B3385" t="inlineStr">
+        <is>
+          <t>EUR/CNY</t>
+        </is>
+      </c>
+      <c r="C3385" t="n">
+        <v>7.6803</v>
+      </c>
+      <c r="D3385" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3385" t="inlineStr">
+        <is>
+          <t>2026-09-22 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3386">
+      <c r="A3386" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B3386" t="inlineStr">
+        <is>
+          <t>EUR/COP</t>
+        </is>
+      </c>
+      <c r="C3386" t="n">
+        <v>3647.936362</v>
+      </c>
+      <c r="D3386" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3386" t="inlineStr">
+        <is>
+          <t>2026-09-22 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3387">
+      <c r="A3387" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B3387" t="inlineStr">
+        <is>
+          <t>EUR/DKK</t>
+        </is>
+      </c>
+      <c r="C3387" t="n">
+        <v>7.4756</v>
+      </c>
+      <c r="D3387" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3387" t="inlineStr">
+        <is>
+          <t>2026-09-22 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3388">
+      <c r="A3388" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B3388" t="inlineStr">
+        <is>
+          <t>EUR/GBP</t>
+        </is>
+      </c>
+      <c r="C3388" t="n">
+        <v>0.8578</v>
+      </c>
+      <c r="D3388" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3388" t="inlineStr">
+        <is>
+          <t>2026-09-22 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3389">
+      <c r="A3389" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B3389" t="inlineStr">
+        <is>
+          <t>EUR/HKD</t>
+        </is>
+      </c>
+      <c r="C3389" t="n">
+        <v>8.9909</v>
+      </c>
+      <c r="D3389" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3389" t="inlineStr">
+        <is>
+          <t>2026-09-22 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3390">
+      <c r="A3390" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B3390" t="inlineStr">
+        <is>
+          <t>EUR/IDR</t>
+        </is>
+      </c>
+      <c r="C3390" t="n">
+        <v>20426.66</v>
+      </c>
+      <c r="D3390" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3390" t="inlineStr">
+        <is>
+          <t>2026-09-22 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3391">
+      <c r="A3391" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B3391" t="inlineStr">
+        <is>
+          <t>EUR/ILS</t>
+        </is>
+      </c>
+      <c r="C3391" t="n">
+        <v>3.4593</v>
+      </c>
+      <c r="D3391" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3391" t="inlineStr">
+        <is>
+          <t>2026-09-22 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3392">
+      <c r="A3392" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B3392" t="inlineStr">
+        <is>
+          <t>EUR/JPY</t>
+        </is>
+      </c>
+      <c r="C3392" t="n">
+        <v>180.17</v>
+      </c>
+      <c r="D3392" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3392" t="inlineStr">
+        <is>
+          <t>2026-09-22 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3393">
+      <c r="A3393" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B3393" t="inlineStr">
+        <is>
+          <t>EUR/KRW</t>
+        </is>
+      </c>
+      <c r="C3393" t="n">
+        <v>1554.55</v>
+      </c>
+      <c r="D3393" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3393" t="inlineStr">
+        <is>
+          <t>2026-09-22 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3394">
+      <c r="A3394" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B3394" t="inlineStr">
+        <is>
+          <t>EUR/MAD</t>
+        </is>
+      </c>
+      <c r="C3394" t="n">
+        <v>10.935739</v>
+      </c>
+      <c r="D3394" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3394" t="inlineStr">
+        <is>
+          <t>2026-09-22 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3395">
+      <c r="A3395" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B3395" t="inlineStr">
+        <is>
+          <t>EUR/PEN</t>
+        </is>
+      </c>
+      <c r="C3395" t="n">
+        <v>3.862727</v>
+      </c>
+      <c r="D3395" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3395" t="inlineStr">
+        <is>
+          <t>2026-09-22 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3396">
+      <c r="A3396" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B3396" t="inlineStr">
+        <is>
+          <t>EUR/PHP</t>
+        </is>
+      </c>
+      <c r="C3396" t="n">
+        <v>71.602</v>
+      </c>
+      <c r="D3396" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3396" t="inlineStr">
+        <is>
+          <t>2026-09-22 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3397">
+      <c r="A3397" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B3397" t="inlineStr">
+        <is>
+          <t>EUR/RUB</t>
+        </is>
+      </c>
+      <c r="C3397" t="n">
+        <v>96.581801</v>
+      </c>
+      <c r="D3397" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3397" t="inlineStr">
+        <is>
+          <t>2026-09-22 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3398">
+      <c r="A3398" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B3398" t="inlineStr">
+        <is>
+          <t>EUR/SAR</t>
+        </is>
+      </c>
+      <c r="C3398" t="n">
+        <v>4.301814</v>
+      </c>
+      <c r="D3398" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3398" t="inlineStr">
+        <is>
+          <t>2026-09-22 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3399">
+      <c r="A3399" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B3399" t="inlineStr">
+        <is>
+          <t>EUR/SEK</t>
+        </is>
+      </c>
+      <c r="C3399" t="n">
+        <v>11.2463</v>
+      </c>
+      <c r="D3399" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3399" t="inlineStr">
+        <is>
+          <t>2026-09-22 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3400">
+      <c r="A3400" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B3400" t="inlineStr">
+        <is>
+          <t>EUR/SGD</t>
+        </is>
+      </c>
+      <c r="C3400" t="n">
+        <v>1.4612</v>
+      </c>
+      <c r="D3400" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3400" t="inlineStr">
+        <is>
+          <t>2026-09-22 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3401">
+      <c r="A3401" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B3401" t="inlineStr">
+        <is>
+          <t>EUR/THB</t>
+        </is>
+      </c>
+      <c r="C3401" t="n">
+        <v>37.988</v>
+      </c>
+      <c r="D3401" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3401" t="inlineStr">
+        <is>
+          <t>2026-09-22 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3402">
+      <c r="A3402" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B3402" t="inlineStr">
+        <is>
+          <t>EUR/TRY</t>
+        </is>
+      </c>
+      <c r="C3402" t="n">
+        <v>55.9492</v>
+      </c>
+      <c r="D3402" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3402" t="inlineStr">
+        <is>
+          <t>2026-09-22 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3403">
+      <c r="A3403" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B3403" t="inlineStr">
+        <is>
+          <t>EUR/USD</t>
+        </is>
+      </c>
+      <c r="C3403" t="n">
+        <v>1.1463</v>
+      </c>
+      <c r="D3403" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3403" t="inlineStr">
+        <is>
+          <t>2026-09-22 07:30 CET</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update currency rates for 2026-09-23
</commit_message>
<xml_diff>
--- a/data/rates.xlsx
+++ b/data/rates.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3403"/>
+  <dimension ref="A1:E3429"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -85493,6 +85493,656 @@
         </is>
       </c>
     </row>
+    <row r="3404">
+      <c r="A3404" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B3404" t="inlineStr">
+        <is>
+          <t>CNY/SGD</t>
+        </is>
+      </c>
+      <c r="C3404" t="n">
+        <v>0.190585</v>
+      </c>
+      <c r="D3404" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3404" t="inlineStr">
+        <is>
+          <t>2026-09-23 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3405">
+      <c r="A3405" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B3405" t="inlineStr">
+        <is>
+          <t>CNY/USD</t>
+        </is>
+      </c>
+      <c r="C3405" t="n">
+        <v>0.149089</v>
+      </c>
+      <c r="D3405" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3405" t="inlineStr">
+        <is>
+          <t>2026-09-23 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3406">
+      <c r="A3406" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B3406" t="inlineStr">
+        <is>
+          <t>EUR/AED</t>
+        </is>
+      </c>
+      <c r="C3406" t="n">
+        <v>4.205633</v>
+      </c>
+      <c r="D3406" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3406" t="inlineStr">
+        <is>
+          <t>2026-09-23 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3407">
+      <c r="A3407" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B3407" t="inlineStr">
+        <is>
+          <t>EUR/ARS</t>
+        </is>
+      </c>
+      <c r="C3407" t="n">
+        <v>1733.423799</v>
+      </c>
+      <c r="D3407" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3407" t="inlineStr">
+        <is>
+          <t>2026-09-23 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3408">
+      <c r="A3408" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B3408" t="inlineStr">
+        <is>
+          <t>EUR/BRL</t>
+        </is>
+      </c>
+      <c r="C3408" t="n">
+        <v>5.8564</v>
+      </c>
+      <c r="D3408" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3408" t="inlineStr">
+        <is>
+          <t>2026-09-23 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3409">
+      <c r="A3409" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B3409" t="inlineStr">
+        <is>
+          <t>EUR/CHF</t>
+        </is>
+      </c>
+      <c r="C3409" t="n">
+        <v>0.9389999999999999</v>
+      </c>
+      <c r="D3409" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3409" t="inlineStr">
+        <is>
+          <t>2026-09-23 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3410">
+      <c r="A3410" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B3410" t="inlineStr">
+        <is>
+          <t>EUR/CLP</t>
+        </is>
+      </c>
+      <c r="C3410" t="n">
+        <v>1086.521511</v>
+      </c>
+      <c r="D3410" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3410" t="inlineStr">
+        <is>
+          <t>2026-09-23 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3411">
+      <c r="A3411" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B3411" t="inlineStr">
+        <is>
+          <t>EUR/CNY</t>
+        </is>
+      </c>
+      <c r="C3411" t="n">
+        <v>7.6538</v>
+      </c>
+      <c r="D3411" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3411" t="inlineStr">
+        <is>
+          <t>2026-09-23 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3412">
+      <c r="A3412" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B3412" t="inlineStr">
+        <is>
+          <t>EUR/COP</t>
+        </is>
+      </c>
+      <c r="C3412" t="n">
+        <v>3672.549801</v>
+      </c>
+      <c r="D3412" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3412" t="inlineStr">
+        <is>
+          <t>2026-09-23 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3413">
+      <c r="A3413" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B3413" t="inlineStr">
+        <is>
+          <t>EUR/DKK</t>
+        </is>
+      </c>
+      <c r="C3413" t="n">
+        <v>7.4756</v>
+      </c>
+      <c r="D3413" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3413" t="inlineStr">
+        <is>
+          <t>2026-09-23 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3414">
+      <c r="A3414" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B3414" t="inlineStr">
+        <is>
+          <t>EUR/GBP</t>
+        </is>
+      </c>
+      <c r="C3414" t="n">
+        <v>0.8595</v>
+      </c>
+      <c r="D3414" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3414" t="inlineStr">
+        <is>
+          <t>2026-09-23 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3415">
+      <c r="A3415" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B3415" t="inlineStr">
+        <is>
+          <t>EUR/HKD</t>
+        </is>
+      </c>
+      <c r="C3415" t="n">
+        <v>8.9506</v>
+      </c>
+      <c r="D3415" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3415" t="inlineStr">
+        <is>
+          <t>2026-09-23 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3416">
+      <c r="A3416" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B3416" t="inlineStr">
+        <is>
+          <t>EUR/IDR</t>
+        </is>
+      </c>
+      <c r="C3416" t="n">
+        <v>20305.82</v>
+      </c>
+      <c r="D3416" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3416" t="inlineStr">
+        <is>
+          <t>2026-09-23 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3417">
+      <c r="A3417" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B3417" t="inlineStr">
+        <is>
+          <t>EUR/ILS</t>
+        </is>
+      </c>
+      <c r="C3417" t="n">
+        <v>3.4417</v>
+      </c>
+      <c r="D3417" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3417" t="inlineStr">
+        <is>
+          <t>2026-09-23 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3418">
+      <c r="A3418" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B3418" t="inlineStr">
+        <is>
+          <t>EUR/JPY</t>
+        </is>
+      </c>
+      <c r="C3418" t="n">
+        <v>180.2</v>
+      </c>
+      <c r="D3418" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3418" t="inlineStr">
+        <is>
+          <t>2026-09-23 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3419">
+      <c r="A3419" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B3419" t="inlineStr">
+        <is>
+          <t>EUR/KRW</t>
+        </is>
+      </c>
+      <c r="C3419" t="n">
+        <v>1558</v>
+      </c>
+      <c r="D3419" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3419" t="inlineStr">
+        <is>
+          <t>2026-09-23 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3420">
+      <c r="A3420" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B3420" t="inlineStr">
+        <is>
+          <t>EUR/MAD</t>
+        </is>
+      </c>
+      <c r="C3420" t="n">
+        <v>10.94728</v>
+      </c>
+      <c r="D3420" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3420" t="inlineStr">
+        <is>
+          <t>2026-09-23 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3421">
+      <c r="A3421" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B3421" t="inlineStr">
+        <is>
+          <t>EUR/PEN</t>
+        </is>
+      </c>
+      <c r="C3421" t="n">
+        <v>3.860812</v>
+      </c>
+      <c r="D3421" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3421" t="inlineStr">
+        <is>
+          <t>2026-09-23 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3422">
+      <c r="A3422" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B3422" t="inlineStr">
+        <is>
+          <t>EUR/PHP</t>
+        </is>
+      </c>
+      <c r="C3422" t="n">
+        <v>71.371</v>
+      </c>
+      <c r="D3422" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3422" t="inlineStr">
+        <is>
+          <t>2026-09-23 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3423">
+      <c r="A3423" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B3423" t="inlineStr">
+        <is>
+          <t>EUR/RUB</t>
+        </is>
+      </c>
+      <c r="C3423" t="n">
+        <v>96.498002</v>
+      </c>
+      <c r="D3423" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3423" t="inlineStr">
+        <is>
+          <t>2026-09-23 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3424">
+      <c r="A3424" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B3424" t="inlineStr">
+        <is>
+          <t>EUR/SAR</t>
+        </is>
+      </c>
+      <c r="C3424" t="n">
+        <v>4.294384</v>
+      </c>
+      <c r="D3424" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3424" t="inlineStr">
+        <is>
+          <t>2026-09-23 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3425">
+      <c r="A3425" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B3425" t="inlineStr">
+        <is>
+          <t>EUR/SEK</t>
+        </is>
+      </c>
+      <c r="C3425" t="n">
+        <v>11.272</v>
+      </c>
+      <c r="D3425" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3425" t="inlineStr">
+        <is>
+          <t>2026-09-23 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3426">
+      <c r="A3426" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B3426" t="inlineStr">
+        <is>
+          <t>EUR/SGD</t>
+        </is>
+      </c>
+      <c r="C3426" t="n">
+        <v>1.4587</v>
+      </c>
+      <c r="D3426" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3426" t="inlineStr">
+        <is>
+          <t>2026-09-23 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3427">
+      <c r="A3427" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B3427" t="inlineStr">
+        <is>
+          <t>EUR/THB</t>
+        </is>
+      </c>
+      <c r="C3427" t="n">
+        <v>37.987</v>
+      </c>
+      <c r="D3427" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3427" t="inlineStr">
+        <is>
+          <t>2026-09-23 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3428">
+      <c r="A3428" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B3428" t="inlineStr">
+        <is>
+          <t>EUR/TRY</t>
+        </is>
+      </c>
+      <c r="C3428" t="n">
+        <v>55.7283</v>
+      </c>
+      <c r="D3428" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3428" t="inlineStr">
+        <is>
+          <t>2026-09-23 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3429">
+      <c r="A3429" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B3429" t="inlineStr">
+        <is>
+          <t>EUR/USD</t>
+        </is>
+      </c>
+      <c r="C3429" t="n">
+        <v>1.1411</v>
+      </c>
+      <c r="D3429" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3429" t="inlineStr">
+        <is>
+          <t>2026-09-23 07:30 CET</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update currency rates for 2026-09-24
</commit_message>
<xml_diff>
--- a/data/rates.xlsx
+++ b/data/rates.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3429"/>
+  <dimension ref="A1:E3455"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -86143,6 +86143,656 @@
         </is>
       </c>
     </row>
+    <row r="3430">
+      <c r="A3430" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B3430" t="inlineStr">
+        <is>
+          <t>CNY/SGD</t>
+        </is>
+      </c>
+      <c r="C3430" t="n">
+        <v>0.190677</v>
+      </c>
+      <c r="D3430" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3430" t="inlineStr">
+        <is>
+          <t>2026-09-24 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3431">
+      <c r="A3431" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B3431" t="inlineStr">
+        <is>
+          <t>CNY/USD</t>
+        </is>
+      </c>
+      <c r="C3431" t="n">
+        <v>0.148974</v>
+      </c>
+      <c r="D3431" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3431" t="inlineStr">
+        <is>
+          <t>2026-09-24 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3432">
+      <c r="A3432" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B3432" t="inlineStr">
+        <is>
+          <t>EUR/AED</t>
+        </is>
+      </c>
+      <c r="C3432" t="n">
+        <v>4.185796</v>
+      </c>
+      <c r="D3432" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3432" t="inlineStr">
+        <is>
+          <t>2026-09-24 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3433">
+      <c r="A3433" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B3433" t="inlineStr">
+        <is>
+          <t>EUR/ARS</t>
+        </is>
+      </c>
+      <c r="C3433" t="n">
+        <v>1728.225455</v>
+      </c>
+      <c r="D3433" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3433" t="inlineStr">
+        <is>
+          <t>2026-09-24 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3434">
+      <c r="A3434" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B3434" t="inlineStr">
+        <is>
+          <t>EUR/BRL</t>
+        </is>
+      </c>
+      <c r="C3434" t="n">
+        <v>5.889</v>
+      </c>
+      <c r="D3434" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3434" t="inlineStr">
+        <is>
+          <t>2026-09-24 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3435">
+      <c r="A3435" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B3435" t="inlineStr">
+        <is>
+          <t>EUR/CHF</t>
+        </is>
+      </c>
+      <c r="C3435" t="n">
+        <v>0.9409</v>
+      </c>
+      <c r="D3435" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3435" t="inlineStr">
+        <is>
+          <t>2026-09-24 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3436">
+      <c r="A3436" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B3436" t="inlineStr">
+        <is>
+          <t>EUR/CLP</t>
+        </is>
+      </c>
+      <c r="C3436" t="n">
+        <v>1080.67767</v>
+      </c>
+      <c r="D3436" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3436" t="inlineStr">
+        <is>
+          <t>2026-09-24 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3437">
+      <c r="A3437" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B3437" t="inlineStr">
+        <is>
+          <t>EUR/CNY</t>
+        </is>
+      </c>
+      <c r="C3437" t="n">
+        <v>7.6302</v>
+      </c>
+      <c r="D3437" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3437" t="inlineStr">
+        <is>
+          <t>2026-09-24 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3438">
+      <c r="A3438" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B3438" t="inlineStr">
+        <is>
+          <t>EUR/COP</t>
+        </is>
+      </c>
+      <c r="C3438" t="n">
+        <v>3657.85683</v>
+      </c>
+      <c r="D3438" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3438" t="inlineStr">
+        <is>
+          <t>2026-09-24 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3439">
+      <c r="A3439" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B3439" t="inlineStr">
+        <is>
+          <t>EUR/DKK</t>
+        </is>
+      </c>
+      <c r="C3439" t="n">
+        <v>7.4756</v>
+      </c>
+      <c r="D3439" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3439" t="inlineStr">
+        <is>
+          <t>2026-09-24 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3440">
+      <c r="A3440" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B3440" t="inlineStr">
+        <is>
+          <t>EUR/GBP</t>
+        </is>
+      </c>
+      <c r="C3440" t="n">
+        <v>0.85986</v>
+      </c>
+      <c r="D3440" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3440" t="inlineStr">
+        <is>
+          <t>2026-09-24 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3441">
+      <c r="A3441" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B3441" t="inlineStr">
+        <is>
+          <t>EUR/HKD</t>
+        </is>
+      </c>
+      <c r="C3441" t="n">
+        <v>8.9148</v>
+      </c>
+      <c r="D3441" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3441" t="inlineStr">
+        <is>
+          <t>2026-09-24 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3442">
+      <c r="A3442" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B3442" t="inlineStr">
+        <is>
+          <t>EUR/IDR</t>
+        </is>
+      </c>
+      <c r="C3442" t="n">
+        <v>20384.1</v>
+      </c>
+      <c r="D3442" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3442" t="inlineStr">
+        <is>
+          <t>2026-09-24 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3443">
+      <c r="A3443" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B3443" t="inlineStr">
+        <is>
+          <t>EUR/ILS</t>
+        </is>
+      </c>
+      <c r="C3443" t="n">
+        <v>3.4649</v>
+      </c>
+      <c r="D3443" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3443" t="inlineStr">
+        <is>
+          <t>2026-09-24 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3444">
+      <c r="A3444" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B3444" t="inlineStr">
+        <is>
+          <t>EUR/JPY</t>
+        </is>
+      </c>
+      <c r="C3444" t="n">
+        <v>180.57</v>
+      </c>
+      <c r="D3444" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3444" t="inlineStr">
+        <is>
+          <t>2026-09-24 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3445">
+      <c r="A3445" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B3445" t="inlineStr">
+        <is>
+          <t>EUR/KRW</t>
+        </is>
+      </c>
+      <c r="C3445" t="n">
+        <v>1555.69</v>
+      </c>
+      <c r="D3445" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3445" t="inlineStr">
+        <is>
+          <t>2026-09-24 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3446">
+      <c r="A3446" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B3446" t="inlineStr">
+        <is>
+          <t>EUR/MAD</t>
+        </is>
+      </c>
+      <c r="C3446" t="n">
+        <v>10.94296</v>
+      </c>
+      <c r="D3446" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3446" t="inlineStr">
+        <is>
+          <t>2026-09-24 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3447">
+      <c r="A3447" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B3447" t="inlineStr">
+        <is>
+          <t>EUR/PEN</t>
+        </is>
+      </c>
+      <c r="C3447" t="n">
+        <v>3.855002</v>
+      </c>
+      <c r="D3447" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3447" t="inlineStr">
+        <is>
+          <t>2026-09-24 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3448">
+      <c r="A3448" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B3448" t="inlineStr">
+        <is>
+          <t>EUR/PHP</t>
+        </is>
+      </c>
+      <c r="C3448" t="n">
+        <v>71.328</v>
+      </c>
+      <c r="D3448" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3448" t="inlineStr">
+        <is>
+          <t>2026-09-24 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3449">
+      <c r="A3449" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B3449" t="inlineStr">
+        <is>
+          <t>EUR/RUB</t>
+        </is>
+      </c>
+      <c r="C3449" t="n">
+        <v>96.03554</v>
+      </c>
+      <c r="D3449" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3449" t="inlineStr">
+        <is>
+          <t>2026-09-24 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3450">
+      <c r="A3450" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B3450" t="inlineStr">
+        <is>
+          <t>EUR/SAR</t>
+        </is>
+      </c>
+      <c r="C3450" t="n">
+        <v>4.274128</v>
+      </c>
+      <c r="D3450" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3450" t="inlineStr">
+        <is>
+          <t>2026-09-24 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3451">
+      <c r="A3451" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B3451" t="inlineStr">
+        <is>
+          <t>EUR/SEK</t>
+        </is>
+      </c>
+      <c r="C3451" t="n">
+        <v>11.2645</v>
+      </c>
+      <c r="D3451" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3451" t="inlineStr">
+        <is>
+          <t>2026-09-24 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3452">
+      <c r="A3452" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B3452" t="inlineStr">
+        <is>
+          <t>EUR/SGD</t>
+        </is>
+      </c>
+      <c r="C3452" t="n">
+        <v>1.4549</v>
+      </c>
+      <c r="D3452" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3452" t="inlineStr">
+        <is>
+          <t>2026-09-24 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3453">
+      <c r="A3453" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B3453" t="inlineStr">
+        <is>
+          <t>EUR/THB</t>
+        </is>
+      </c>
+      <c r="C3453" t="n">
+        <v>38.057</v>
+      </c>
+      <c r="D3453" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3453" t="inlineStr">
+        <is>
+          <t>2026-09-24 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3454">
+      <c r="A3454" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B3454" t="inlineStr">
+        <is>
+          <t>EUR/TRY</t>
+        </is>
+      </c>
+      <c r="C3454" t="n">
+        <v>55.5332</v>
+      </c>
+      <c r="D3454" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3454" t="inlineStr">
+        <is>
+          <t>2026-09-24 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3455">
+      <c r="A3455" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B3455" t="inlineStr">
+        <is>
+          <t>EUR/USD</t>
+        </is>
+      </c>
+      <c r="C3455" t="n">
+        <v>1.1367</v>
+      </c>
+      <c r="D3455" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3455" t="inlineStr">
+        <is>
+          <t>2026-09-24 07:30 CET</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update currency rates for 2026-09-25
</commit_message>
<xml_diff>
--- a/data/rates.xlsx
+++ b/data/rates.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3455"/>
+  <dimension ref="A1:E3481"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -86793,6 +86793,656 @@
         </is>
       </c>
     </row>
+    <row r="3456">
+      <c r="A3456" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B3456" t="inlineStr">
+        <is>
+          <t>CNY/SGD</t>
+        </is>
+      </c>
+      <c r="C3456" t="n">
+        <v>0.190239</v>
+      </c>
+      <c r="D3456" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3456" t="inlineStr">
+        <is>
+          <t>2026-09-25 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3457">
+      <c r="A3457" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B3457" t="inlineStr">
+        <is>
+          <t>CNY/USD</t>
+        </is>
+      </c>
+      <c r="C3457" t="n">
+        <v>0.14896</v>
+      </c>
+      <c r="D3457" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3457" t="inlineStr">
+        <is>
+          <t>2026-09-25 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3458">
+      <c r="A3458" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B3458" t="inlineStr">
+        <is>
+          <t>EUR/AED</t>
+        </is>
+      </c>
+      <c r="C3458" t="n">
+        <v>4.179551</v>
+      </c>
+      <c r="D3458" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3458" t="inlineStr">
+        <is>
+          <t>2026-09-25 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3459">
+      <c r="A3459" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B3459" t="inlineStr">
+        <is>
+          <t>EUR/ARS</t>
+        </is>
+      </c>
+      <c r="C3459" t="n">
+        <v>1728.429443</v>
+      </c>
+      <c r="D3459" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3459" t="inlineStr">
+        <is>
+          <t>2026-09-25 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3460">
+      <c r="A3460" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B3460" t="inlineStr">
+        <is>
+          <t>EUR/BRL</t>
+        </is>
+      </c>
+      <c r="C3460" t="n">
+        <v>5.9091</v>
+      </c>
+      <c r="D3460" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3460" t="inlineStr">
+        <is>
+          <t>2026-09-25 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3461">
+      <c r="A3461" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B3461" t="inlineStr">
+        <is>
+          <t>EUR/CHF</t>
+        </is>
+      </c>
+      <c r="C3461" t="n">
+        <v>0.9445</v>
+      </c>
+      <c r="D3461" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3461" t="inlineStr">
+        <is>
+          <t>2026-09-25 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3462">
+      <c r="A3462" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B3462" t="inlineStr">
+        <is>
+          <t>EUR/CLP</t>
+        </is>
+      </c>
+      <c r="C3462" t="n">
+        <v>1095.011772</v>
+      </c>
+      <c r="D3462" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3462" t="inlineStr">
+        <is>
+          <t>2026-09-25 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3463">
+      <c r="A3463" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B3463" t="inlineStr">
+        <is>
+          <t>EUR/CNY</t>
+        </is>
+      </c>
+      <c r="C3463" t="n">
+        <v>7.6551</v>
+      </c>
+      <c r="D3463" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3463" t="inlineStr">
+        <is>
+          <t>2026-09-25 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3464">
+      <c r="A3464" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B3464" t="inlineStr">
+        <is>
+          <t>EUR/COP</t>
+        </is>
+      </c>
+      <c r="C3464" t="n">
+        <v>3730.994223</v>
+      </c>
+      <c r="D3464" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3464" t="inlineStr">
+        <is>
+          <t>2026-09-25 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3465">
+      <c r="A3465" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B3465" t="inlineStr">
+        <is>
+          <t>EUR/DKK</t>
+        </is>
+      </c>
+      <c r="C3465" t="n">
+        <v>7.4755</v>
+      </c>
+      <c r="D3465" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3465" t="inlineStr">
+        <is>
+          <t>2026-09-25 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3466">
+      <c r="A3466" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B3466" t="inlineStr">
+        <is>
+          <t>EUR/GBP</t>
+        </is>
+      </c>
+      <c r="C3466" t="n">
+        <v>0.86045</v>
+      </c>
+      <c r="D3466" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3466" t="inlineStr">
+        <is>
+          <t>2026-09-25 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3467">
+      <c r="A3467" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B3467" t="inlineStr">
+        <is>
+          <t>EUR/HKD</t>
+        </is>
+      </c>
+      <c r="C3467" t="n">
+        <v>8.9445</v>
+      </c>
+      <c r="D3467" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3467" t="inlineStr">
+        <is>
+          <t>2026-09-25 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3468">
+      <c r="A3468" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B3468" t="inlineStr">
+        <is>
+          <t>EUR/IDR</t>
+        </is>
+      </c>
+      <c r="C3468" t="n">
+        <v>20427.22</v>
+      </c>
+      <c r="D3468" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3468" t="inlineStr">
+        <is>
+          <t>2026-09-25 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3469">
+      <c r="A3469" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B3469" t="inlineStr">
+        <is>
+          <t>EUR/ILS</t>
+        </is>
+      </c>
+      <c r="C3469" t="n">
+        <v>3.4594</v>
+      </c>
+      <c r="D3469" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3469" t="inlineStr">
+        <is>
+          <t>2026-09-25 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3470">
+      <c r="A3470" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B3470" t="inlineStr">
+        <is>
+          <t>EUR/JPY</t>
+        </is>
+      </c>
+      <c r="C3470" t="n">
+        <v>179.7</v>
+      </c>
+      <c r="D3470" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3470" t="inlineStr">
+        <is>
+          <t>2026-09-25 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3471">
+      <c r="A3471" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B3471" t="inlineStr">
+        <is>
+          <t>EUR/KRW</t>
+        </is>
+      </c>
+      <c r="C3471" t="n">
+        <v>1545.16</v>
+      </c>
+      <c r="D3471" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3471" t="inlineStr">
+        <is>
+          <t>2026-09-25 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3472">
+      <c r="A3472" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B3472" t="inlineStr">
+        <is>
+          <t>EUR/MAD</t>
+        </is>
+      </c>
+      <c r="C3472" t="n">
+        <v>10.936386</v>
+      </c>
+      <c r="D3472" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3472" t="inlineStr">
+        <is>
+          <t>2026-09-25 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3473">
+      <c r="A3473" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B3473" t="inlineStr">
+        <is>
+          <t>EUR/PEN</t>
+        </is>
+      </c>
+      <c r="C3473" t="n">
+        <v>3.865153</v>
+      </c>
+      <c r="D3473" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3473" t="inlineStr">
+        <is>
+          <t>2026-09-25 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3474">
+      <c r="A3474" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B3474" t="inlineStr">
+        <is>
+          <t>EUR/PHP</t>
+        </is>
+      </c>
+      <c r="C3474" t="n">
+        <v>71.244</v>
+      </c>
+      <c r="D3474" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3474" t="inlineStr">
+        <is>
+          <t>2026-09-25 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3475">
+      <c r="A3475" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B3475" t="inlineStr">
+        <is>
+          <t>EUR/RUB</t>
+        </is>
+      </c>
+      <c r="C3475" t="n">
+        <v>96.664879</v>
+      </c>
+      <c r="D3475" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3475" t="inlineStr">
+        <is>
+          <t>2026-09-25 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3476">
+      <c r="A3476" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B3476" t="inlineStr">
+        <is>
+          <t>EUR/SAR</t>
+        </is>
+      </c>
+      <c r="C3476" t="n">
+        <v>4.267751</v>
+      </c>
+      <c r="D3476" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3476" t="inlineStr">
+        <is>
+          <t>2026-09-25 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3477">
+      <c r="A3477" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B3477" t="inlineStr">
+        <is>
+          <t>EUR/SEK</t>
+        </is>
+      </c>
+      <c r="C3477" t="n">
+        <v>11.29</v>
+      </c>
+      <c r="D3477" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3477" t="inlineStr">
+        <is>
+          <t>2026-09-25 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3478">
+      <c r="A3478" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B3478" t="inlineStr">
+        <is>
+          <t>EUR/SGD</t>
+        </is>
+      </c>
+      <c r="C3478" t="n">
+        <v>1.4563</v>
+      </c>
+      <c r="D3478" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3478" t="inlineStr">
+        <is>
+          <t>2026-09-25 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3479">
+      <c r="A3479" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B3479" t="inlineStr">
+        <is>
+          <t>EUR/THB</t>
+        </is>
+      </c>
+      <c r="C3479" t="n">
+        <v>38.023</v>
+      </c>
+      <c r="D3479" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3479" t="inlineStr">
+        <is>
+          <t>2026-09-25 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3480">
+      <c r="A3480" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B3480" t="inlineStr">
+        <is>
+          <t>EUR/TRY</t>
+        </is>
+      </c>
+      <c r="C3480" t="n">
+        <v>55.7975</v>
+      </c>
+      <c r="D3480" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3480" t="inlineStr">
+        <is>
+          <t>2026-09-25 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3481">
+      <c r="A3481" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B3481" t="inlineStr">
+        <is>
+          <t>EUR/USD</t>
+        </is>
+      </c>
+      <c r="C3481" t="n">
+        <v>1.1403</v>
+      </c>
+      <c r="D3481" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3481" t="inlineStr">
+        <is>
+          <t>2026-09-25 07:30 CET</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update currency rates for 2026-09-28
</commit_message>
<xml_diff>
--- a/data/rates.xlsx
+++ b/data/rates.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3481"/>
+  <dimension ref="A1:E3507"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -87443,6 +87443,656 @@
         </is>
       </c>
     </row>
+    <row r="3482">
+      <c r="A3482" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B3482" t="inlineStr">
+        <is>
+          <t>CNY/SGD</t>
+        </is>
+      </c>
+      <c r="C3482" t="n">
+        <v>0.190408</v>
+      </c>
+      <c r="D3482" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3482" t="inlineStr">
+        <is>
+          <t>2026-09-29 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3483">
+      <c r="A3483" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B3483" t="inlineStr">
+        <is>
+          <t>CNY/USD</t>
+        </is>
+      </c>
+      <c r="C3483" t="n">
+        <v>0.14902</v>
+      </c>
+      <c r="D3483" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3483" t="inlineStr">
+        <is>
+          <t>2026-09-29 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3484">
+      <c r="A3484" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B3484" t="inlineStr">
+        <is>
+          <t>EUR/AED</t>
+        </is>
+      </c>
+      <c r="C3484" t="n">
+        <v>4.182816</v>
+      </c>
+      <c r="D3484" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3484" t="inlineStr">
+        <is>
+          <t>2026-09-29 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3485">
+      <c r="A3485" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B3485" t="inlineStr">
+        <is>
+          <t>EUR/ARS</t>
+        </is>
+      </c>
+      <c r="C3485" t="n">
+        <v>1735.730414</v>
+      </c>
+      <c r="D3485" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3485" t="inlineStr">
+        <is>
+          <t>2026-09-29 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3486">
+      <c r="A3486" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B3486" t="inlineStr">
+        <is>
+          <t>EUR/BRL</t>
+        </is>
+      </c>
+      <c r="C3486" t="n">
+        <v>5.9186</v>
+      </c>
+      <c r="D3486" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3486" t="inlineStr">
+        <is>
+          <t>2026-09-29 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3487">
+      <c r="A3487" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B3487" t="inlineStr">
+        <is>
+          <t>EUR/CHF</t>
+        </is>
+      </c>
+      <c r="C3487" t="n">
+        <v>0.9464</v>
+      </c>
+      <c r="D3487" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3487" t="inlineStr">
+        <is>
+          <t>2026-09-29 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3488">
+      <c r="A3488" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B3488" t="inlineStr">
+        <is>
+          <t>EUR/CLP</t>
+        </is>
+      </c>
+      <c r="C3488" t="n">
+        <v>1096.800746</v>
+      </c>
+      <c r="D3488" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3488" t="inlineStr">
+        <is>
+          <t>2026-09-29 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3489">
+      <c r="A3489" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B3489" t="inlineStr">
+        <is>
+          <t>EUR/CNY</t>
+        </is>
+      </c>
+      <c r="C3489" t="n">
+        <v>7.6352</v>
+      </c>
+      <c r="D3489" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3489" t="inlineStr">
+        <is>
+          <t>2026-09-29 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3490">
+      <c r="A3490" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B3490" t="inlineStr">
+        <is>
+          <t>EUR/COP</t>
+        </is>
+      </c>
+      <c r="C3490" t="n">
+        <v>3805.123811</v>
+      </c>
+      <c r="D3490" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3490" t="inlineStr">
+        <is>
+          <t>2026-09-29 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3491">
+      <c r="A3491" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B3491" t="inlineStr">
+        <is>
+          <t>EUR/DKK</t>
+        </is>
+      </c>
+      <c r="C3491" t="n">
+        <v>7.4752</v>
+      </c>
+      <c r="D3491" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3491" t="inlineStr">
+        <is>
+          <t>2026-09-29 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3492">
+      <c r="A3492" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B3492" t="inlineStr">
+        <is>
+          <t>EUR/GBP</t>
+        </is>
+      </c>
+      <c r="C3492" t="n">
+        <v>0.85785</v>
+      </c>
+      <c r="D3492" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3492" t="inlineStr">
+        <is>
+          <t>2026-09-29 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3493">
+      <c r="A3493" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B3493" t="inlineStr">
+        <is>
+          <t>EUR/HKD</t>
+        </is>
+      </c>
+      <c r="C3493" t="n">
+        <v>8.925800000000001</v>
+      </c>
+      <c r="D3493" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3493" t="inlineStr">
+        <is>
+          <t>2026-09-29 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3494">
+      <c r="A3494" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B3494" t="inlineStr">
+        <is>
+          <t>EUR/IDR</t>
+        </is>
+      </c>
+      <c r="C3494" t="n">
+        <v>20453.78</v>
+      </c>
+      <c r="D3494" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3494" t="inlineStr">
+        <is>
+          <t>2026-09-29 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3495">
+      <c r="A3495" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B3495" t="inlineStr">
+        <is>
+          <t>EUR/ILS</t>
+        </is>
+      </c>
+      <c r="C3495" t="n">
+        <v>3.4854</v>
+      </c>
+      <c r="D3495" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3495" t="inlineStr">
+        <is>
+          <t>2026-09-29 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3496">
+      <c r="A3496" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B3496" t="inlineStr">
+        <is>
+          <t>EUR/JPY</t>
+        </is>
+      </c>
+      <c r="C3496" t="n">
+        <v>178.5</v>
+      </c>
+      <c r="D3496" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3496" t="inlineStr">
+        <is>
+          <t>2026-09-29 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3497">
+      <c r="A3497" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B3497" t="inlineStr">
+        <is>
+          <t>EUR/KRW</t>
+        </is>
+      </c>
+      <c r="C3497" t="n">
+        <v>1545.05</v>
+      </c>
+      <c r="D3497" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3497" t="inlineStr">
+        <is>
+          <t>2026-09-29 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3498">
+      <c r="A3498" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B3498" t="inlineStr">
+        <is>
+          <t>EUR/MAD</t>
+        </is>
+      </c>
+      <c r="C3498" t="n">
+        <v>10.947254</v>
+      </c>
+      <c r="D3498" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3498" t="inlineStr">
+        <is>
+          <t>2026-09-29 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3499">
+      <c r="A3499" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B3499" t="inlineStr">
+        <is>
+          <t>EUR/PEN</t>
+        </is>
+      </c>
+      <c r="C3499" t="n">
+        <v>3.867926</v>
+      </c>
+      <c r="D3499" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3499" t="inlineStr">
+        <is>
+          <t>2026-09-29 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3500">
+      <c r="A3500" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B3500" t="inlineStr">
+        <is>
+          <t>EUR/PHP</t>
+        </is>
+      </c>
+      <c r="C3500" t="n">
+        <v>71.099</v>
+      </c>
+      <c r="D3500" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3500" t="inlineStr">
+        <is>
+          <t>2026-09-29 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3501">
+      <c r="A3501" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B3501" t="inlineStr">
+        <is>
+          <t>EUR/RUB</t>
+        </is>
+      </c>
+      <c r="C3501" t="n">
+        <v>96.061131</v>
+      </c>
+      <c r="D3501" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3501" t="inlineStr">
+        <is>
+          <t>2026-09-29 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3502">
+      <c r="A3502" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B3502" t="inlineStr">
+        <is>
+          <t>EUR/SAR</t>
+        </is>
+      </c>
+      <c r="C3502" t="n">
+        <v>4.271085</v>
+      </c>
+      <c r="D3502" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3502" t="inlineStr">
+        <is>
+          <t>2026-09-29 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3503">
+      <c r="A3503" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B3503" t="inlineStr">
+        <is>
+          <t>EUR/SEK</t>
+        </is>
+      </c>
+      <c r="C3503" t="n">
+        <v>11.3205</v>
+      </c>
+      <c r="D3503" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3503" t="inlineStr">
+        <is>
+          <t>2026-09-29 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3504">
+      <c r="A3504" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B3504" t="inlineStr">
+        <is>
+          <t>EUR/SGD</t>
+        </is>
+      </c>
+      <c r="C3504" t="n">
+        <v>1.4538</v>
+      </c>
+      <c r="D3504" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3504" t="inlineStr">
+        <is>
+          <t>2026-09-29 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3505">
+      <c r="A3505" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B3505" t="inlineStr">
+        <is>
+          <t>EUR/THB</t>
+        </is>
+      </c>
+      <c r="C3505" t="n">
+        <v>38.196</v>
+      </c>
+      <c r="D3505" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3505" t="inlineStr">
+        <is>
+          <t>2026-09-29 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3506">
+      <c r="A3506" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B3506" t="inlineStr">
+        <is>
+          <t>EUR/TRY</t>
+        </is>
+      </c>
+      <c r="C3506" t="n">
+        <v>55.7318</v>
+      </c>
+      <c r="D3506" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3506" t="inlineStr">
+        <is>
+          <t>2026-09-29 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3507">
+      <c r="A3507" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B3507" t="inlineStr">
+        <is>
+          <t>EUR/USD</t>
+        </is>
+      </c>
+      <c r="C3507" t="n">
+        <v>1.1378</v>
+      </c>
+      <c r="D3507" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3507" t="inlineStr">
+        <is>
+          <t>2026-09-29 07:30 CET</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update currency rates for 2026-09-29
</commit_message>
<xml_diff>
--- a/data/rates.xlsx
+++ b/data/rates.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3507"/>
+  <dimension ref="A1:E3533"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -88093,6 +88093,656 @@
         </is>
       </c>
     </row>
+    <row r="3508">
+      <c r="A3508" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B3508" t="inlineStr">
+        <is>
+          <t>CNY/SGD</t>
+        </is>
+      </c>
+      <c r="C3508" t="n">
+        <v>0.190549</v>
+      </c>
+      <c r="D3508" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3508" t="inlineStr">
+        <is>
+          <t>2026-09-29 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3509">
+      <c r="A3509" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B3509" t="inlineStr">
+        <is>
+          <t>CNY/USD</t>
+        </is>
+      </c>
+      <c r="C3509" t="n">
+        <v>0.149178</v>
+      </c>
+      <c r="D3509" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3509" t="inlineStr">
+        <is>
+          <t>2026-09-29 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3510">
+      <c r="A3510" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B3510" t="inlineStr">
+        <is>
+          <t>EUR/AED</t>
+        </is>
+      </c>
+      <c r="C3510" t="n">
+        <v>4.176174</v>
+      </c>
+      <c r="D3510" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3510" t="inlineStr">
+        <is>
+          <t>2026-09-29 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3511">
+      <c r="A3511" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B3511" t="inlineStr">
+        <is>
+          <t>EUR/ARS</t>
+        </is>
+      </c>
+      <c r="C3511" t="n">
+        <v>1738.421219</v>
+      </c>
+      <c r="D3511" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3511" t="inlineStr">
+        <is>
+          <t>2026-09-29 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3512">
+      <c r="A3512" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B3512" t="inlineStr">
+        <is>
+          <t>EUR/BRL</t>
+        </is>
+      </c>
+      <c r="C3512" t="n">
+        <v>5.9177</v>
+      </c>
+      <c r="D3512" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3512" t="inlineStr">
+        <is>
+          <t>2026-09-29 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3513">
+      <c r="A3513" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B3513" t="inlineStr">
+        <is>
+          <t>EUR/CHF</t>
+        </is>
+      </c>
+      <c r="C3513" t="n">
+        <v>0.9461000000000001</v>
+      </c>
+      <c r="D3513" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3513" t="inlineStr">
+        <is>
+          <t>2026-09-29 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3514">
+      <c r="A3514" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B3514" t="inlineStr">
+        <is>
+          <t>EUR/CLP</t>
+        </is>
+      </c>
+      <c r="C3514" t="n">
+        <v>1094.088216</v>
+      </c>
+      <c r="D3514" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3514" t="inlineStr">
+        <is>
+          <t>2026-09-29 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3515">
+      <c r="A3515" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B3515" t="inlineStr">
+        <is>
+          <t>EUR/CNY</t>
+        </is>
+      </c>
+      <c r="C3515" t="n">
+        <v>7.6117</v>
+      </c>
+      <c r="D3515" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3515" t="inlineStr">
+        <is>
+          <t>2026-09-29 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3516">
+      <c r="A3516" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B3516" t="inlineStr">
+        <is>
+          <t>EUR/COP</t>
+        </is>
+      </c>
+      <c r="C3516" t="n">
+        <v>3758.847047</v>
+      </c>
+      <c r="D3516" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3516" t="inlineStr">
+        <is>
+          <t>2026-09-29 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3517">
+      <c r="A3517" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B3517" t="inlineStr">
+        <is>
+          <t>EUR/DKK</t>
+        </is>
+      </c>
+      <c r="C3517" t="n">
+        <v>7.4754</v>
+      </c>
+      <c r="D3517" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3517" t="inlineStr">
+        <is>
+          <t>2026-09-29 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3518">
+      <c r="A3518" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B3518" t="inlineStr">
+        <is>
+          <t>EUR/GBP</t>
+        </is>
+      </c>
+      <c r="C3518" t="n">
+        <v>0.8571800000000001</v>
+      </c>
+      <c r="D3518" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3518" t="inlineStr">
+        <is>
+          <t>2026-09-29 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3519">
+      <c r="A3519" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B3519" t="inlineStr">
+        <is>
+          <t>EUR/HKD</t>
+        </is>
+      </c>
+      <c r="C3519" t="n">
+        <v>8.9091</v>
+      </c>
+      <c r="D3519" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3519" t="inlineStr">
+        <is>
+          <t>2026-09-29 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3520">
+      <c r="A3520" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B3520" t="inlineStr">
+        <is>
+          <t>EUR/IDR</t>
+        </is>
+      </c>
+      <c r="C3520" t="n">
+        <v>20350.09</v>
+      </c>
+      <c r="D3520" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3520" t="inlineStr">
+        <is>
+          <t>2026-09-29 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3521">
+      <c r="A3521" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B3521" t="inlineStr">
+        <is>
+          <t>EUR/ILS</t>
+        </is>
+      </c>
+      <c r="C3521" t="n">
+        <v>3.4702</v>
+      </c>
+      <c r="D3521" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3521" t="inlineStr">
+        <is>
+          <t>2026-09-29 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3522">
+      <c r="A3522" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B3522" t="inlineStr">
+        <is>
+          <t>EUR/JPY</t>
+        </is>
+      </c>
+      <c r="C3522" t="n">
+        <v>178.41</v>
+      </c>
+      <c r="D3522" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3522" t="inlineStr">
+        <is>
+          <t>2026-09-29 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3523">
+      <c r="A3523" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B3523" t="inlineStr">
+        <is>
+          <t>EUR/KRW</t>
+        </is>
+      </c>
+      <c r="C3523" t="n">
+        <v>1536.74</v>
+      </c>
+      <c r="D3523" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3523" t="inlineStr">
+        <is>
+          <t>2026-09-29 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3524">
+      <c r="A3524" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B3524" t="inlineStr">
+        <is>
+          <t>EUR/MAD</t>
+        </is>
+      </c>
+      <c r="C3524" t="n">
+        <v>10.96131</v>
+      </c>
+      <c r="D3524" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3524" t="inlineStr">
+        <is>
+          <t>2026-09-29 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3525">
+      <c r="A3525" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B3525" t="inlineStr">
+        <is>
+          <t>EUR/PEN</t>
+        </is>
+      </c>
+      <c r="C3525" t="n">
+        <v>3.88764</v>
+      </c>
+      <c r="D3525" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3525" t="inlineStr">
+        <is>
+          <t>2026-09-29 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3526">
+      <c r="A3526" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B3526" t="inlineStr">
+        <is>
+          <t>EUR/PHP</t>
+        </is>
+      </c>
+      <c r="C3526" t="n">
+        <v>71.02200000000001</v>
+      </c>
+      <c r="D3526" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3526" t="inlineStr">
+        <is>
+          <t>2026-09-29 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3527">
+      <c r="A3527" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B3527" t="inlineStr">
+        <is>
+          <t>EUR/RUB</t>
+        </is>
+      </c>
+      <c r="C3527" t="n">
+        <v>96.024484</v>
+      </c>
+      <c r="D3527" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3527" t="inlineStr">
+        <is>
+          <t>2026-09-29 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3528">
+      <c r="A3528" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B3528" t="inlineStr">
+        <is>
+          <t>EUR/SAR</t>
+        </is>
+      </c>
+      <c r="C3528" t="n">
+        <v>4.264303</v>
+      </c>
+      <c r="D3528" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3528" t="inlineStr">
+        <is>
+          <t>2026-09-29 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3529">
+      <c r="A3529" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B3529" t="inlineStr">
+        <is>
+          <t>EUR/SEK</t>
+        </is>
+      </c>
+      <c r="C3529" t="n">
+        <v>11.321</v>
+      </c>
+      <c r="D3529" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3529" t="inlineStr">
+        <is>
+          <t>2026-09-29 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3530">
+      <c r="A3530" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B3530" t="inlineStr">
+        <is>
+          <t>EUR/SGD</t>
+        </is>
+      </c>
+      <c r="C3530" t="n">
+        <v>1.4504</v>
+      </c>
+      <c r="D3530" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3530" t="inlineStr">
+        <is>
+          <t>2026-09-29 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3531">
+      <c r="A3531" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B3531" t="inlineStr">
+        <is>
+          <t>EUR/THB</t>
+        </is>
+      </c>
+      <c r="C3531" t="n">
+        <v>38.056</v>
+      </c>
+      <c r="D3531" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3531" t="inlineStr">
+        <is>
+          <t>2026-09-29 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3532">
+      <c r="A3532" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B3532" t="inlineStr">
+        <is>
+          <t>EUR/TRY</t>
+        </is>
+      </c>
+      <c r="C3532" t="n">
+        <v>55.6398</v>
+      </c>
+      <c r="D3532" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3532" t="inlineStr">
+        <is>
+          <t>2026-09-29 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3533">
+      <c r="A3533" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B3533" t="inlineStr">
+        <is>
+          <t>EUR/USD</t>
+        </is>
+      </c>
+      <c r="C3533" t="n">
+        <v>1.1355</v>
+      </c>
+      <c r="D3533" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3533" t="inlineStr">
+        <is>
+          <t>2026-09-29 07:30 CET</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update currency rates for 2026-09-30
</commit_message>
<xml_diff>
--- a/data/rates.xlsx
+++ b/data/rates.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3533"/>
+  <dimension ref="A1:E3559"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -88743,6 +88743,656 @@
         </is>
       </c>
     </row>
+    <row r="3534">
+      <c r="A3534" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B3534" t="inlineStr">
+        <is>
+          <t>CNY/SGD</t>
+        </is>
+      </c>
+      <c r="C3534" t="n">
+        <v>0.190503</v>
+      </c>
+      <c r="D3534" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3534" t="inlineStr">
+        <is>
+          <t>2026-09-30 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3535">
+      <c r="A3535" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B3535" t="inlineStr">
+        <is>
+          <t>CNY/USD</t>
+        </is>
+      </c>
+      <c r="C3535" t="n">
+        <v>0.149153</v>
+      </c>
+      <c r="D3535" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3535" t="inlineStr">
+        <is>
+          <t>2026-09-30 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3536">
+      <c r="A3536" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B3536" t="inlineStr">
+        <is>
+          <t>EUR/AED</t>
+        </is>
+      </c>
+      <c r="C3536" t="n">
+        <v>4.16613</v>
+      </c>
+      <c r="D3536" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3536" t="inlineStr">
+        <is>
+          <t>2026-09-30 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3537">
+      <c r="A3537" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B3537" t="inlineStr">
+        <is>
+          <t>EUR/ARS</t>
+        </is>
+      </c>
+      <c r="C3537" t="n">
+        <v>1728.81048</v>
+      </c>
+      <c r="D3537" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3537" t="inlineStr">
+        <is>
+          <t>2026-09-30 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3538">
+      <c r="A3538" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B3538" t="inlineStr">
+        <is>
+          <t>EUR/BRL</t>
+        </is>
+      </c>
+      <c r="C3538" t="n">
+        <v>5.9077</v>
+      </c>
+      <c r="D3538" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3538" t="inlineStr">
+        <is>
+          <t>2026-09-30 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3539">
+      <c r="A3539" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B3539" t="inlineStr">
+        <is>
+          <t>EUR/CHF</t>
+        </is>
+      </c>
+      <c r="C3539" t="n">
+        <v>0.9478</v>
+      </c>
+      <c r="D3539" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3539" t="inlineStr">
+        <is>
+          <t>2026-09-30 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3540">
+      <c r="A3540" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B3540" t="inlineStr">
+        <is>
+          <t>EUR/CLP</t>
+        </is>
+      </c>
+      <c r="C3540" t="n">
+        <v>1098.269116</v>
+      </c>
+      <c r="D3540" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3540" t="inlineStr">
+        <is>
+          <t>2026-09-30 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3541">
+      <c r="A3541" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B3541" t="inlineStr">
+        <is>
+          <t>EUR/CNY</t>
+        </is>
+      </c>
+      <c r="C3541" t="n">
+        <v>7.613</v>
+      </c>
+      <c r="D3541" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3541" t="inlineStr">
+        <is>
+          <t>2026-09-30 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3542">
+      <c r="A3542" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B3542" t="inlineStr">
+        <is>
+          <t>EUR/COP</t>
+        </is>
+      </c>
+      <c r="C3542" t="n">
+        <v>3825.056839</v>
+      </c>
+      <c r="D3542" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3542" t="inlineStr">
+        <is>
+          <t>2026-09-30 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3543">
+      <c r="A3543" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B3543" t="inlineStr">
+        <is>
+          <t>EUR/DKK</t>
+        </is>
+      </c>
+      <c r="C3543" t="n">
+        <v>7.4755</v>
+      </c>
+      <c r="D3543" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3543" t="inlineStr">
+        <is>
+          <t>2026-09-30 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3544">
+      <c r="A3544" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B3544" t="inlineStr">
+        <is>
+          <t>EUR/GBP</t>
+        </is>
+      </c>
+      <c r="C3544" t="n">
+        <v>0.85463</v>
+      </c>
+      <c r="D3544" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3544" t="inlineStr">
+        <is>
+          <t>2026-09-30 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3545">
+      <c r="A3545" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B3545" t="inlineStr">
+        <is>
+          <t>EUR/HKD</t>
+        </is>
+      </c>
+      <c r="C3545" t="n">
+        <v>8.9095</v>
+      </c>
+      <c r="D3545" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3545" t="inlineStr">
+        <is>
+          <t>2026-09-30 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3546">
+      <c r="A3546" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B3546" t="inlineStr">
+        <is>
+          <t>EUR/IDR</t>
+        </is>
+      </c>
+      <c r="C3546" t="n">
+        <v>20315.34</v>
+      </c>
+      <c r="D3546" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3546" t="inlineStr">
+        <is>
+          <t>2026-09-30 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3547">
+      <c r="A3547" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B3547" t="inlineStr">
+        <is>
+          <t>EUR/ILS</t>
+        </is>
+      </c>
+      <c r="C3547" t="n">
+        <v>3.4901</v>
+      </c>
+      <c r="D3547" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3547" t="inlineStr">
+        <is>
+          <t>2026-09-30 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3548">
+      <c r="A3548" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B3548" t="inlineStr">
+        <is>
+          <t>EUR/JPY</t>
+        </is>
+      </c>
+      <c r="C3548" t="n">
+        <v>178.27</v>
+      </c>
+      <c r="D3548" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3548" t="inlineStr">
+        <is>
+          <t>2026-09-30 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3549">
+      <c r="A3549" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B3549" t="inlineStr">
+        <is>
+          <t>EUR/KRW</t>
+        </is>
+      </c>
+      <c r="C3549" t="n">
+        <v>1539.06</v>
+      </c>
+      <c r="D3549" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3549" t="inlineStr">
+        <is>
+          <t>2026-09-30 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3550">
+      <c r="A3550" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B3550" t="inlineStr">
+        <is>
+          <t>EUR/MAD</t>
+        </is>
+      </c>
+      <c r="C3550" t="n">
+        <v>10.965569</v>
+      </c>
+      <c r="D3550" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3550" t="inlineStr">
+        <is>
+          <t>2026-09-30 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3551">
+      <c r="A3551" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B3551" t="inlineStr">
+        <is>
+          <t>EUR/PEN</t>
+        </is>
+      </c>
+      <c r="C3551" t="n">
+        <v>3.897351</v>
+      </c>
+      <c r="D3551" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3551" t="inlineStr">
+        <is>
+          <t>2026-09-30 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3552">
+      <c r="A3552" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B3552" t="inlineStr">
+        <is>
+          <t>EUR/PHP</t>
+        </is>
+      </c>
+      <c r="C3552" t="n">
+        <v>71.20399999999999</v>
+      </c>
+      <c r="D3552" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3552" t="inlineStr">
+        <is>
+          <t>2026-09-30 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3553">
+      <c r="A3553" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B3553" t="inlineStr">
+        <is>
+          <t>EUR/RUB</t>
+        </is>
+      </c>
+      <c r="C3553" t="n">
+        <v>95.377284</v>
+      </c>
+      <c r="D3553" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3553" t="inlineStr">
+        <is>
+          <t>2026-09-30 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3554">
+      <c r="A3554" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B3554" t="inlineStr">
+        <is>
+          <t>EUR/SAR</t>
+        </is>
+      </c>
+      <c r="C3554" t="n">
+        <v>4.254047</v>
+      </c>
+      <c r="D3554" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3554" t="inlineStr">
+        <is>
+          <t>2026-09-30 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3555">
+      <c r="A3555" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B3555" t="inlineStr">
+        <is>
+          <t>EUR/SEK</t>
+        </is>
+      </c>
+      <c r="C3555" t="n">
+        <v>11.331</v>
+      </c>
+      <c r="D3555" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3555" t="inlineStr">
+        <is>
+          <t>2026-09-30 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3556">
+      <c r="A3556" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B3556" t="inlineStr">
+        <is>
+          <t>EUR/SGD</t>
+        </is>
+      </c>
+      <c r="C3556" t="n">
+        <v>1.4503</v>
+      </c>
+      <c r="D3556" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3556" t="inlineStr">
+        <is>
+          <t>2026-09-30 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3557">
+      <c r="A3557" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B3557" t="inlineStr">
+        <is>
+          <t>EUR/THB</t>
+        </is>
+      </c>
+      <c r="C3557" t="n">
+        <v>38.113</v>
+      </c>
+      <c r="D3557" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3557" t="inlineStr">
+        <is>
+          <t>2026-09-30 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3558">
+      <c r="A3558" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B3558" t="inlineStr">
+        <is>
+          <t>EUR/TRY</t>
+        </is>
+      </c>
+      <c r="C3558" t="n">
+        <v>55.6596</v>
+      </c>
+      <c r="D3558" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3558" t="inlineStr">
+        <is>
+          <t>2026-09-30 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3559">
+      <c r="A3559" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B3559" t="inlineStr">
+        <is>
+          <t>EUR/USD</t>
+        </is>
+      </c>
+      <c r="C3559" t="n">
+        <v>1.1355</v>
+      </c>
+      <c r="D3559" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3559" t="inlineStr">
+        <is>
+          <t>2026-09-30 07:30 CET</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update currency rates for 2026-10-01
</commit_message>
<xml_diff>
--- a/data/rates.xlsx
+++ b/data/rates.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3559"/>
+  <dimension ref="A1:E3585"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -89393,6 +89393,656 @@
         </is>
       </c>
     </row>
+    <row r="3560">
+      <c r="A3560" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B3560" t="inlineStr">
+        <is>
+          <t>CNY/SGD</t>
+        </is>
+      </c>
+      <c r="C3560" t="n">
+        <v>0.190896</v>
+      </c>
+      <c r="D3560" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3560" t="inlineStr">
+        <is>
+          <t>2026-10-01 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3561">
+      <c r="A3561" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B3561" t="inlineStr">
+        <is>
+          <t>CNY/USD</t>
+        </is>
+      </c>
+      <c r="C3561" t="n">
+        <v>0.149152</v>
+      </c>
+      <c r="D3561" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3561" t="inlineStr">
+        <is>
+          <t>2026-10-01 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3562">
+      <c r="A3562" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B3562" t="inlineStr">
+        <is>
+          <t>EUR/AED</t>
+        </is>
+      </c>
+      <c r="C3562" t="n">
+        <v>4.16537</v>
+      </c>
+      <c r="D3562" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3562" t="inlineStr">
+        <is>
+          <t>2026-10-01 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3563">
+      <c r="A3563" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B3563" t="inlineStr">
+        <is>
+          <t>EUR/ARS</t>
+        </is>
+      </c>
+      <c r="C3563" t="n">
+        <v>1721.180525</v>
+      </c>
+      <c r="D3563" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3563" t="inlineStr">
+        <is>
+          <t>2026-10-01 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3564">
+      <c r="A3564" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B3564" t="inlineStr">
+        <is>
+          <t>EUR/BRL</t>
+        </is>
+      </c>
+      <c r="C3564" t="n">
+        <v>5.862</v>
+      </c>
+      <c r="D3564" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3564" t="inlineStr">
+        <is>
+          <t>2026-10-01 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3565">
+      <c r="A3565" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B3565" t="inlineStr">
+        <is>
+          <t>EUR/CHF</t>
+        </is>
+      </c>
+      <c r="C3565" t="n">
+        <v>0.9437</v>
+      </c>
+      <c r="D3565" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3565" t="inlineStr">
+        <is>
+          <t>2026-10-01 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3566">
+      <c r="A3566" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B3566" t="inlineStr">
+        <is>
+          <t>EUR/CLP</t>
+        </is>
+      </c>
+      <c r="C3566" t="n">
+        <v>1105.034018</v>
+      </c>
+      <c r="D3566" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3566" t="inlineStr">
+        <is>
+          <t>2026-10-01 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3567">
+      <c r="A3567" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B3567" t="inlineStr">
+        <is>
+          <t>EUR/CNY</t>
+        </is>
+      </c>
+      <c r="C3567" t="n">
+        <v>7.5748</v>
+      </c>
+      <c r="D3567" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3567" t="inlineStr">
+        <is>
+          <t>2026-10-01 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3568">
+      <c r="A3568" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B3568" t="inlineStr">
+        <is>
+          <t>EUR/COP</t>
+        </is>
+      </c>
+      <c r="C3568" t="n">
+        <v>3788.161988</v>
+      </c>
+      <c r="D3568" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3568" t="inlineStr">
+        <is>
+          <t>2026-10-01 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3569">
+      <c r="A3569" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B3569" t="inlineStr">
+        <is>
+          <t>EUR/DKK</t>
+        </is>
+      </c>
+      <c r="C3569" t="n">
+        <v>7.4758</v>
+      </c>
+      <c r="D3569" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3569" t="inlineStr">
+        <is>
+          <t>2026-10-01 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3570">
+      <c r="A3570" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B3570" t="inlineStr">
+        <is>
+          <t>EUR/GBP</t>
+        </is>
+      </c>
+      <c r="C3570" t="n">
+        <v>0.85373</v>
+      </c>
+      <c r="D3570" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3570" t="inlineStr">
+        <is>
+          <t>2026-10-01 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3571">
+      <c r="A3571" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B3571" t="inlineStr">
+        <is>
+          <t>EUR/HKD</t>
+        </is>
+      </c>
+      <c r="C3571" t="n">
+        <v>8.8658</v>
+      </c>
+      <c r="D3571" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3571" t="inlineStr">
+        <is>
+          <t>2026-10-01 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3572">
+      <c r="A3572" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B3572" t="inlineStr">
+        <is>
+          <t>EUR/IDR</t>
+        </is>
+      </c>
+      <c r="C3572" t="n">
+        <v>20274.71</v>
+      </c>
+      <c r="D3572" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3572" t="inlineStr">
+        <is>
+          <t>2026-10-01 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3573">
+      <c r="A3573" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B3573" t="inlineStr">
+        <is>
+          <t>EUR/ILS</t>
+        </is>
+      </c>
+      <c r="C3573" t="n">
+        <v>3.4755</v>
+      </c>
+      <c r="D3573" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3573" t="inlineStr">
+        <is>
+          <t>2026-10-01 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3574">
+      <c r="A3574" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B3574" t="inlineStr">
+        <is>
+          <t>EUR/JPY</t>
+        </is>
+      </c>
+      <c r="C3574" t="n">
+        <v>178.49</v>
+      </c>
+      <c r="D3574" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3574" t="inlineStr">
+        <is>
+          <t>2026-10-01 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3575">
+      <c r="A3575" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B3575" t="inlineStr">
+        <is>
+          <t>EUR/KRW</t>
+        </is>
+      </c>
+      <c r="C3575" t="n">
+        <v>1537.96</v>
+      </c>
+      <c r="D3575" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3575" t="inlineStr">
+        <is>
+          <t>2026-10-01 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3576">
+      <c r="A3576" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B3576" t="inlineStr">
+        <is>
+          <t>EUR/MAD</t>
+        </is>
+      </c>
+      <c r="C3576" t="n">
+        <v>10.999787</v>
+      </c>
+      <c r="D3576" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3576" t="inlineStr">
+        <is>
+          <t>2026-10-01 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3577">
+      <c r="A3577" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B3577" t="inlineStr">
+        <is>
+          <t>EUR/PEN</t>
+        </is>
+      </c>
+      <c r="C3577" t="n">
+        <v>3.90533</v>
+      </c>
+      <c r="D3577" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3577" t="inlineStr">
+        <is>
+          <t>2026-10-01 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3578">
+      <c r="A3578" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B3578" t="inlineStr">
+        <is>
+          <t>EUR/PHP</t>
+        </is>
+      </c>
+      <c r="C3578" t="n">
+        <v>70.95</v>
+      </c>
+      <c r="D3578" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3578" t="inlineStr">
+        <is>
+          <t>2026-10-01 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3579">
+      <c r="A3579" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B3579" t="inlineStr">
+        <is>
+          <t>EUR/RUB</t>
+        </is>
+      </c>
+      <c r="C3579" t="n">
+        <v>94.867806</v>
+      </c>
+      <c r="D3579" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3579" t="inlineStr">
+        <is>
+          <t>2026-10-01 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3580">
+      <c r="A3580" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B3580" t="inlineStr">
+        <is>
+          <t>EUR/SAR</t>
+        </is>
+      </c>
+      <c r="C3580" t="n">
+        <v>4.253271</v>
+      </c>
+      <c r="D3580" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3580" t="inlineStr">
+        <is>
+          <t>2026-10-01 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3581">
+      <c r="A3581" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B3581" t="inlineStr">
+        <is>
+          <t>EUR/SEK</t>
+        </is>
+      </c>
+      <c r="C3581" t="n">
+        <v>11.331</v>
+      </c>
+      <c r="D3581" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3581" t="inlineStr">
+        <is>
+          <t>2026-10-01 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3582">
+      <c r="A3582" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B3582" t="inlineStr">
+        <is>
+          <t>EUR/SGD</t>
+        </is>
+      </c>
+      <c r="C3582" t="n">
+        <v>1.446</v>
+      </c>
+      <c r="D3582" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3582" t="inlineStr">
+        <is>
+          <t>2026-10-01 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3583">
+      <c r="A3583" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B3583" t="inlineStr">
+        <is>
+          <t>EUR/THB</t>
+        </is>
+      </c>
+      <c r="C3583" t="n">
+        <v>38.023</v>
+      </c>
+      <c r="D3583" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3583" t="inlineStr">
+        <is>
+          <t>2026-10-01 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3584">
+      <c r="A3584" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B3584" t="inlineStr">
+        <is>
+          <t>EUR/TRY</t>
+        </is>
+      </c>
+      <c r="C3584" t="n">
+        <v>55.3993</v>
+      </c>
+      <c r="D3584" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3584" t="inlineStr">
+        <is>
+          <t>2026-10-01 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3585">
+      <c r="A3585" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B3585" t="inlineStr">
+        <is>
+          <t>EUR/USD</t>
+        </is>
+      </c>
+      <c r="C3585" t="n">
+        <v>1.1298</v>
+      </c>
+      <c r="D3585" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3585" t="inlineStr">
+        <is>
+          <t>2026-10-01 07:30 CET</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update currency rates for 2026-10-02
</commit_message>
<xml_diff>
--- a/data/rates.xlsx
+++ b/data/rates.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3585"/>
+  <dimension ref="A1:E3611"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -90043,6 +90043,656 @@
         </is>
       </c>
     </row>
+    <row r="3586">
+      <c r="A3586" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B3586" t="inlineStr">
+        <is>
+          <t>CNY/SGD</t>
+        </is>
+      </c>
+      <c r="C3586" t="n">
+        <v>0.190887</v>
+      </c>
+      <c r="D3586" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3586" t="inlineStr">
+        <is>
+          <t>2026-10-02 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3587">
+      <c r="A3587" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B3587" t="inlineStr">
+        <is>
+          <t>CNY/USD</t>
+        </is>
+      </c>
+      <c r="C3587" t="n">
+        <v>0.149152</v>
+      </c>
+      <c r="D3587" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3587" t="inlineStr">
+        <is>
+          <t>2026-10-02 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3588">
+      <c r="A3588" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B3588" t="inlineStr">
+        <is>
+          <t>EUR/AED</t>
+        </is>
+      </c>
+      <c r="C3588" t="n">
+        <v>4.139036</v>
+      </c>
+      <c r="D3588" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3588" t="inlineStr">
+        <is>
+          <t>2026-10-02 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3589">
+      <c r="A3589" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B3589" t="inlineStr">
+        <is>
+          <t>EUR/ARS</t>
+        </is>
+      </c>
+      <c r="C3589" t="n">
+        <v>1716.728456</v>
+      </c>
+      <c r="D3589" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3589" t="inlineStr">
+        <is>
+          <t>2026-10-02 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3590">
+      <c r="A3590" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B3590" t="inlineStr">
+        <is>
+          <t>EUR/BRL</t>
+        </is>
+      </c>
+      <c r="C3590" t="n">
+        <v>5.861</v>
+      </c>
+      <c r="D3590" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3590" t="inlineStr">
+        <is>
+          <t>2026-10-02 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3591">
+      <c r="A3591" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B3591" t="inlineStr">
+        <is>
+          <t>EUR/CHF</t>
+        </is>
+      </c>
+      <c r="C3591" t="n">
+        <v>0.9278999999999999</v>
+      </c>
+      <c r="D3591" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3591" t="inlineStr">
+        <is>
+          <t>2026-10-02 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3592">
+      <c r="A3592" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B3592" t="inlineStr">
+        <is>
+          <t>EUR/CLP</t>
+        </is>
+      </c>
+      <c r="C3592" t="n">
+        <v>1099.79502</v>
+      </c>
+      <c r="D3592" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3592" t="inlineStr">
+        <is>
+          <t>2026-10-02 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3593">
+      <c r="A3593" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B3593" t="inlineStr">
+        <is>
+          <t>EUR/CNY</t>
+        </is>
+      </c>
+      <c r="C3593" t="n">
+        <v>7.5259</v>
+      </c>
+      <c r="D3593" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3593" t="inlineStr">
+        <is>
+          <t>2026-10-02 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3594">
+      <c r="A3594" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B3594" t="inlineStr">
+        <is>
+          <t>EUR/COP</t>
+        </is>
+      </c>
+      <c r="C3594" t="n">
+        <v>3734.98195</v>
+      </c>
+      <c r="D3594" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3594" t="inlineStr">
+        <is>
+          <t>2026-10-02 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3595">
+      <c r="A3595" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B3595" t="inlineStr">
+        <is>
+          <t>EUR/DKK</t>
+        </is>
+      </c>
+      <c r="C3595" t="n">
+        <v>7.4736</v>
+      </c>
+      <c r="D3595" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3595" t="inlineStr">
+        <is>
+          <t>2026-10-02 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3596">
+      <c r="A3596" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B3596" t="inlineStr">
+        <is>
+          <t>EUR/GBP</t>
+        </is>
+      </c>
+      <c r="C3596" t="n">
+        <v>0.85033</v>
+      </c>
+      <c r="D3596" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3596" t="inlineStr">
+        <is>
+          <t>2026-10-02 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3597">
+      <c r="A3597" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B3597" t="inlineStr">
+        <is>
+          <t>EUR/HKD</t>
+        </is>
+      </c>
+      <c r="C3597" t="n">
+        <v>8.808400000000001</v>
+      </c>
+      <c r="D3597" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3597" t="inlineStr">
+        <is>
+          <t>2026-10-02 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3598">
+      <c r="A3598" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B3598" t="inlineStr">
+        <is>
+          <t>EUR/IDR</t>
+        </is>
+      </c>
+      <c r="C3598" t="n">
+        <v>20149.32</v>
+      </c>
+      <c r="D3598" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3598" t="inlineStr">
+        <is>
+          <t>2026-10-02 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3599">
+      <c r="A3599" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B3599" t="inlineStr">
+        <is>
+          <t>EUR/ILS</t>
+        </is>
+      </c>
+      <c r="C3599" t="n">
+        <v>3.4408</v>
+      </c>
+      <c r="D3599" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3599" t="inlineStr">
+        <is>
+          <t>2026-10-02 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3600">
+      <c r="A3600" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B3600" t="inlineStr">
+        <is>
+          <t>EUR/JPY</t>
+        </is>
+      </c>
+      <c r="C3600" t="n">
+        <v>176.99</v>
+      </c>
+      <c r="D3600" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3600" t="inlineStr">
+        <is>
+          <t>2026-10-02 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3601">
+      <c r="A3601" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B3601" t="inlineStr">
+        <is>
+          <t>EUR/KRW</t>
+        </is>
+      </c>
+      <c r="C3601" t="n">
+        <v>1513.44</v>
+      </c>
+      <c r="D3601" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3601" t="inlineStr">
+        <is>
+          <t>2026-10-02 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3602">
+      <c r="A3602" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B3602" t="inlineStr">
+        <is>
+          <t>EUR/MAD</t>
+        </is>
+      </c>
+      <c r="C3602" t="n">
+        <v>11.01036</v>
+      </c>
+      <c r="D3602" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3602" t="inlineStr">
+        <is>
+          <t>2026-10-02 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3603">
+      <c r="A3603" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B3603" t="inlineStr">
+        <is>
+          <t>EUR/PEN</t>
+        </is>
+      </c>
+      <c r="C3603" t="n">
+        <v>3.890053</v>
+      </c>
+      <c r="D3603" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3603" t="inlineStr">
+        <is>
+          <t>2026-10-02 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3604">
+      <c r="A3604" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B3604" t="inlineStr">
+        <is>
+          <t>EUR/PHP</t>
+        </is>
+      </c>
+      <c r="C3604" t="n">
+        <v>70.265</v>
+      </c>
+      <c r="D3604" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3604" t="inlineStr">
+        <is>
+          <t>2026-10-02 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3605">
+      <c r="A3605" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B3605" t="inlineStr">
+        <is>
+          <t>EUR/RUB</t>
+        </is>
+      </c>
+      <c r="C3605" t="n">
+        <v>94.241169</v>
+      </c>
+      <c r="D3605" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3605" t="inlineStr">
+        <is>
+          <t>2026-10-02 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3606">
+      <c r="A3606" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B3606" t="inlineStr">
+        <is>
+          <t>EUR/SAR</t>
+        </is>
+      </c>
+      <c r="C3606" t="n">
+        <v>4.226382</v>
+      </c>
+      <c r="D3606" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3606" t="inlineStr">
+        <is>
+          <t>2026-10-02 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3607">
+      <c r="A3607" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B3607" t="inlineStr">
+        <is>
+          <t>EUR/SEK</t>
+        </is>
+      </c>
+      <c r="C3607" t="n">
+        <v>11.29</v>
+      </c>
+      <c r="D3607" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3607" t="inlineStr">
+        <is>
+          <t>2026-10-02 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3608">
+      <c r="A3608" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B3608" t="inlineStr">
+        <is>
+          <t>EUR/SGD</t>
+        </is>
+      </c>
+      <c r="C3608" t="n">
+        <v>1.4366</v>
+      </c>
+      <c r="D3608" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3608" t="inlineStr">
+        <is>
+          <t>2026-10-02 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3609">
+      <c r="A3609" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B3609" t="inlineStr">
+        <is>
+          <t>EUR/THB</t>
+        </is>
+      </c>
+      <c r="C3609" t="n">
+        <v>37.71</v>
+      </c>
+      <c r="D3609" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3609" t="inlineStr">
+        <is>
+          <t>2026-10-02 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3610">
+      <c r="A3610" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B3610" t="inlineStr">
+        <is>
+          <t>EUR/TRY</t>
+        </is>
+      </c>
+      <c r="C3610" t="n">
+        <v>55.165</v>
+      </c>
+      <c r="D3610" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3610" t="inlineStr">
+        <is>
+          <t>2026-10-02 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3611">
+      <c r="A3611" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B3611" t="inlineStr">
+        <is>
+          <t>EUR/USD</t>
+        </is>
+      </c>
+      <c r="C3611" t="n">
+        <v>1.1225</v>
+      </c>
+      <c r="D3611" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3611" t="inlineStr">
+        <is>
+          <t>2026-10-02 07:30 CET</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update currency rates for 2026-10-05
</commit_message>
<xml_diff>
--- a/data/rates.xlsx
+++ b/data/rates.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3611"/>
+  <dimension ref="A1:E3637"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -90693,6 +90693,656 @@
         </is>
       </c>
     </row>
+    <row r="3612">
+      <c r="A3612" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B3612" t="inlineStr">
+        <is>
+          <t>CNY/SGD</t>
+        </is>
+      </c>
+      <c r="C3612" t="n">
+        <v>0.190953</v>
+      </c>
+      <c r="D3612" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3612" t="inlineStr">
+        <is>
+          <t>2026-10-06 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3613">
+      <c r="A3613" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B3613" t="inlineStr">
+        <is>
+          <t>CNY/USD</t>
+        </is>
+      </c>
+      <c r="C3613" t="n">
+        <v>0.149152</v>
+      </c>
+      <c r="D3613" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3613" t="inlineStr">
+        <is>
+          <t>2026-10-06 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3614">
+      <c r="A3614" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B3614" t="inlineStr">
+        <is>
+          <t>EUR/AED</t>
+        </is>
+      </c>
+      <c r="C3614" t="n">
+        <v>4.131859</v>
+      </c>
+      <c r="D3614" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3614" t="inlineStr">
+        <is>
+          <t>2026-10-06 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3615">
+      <c r="A3615" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B3615" t="inlineStr">
+        <is>
+          <t>EUR/ARS</t>
+        </is>
+      </c>
+      <c r="C3615" t="n">
+        <v>1713.595414</v>
+      </c>
+      <c r="D3615" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3615" t="inlineStr">
+        <is>
+          <t>2026-10-06 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3616">
+      <c r="A3616" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B3616" t="inlineStr">
+        <is>
+          <t>EUR/BRL</t>
+        </is>
+      </c>
+      <c r="C3616" t="n">
+        <v>5.5849</v>
+      </c>
+      <c r="D3616" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3616" t="inlineStr">
+        <is>
+          <t>2026-10-06 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3617">
+      <c r="A3617" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B3617" t="inlineStr">
+        <is>
+          <t>EUR/CHF</t>
+        </is>
+      </c>
+      <c r="C3617" t="n">
+        <v>0.9311</v>
+      </c>
+      <c r="D3617" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3617" t="inlineStr">
+        <is>
+          <t>2026-10-06 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3618">
+      <c r="A3618" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B3618" t="inlineStr">
+        <is>
+          <t>EUR/CLP</t>
+        </is>
+      </c>
+      <c r="C3618" t="n">
+        <v>1110.206874</v>
+      </c>
+      <c r="D3618" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3618" t="inlineStr">
+        <is>
+          <t>2026-10-06 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3619">
+      <c r="A3619" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B3619" t="inlineStr">
+        <is>
+          <t>EUR/CNY</t>
+        </is>
+      </c>
+      <c r="C3619" t="n">
+        <v>7.5118</v>
+      </c>
+      <c r="D3619" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3619" t="inlineStr">
+        <is>
+          <t>2026-10-06 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3620">
+      <c r="A3620" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B3620" t="inlineStr">
+        <is>
+          <t>EUR/COP</t>
+        </is>
+      </c>
+      <c r="C3620" t="n">
+        <v>3716.852803</v>
+      </c>
+      <c r="D3620" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3620" t="inlineStr">
+        <is>
+          <t>2026-10-06 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3621">
+      <c r="A3621" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B3621" t="inlineStr">
+        <is>
+          <t>EUR/DKK</t>
+        </is>
+      </c>
+      <c r="C3621" t="n">
+        <v>7.4745</v>
+      </c>
+      <c r="D3621" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3621" t="inlineStr">
+        <is>
+          <t>2026-10-06 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3622">
+      <c r="A3622" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B3622" t="inlineStr">
+        <is>
+          <t>EUR/GBP</t>
+        </is>
+      </c>
+      <c r="C3622" t="n">
+        <v>0.8472</v>
+      </c>
+      <c r="D3622" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3622" t="inlineStr">
+        <is>
+          <t>2026-10-06 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3623">
+      <c r="A3623" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B3623" t="inlineStr">
+        <is>
+          <t>EUR/HKD</t>
+        </is>
+      </c>
+      <c r="C3623" t="n">
+        <v>8.7925</v>
+      </c>
+      <c r="D3623" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3623" t="inlineStr">
+        <is>
+          <t>2026-10-06 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3624">
+      <c r="A3624" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B3624" t="inlineStr">
+        <is>
+          <t>EUR/IDR</t>
+        </is>
+      </c>
+      <c r="C3624" t="n">
+        <v>20069.89</v>
+      </c>
+      <c r="D3624" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3624" t="inlineStr">
+        <is>
+          <t>2026-10-06 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3625">
+      <c r="A3625" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B3625" t="inlineStr">
+        <is>
+          <t>EUR/ILS</t>
+        </is>
+      </c>
+      <c r="C3625" t="n">
+        <v>3.431</v>
+      </c>
+      <c r="D3625" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3625" t="inlineStr">
+        <is>
+          <t>2026-10-06 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3626">
+      <c r="A3626" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B3626" t="inlineStr">
+        <is>
+          <t>EUR/JPY</t>
+        </is>
+      </c>
+      <c r="C3626" t="n">
+        <v>177.28</v>
+      </c>
+      <c r="D3626" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3626" t="inlineStr">
+        <is>
+          <t>2026-10-06 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3627">
+      <c r="A3627" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B3627" t="inlineStr">
+        <is>
+          <t>EUR/KRW</t>
+        </is>
+      </c>
+      <c r="C3627" t="n">
+        <v>1505.8</v>
+      </c>
+      <c r="D3627" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3627" t="inlineStr">
+        <is>
+          <t>2026-10-06 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3628">
+      <c r="A3628" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B3628" t="inlineStr">
+        <is>
+          <t>EUR/MAD</t>
+        </is>
+      </c>
+      <c r="C3628" t="n">
+        <v>11.144826</v>
+      </c>
+      <c r="D3628" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3628" t="inlineStr">
+        <is>
+          <t>2026-10-06 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3629">
+      <c r="A3629" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B3629" t="inlineStr">
+        <is>
+          <t>EUR/PEN</t>
+        </is>
+      </c>
+      <c r="C3629" t="n">
+        <v>3.888016</v>
+      </c>
+      <c r="D3629" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3629" t="inlineStr">
+        <is>
+          <t>2026-10-06 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3630">
+      <c r="A3630" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B3630" t="inlineStr">
+        <is>
+          <t>EUR/PHP</t>
+        </is>
+      </c>
+      <c r="C3630" t="n">
+        <v>70.21899999999999</v>
+      </c>
+      <c r="D3630" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3630" t="inlineStr">
+        <is>
+          <t>2026-10-06 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3631">
+      <c r="A3631" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B3631" t="inlineStr">
+        <is>
+          <t>EUR/RUB</t>
+        </is>
+      </c>
+      <c r="C3631" t="n">
+        <v>94.19824800000001</v>
+      </c>
+      <c r="D3631" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3631" t="inlineStr">
+        <is>
+          <t>2026-10-06 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3632">
+      <c r="A3632" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B3632" t="inlineStr">
+        <is>
+          <t>EUR/SAR</t>
+        </is>
+      </c>
+      <c r="C3632" t="n">
+        <v>4.219052</v>
+      </c>
+      <c r="D3632" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3632" t="inlineStr">
+        <is>
+          <t>2026-10-06 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3633">
+      <c r="A3633" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B3633" t="inlineStr">
+        <is>
+          <t>EUR/SEK</t>
+        </is>
+      </c>
+      <c r="C3633" t="n">
+        <v>11.2525</v>
+      </c>
+      <c r="D3633" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3633" t="inlineStr">
+        <is>
+          <t>2026-10-06 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3634">
+      <c r="A3634" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B3634" t="inlineStr">
+        <is>
+          <t>EUR/SGD</t>
+        </is>
+      </c>
+      <c r="C3634" t="n">
+        <v>1.4344</v>
+      </c>
+      <c r="D3634" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3634" t="inlineStr">
+        <is>
+          <t>2026-10-06 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3635">
+      <c r="A3635" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B3635" t="inlineStr">
+        <is>
+          <t>EUR/THB</t>
+        </is>
+      </c>
+      <c r="C3635" t="n">
+        <v>37.752</v>
+      </c>
+      <c r="D3635" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3635" t="inlineStr">
+        <is>
+          <t>2026-10-06 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3636">
+      <c r="A3636" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B3636" t="inlineStr">
+        <is>
+          <t>EUR/TRY</t>
+        </is>
+      </c>
+      <c r="C3636" t="n">
+        <v>55.0755</v>
+      </c>
+      <c r="D3636" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3636" t="inlineStr">
+        <is>
+          <t>2026-10-06 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3637">
+      <c r="A3637" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B3637" t="inlineStr">
+        <is>
+          <t>EUR/USD</t>
+        </is>
+      </c>
+      <c r="C3637" t="n">
+        <v>1.1204</v>
+      </c>
+      <c r="D3637" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3637" t="inlineStr">
+        <is>
+          <t>2026-10-06 07:30 CET</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update currency rates for 2026-10-06
</commit_message>
<xml_diff>
--- a/data/rates.xlsx
+++ b/data/rates.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3637"/>
+  <dimension ref="A1:E3663"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -91343,6 +91343,656 @@
         </is>
       </c>
     </row>
+    <row r="3638">
+      <c r="A3638" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B3638" t="inlineStr">
+        <is>
+          <t>CNY/SGD</t>
+        </is>
+      </c>
+      <c r="C3638" t="n">
+        <v>0.190486</v>
+      </c>
+      <c r="D3638" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3638" t="inlineStr">
+        <is>
+          <t>2026-10-06 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3639">
+      <c r="A3639" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B3639" t="inlineStr">
+        <is>
+          <t>CNY/USD</t>
+        </is>
+      </c>
+      <c r="C3639" t="n">
+        <v>0.149152</v>
+      </c>
+      <c r="D3639" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3639" t="inlineStr">
+        <is>
+          <t>2026-10-06 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3640">
+      <c r="A3640" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B3640" t="inlineStr">
+        <is>
+          <t>EUR/AED</t>
+        </is>
+      </c>
+      <c r="C3640" t="n">
+        <v>4.117489</v>
+      </c>
+      <c r="D3640" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3640" t="inlineStr">
+        <is>
+          <t>2026-10-06 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3641">
+      <c r="A3641" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B3641" t="inlineStr">
+        <is>
+          <t>EUR/ARS</t>
+        </is>
+      </c>
+      <c r="C3641" t="n">
+        <v>1703.331974</v>
+      </c>
+      <c r="D3641" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3641" t="inlineStr">
+        <is>
+          <t>2026-10-06 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3642">
+      <c r="A3642" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B3642" t="inlineStr">
+        <is>
+          <t>EUR/BRL</t>
+        </is>
+      </c>
+      <c r="C3642" t="n">
+        <v>5.5991</v>
+      </c>
+      <c r="D3642" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3642" t="inlineStr">
+        <is>
+          <t>2026-10-06 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3643">
+      <c r="A3643" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B3643" t="inlineStr">
+        <is>
+          <t>EUR/CHF</t>
+        </is>
+      </c>
+      <c r="C3643" t="n">
+        <v>0.9359</v>
+      </c>
+      <c r="D3643" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3643" t="inlineStr">
+        <is>
+          <t>2026-10-06 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3644">
+      <c r="A3644" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B3644" t="inlineStr">
+        <is>
+          <t>EUR/CLP</t>
+        </is>
+      </c>
+      <c r="C3644" t="n">
+        <v>1107.320731</v>
+      </c>
+      <c r="D3644" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3644" t="inlineStr">
+        <is>
+          <t>2026-10-06 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3645">
+      <c r="A3645" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B3645" t="inlineStr">
+        <is>
+          <t>EUR/CNY</t>
+        </is>
+      </c>
+      <c r="C3645" t="n">
+        <v>7.5554</v>
+      </c>
+      <c r="D3645" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3645" t="inlineStr">
+        <is>
+          <t>2026-10-06 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3646">
+      <c r="A3646" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B3646" t="inlineStr">
+        <is>
+          <t>EUR/COP</t>
+        </is>
+      </c>
+      <c r="C3646" t="n">
+        <v>3676.469436</v>
+      </c>
+      <c r="D3646" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3646" t="inlineStr">
+        <is>
+          <t>2026-10-06 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3647">
+      <c r="A3647" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B3647" t="inlineStr">
+        <is>
+          <t>EUR/DKK</t>
+        </is>
+      </c>
+      <c r="C3647" t="n">
+        <v>7.4747</v>
+      </c>
+      <c r="D3647" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3647" t="inlineStr">
+        <is>
+          <t>2026-10-06 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3648">
+      <c r="A3648" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B3648" t="inlineStr">
+        <is>
+          <t>EUR/GBP</t>
+        </is>
+      </c>
+      <c r="C3648" t="n">
+        <v>0.8488</v>
+      </c>
+      <c r="D3648" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3648" t="inlineStr">
+        <is>
+          <t>2026-10-06 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3649">
+      <c r="A3649" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B3649" t="inlineStr">
+        <is>
+          <t>EUR/HKD</t>
+        </is>
+      </c>
+      <c r="C3649" t="n">
+        <v>8.8438</v>
+      </c>
+      <c r="D3649" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3649" t="inlineStr">
+        <is>
+          <t>2026-10-06 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3650">
+      <c r="A3650" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B3650" t="inlineStr">
+        <is>
+          <t>EUR/IDR</t>
+        </is>
+      </c>
+      <c r="C3650" t="n">
+        <v>20104.8</v>
+      </c>
+      <c r="D3650" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3650" t="inlineStr">
+        <is>
+          <t>2026-10-06 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3651">
+      <c r="A3651" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B3651" t="inlineStr">
+        <is>
+          <t>EUR/ILS</t>
+        </is>
+      </c>
+      <c r="C3651" t="n">
+        <v>3.4348</v>
+      </c>
+      <c r="D3651" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3651" t="inlineStr">
+        <is>
+          <t>2026-10-06 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3652">
+      <c r="A3652" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B3652" t="inlineStr">
+        <is>
+          <t>EUR/JPY</t>
+        </is>
+      </c>
+      <c r="C3652" t="n">
+        <v>178.15</v>
+      </c>
+      <c r="D3652" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3652" t="inlineStr">
+        <is>
+          <t>2026-10-06 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3653">
+      <c r="A3653" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B3653" t="inlineStr">
+        <is>
+          <t>EUR/KRW</t>
+        </is>
+      </c>
+      <c r="C3653" t="n">
+        <v>1508.67</v>
+      </c>
+      <c r="D3653" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3653" t="inlineStr">
+        <is>
+          <t>2026-10-06 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3654">
+      <c r="A3654" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B3654" t="inlineStr">
+        <is>
+          <t>EUR/MAD</t>
+        </is>
+      </c>
+      <c r="C3654" t="n">
+        <v>11.17856</v>
+      </c>
+      <c r="D3654" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3654" t="inlineStr">
+        <is>
+          <t>2026-10-06 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3655">
+      <c r="A3655" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B3655" t="inlineStr">
+        <is>
+          <t>EUR/PEN</t>
+        </is>
+      </c>
+      <c r="C3655" t="n">
+        <v>3.858464</v>
+      </c>
+      <c r="D3655" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3655" t="inlineStr">
+        <is>
+          <t>2026-10-06 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3656">
+      <c r="A3656" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B3656" t="inlineStr">
+        <is>
+          <t>EUR/PHP</t>
+        </is>
+      </c>
+      <c r="C3656" t="n">
+        <v>70.702</v>
+      </c>
+      <c r="D3656" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3656" t="inlineStr">
+        <is>
+          <t>2026-10-06 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3657">
+      <c r="A3657" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B3657" t="inlineStr">
+        <is>
+          <t>EUR/RUB</t>
+        </is>
+      </c>
+      <c r="C3657" t="n">
+        <v>95.487292</v>
+      </c>
+      <c r="D3657" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3657" t="inlineStr">
+        <is>
+          <t>2026-10-06 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3658">
+      <c r="A3658" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B3658" t="inlineStr">
+        <is>
+          <t>EUR/SAR</t>
+        </is>
+      </c>
+      <c r="C3658" t="n">
+        <v>4.204379</v>
+      </c>
+      <c r="D3658" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3658" t="inlineStr">
+        <is>
+          <t>2026-10-06 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3659">
+      <c r="A3659" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B3659" t="inlineStr">
+        <is>
+          <t>EUR/SEK</t>
+        </is>
+      </c>
+      <c r="C3659" t="n">
+        <v>11.2425</v>
+      </c>
+      <c r="D3659" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3659" t="inlineStr">
+        <is>
+          <t>2026-10-06 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3660">
+      <c r="A3660" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B3660" t="inlineStr">
+        <is>
+          <t>EUR/SGD</t>
+        </is>
+      </c>
+      <c r="C3660" t="n">
+        <v>1.4392</v>
+      </c>
+      <c r="D3660" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3660" t="inlineStr">
+        <is>
+          <t>2026-10-06 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3661">
+      <c r="A3661" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B3661" t="inlineStr">
+        <is>
+          <t>EUR/THB</t>
+        </is>
+      </c>
+      <c r="C3661" t="n">
+        <v>37.836</v>
+      </c>
+      <c r="D3661" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3661" t="inlineStr">
+        <is>
+          <t>2026-10-06 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3662">
+      <c r="A3662" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B3662" t="inlineStr">
+        <is>
+          <t>EUR/TRY</t>
+        </is>
+      </c>
+      <c r="C3662" t="n">
+        <v>55.4196</v>
+      </c>
+      <c r="D3662" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3662" t="inlineStr">
+        <is>
+          <t>2026-10-06 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3663">
+      <c r="A3663" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B3663" t="inlineStr">
+        <is>
+          <t>EUR/USD</t>
+        </is>
+      </c>
+      <c r="C3663" t="n">
+        <v>1.1269</v>
+      </c>
+      <c r="D3663" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3663" t="inlineStr">
+        <is>
+          <t>2026-10-06 07:30 CET</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update currency rates for 2026-10-07
</commit_message>
<xml_diff>
--- a/data/rates.xlsx
+++ b/data/rates.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3663"/>
+  <dimension ref="A1:E3689"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -91993,6 +91993,656 @@
         </is>
       </c>
     </row>
+    <row r="3664">
+      <c r="A3664" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B3664" t="inlineStr">
+        <is>
+          <t>CNY/SGD</t>
+        </is>
+      </c>
+      <c r="C3664" t="n">
+        <v>0.190974</v>
+      </c>
+      <c r="D3664" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3664" t="inlineStr">
+        <is>
+          <t>2026-10-08 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3665">
+      <c r="A3665" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B3665" t="inlineStr">
+        <is>
+          <t>CNY/USD</t>
+        </is>
+      </c>
+      <c r="C3665" t="n">
+        <v>0.149152</v>
+      </c>
+      <c r="D3665" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3665" t="inlineStr">
+        <is>
+          <t>2026-10-08 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3666">
+      <c r="A3666" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B3666" t="inlineStr">
+        <is>
+          <t>EUR/AED</t>
+        </is>
+      </c>
+      <c r="C3666" t="n">
+        <v>4.13222</v>
+      </c>
+      <c r="D3666" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3666" t="inlineStr">
+        <is>
+          <t>2026-10-08 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3667">
+      <c r="A3667" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B3667" t="inlineStr">
+        <is>
+          <t>EUR/ARS</t>
+        </is>
+      </c>
+      <c r="C3667" t="n">
+        <v>1710.609777</v>
+      </c>
+      <c r="D3667" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3667" t="inlineStr">
+        <is>
+          <t>2026-10-08 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3668">
+      <c r="A3668" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B3668" t="inlineStr">
+        <is>
+          <t>EUR/BRL</t>
+        </is>
+      </c>
+      <c r="C3668" t="n">
+        <v>5.5953</v>
+      </c>
+      <c r="D3668" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3668" t="inlineStr">
+        <is>
+          <t>2026-10-08 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3669">
+      <c r="A3669" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B3669" t="inlineStr">
+        <is>
+          <t>EUR/CHF</t>
+        </is>
+      </c>
+      <c r="C3669" t="n">
+        <v>0.9308999999999999</v>
+      </c>
+      <c r="D3669" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3669" t="inlineStr">
+        <is>
+          <t>2026-10-08 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3670">
+      <c r="A3670" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B3670" t="inlineStr">
+        <is>
+          <t>EUR/CLP</t>
+        </is>
+      </c>
+      <c r="C3670" t="n">
+        <v>1093.493955</v>
+      </c>
+      <c r="D3670" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3670" t="inlineStr">
+        <is>
+          <t>2026-10-08 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3671">
+      <c r="A3671" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B3671" t="inlineStr">
+        <is>
+          <t>EUR/CNY</t>
+        </is>
+      </c>
+      <c r="C3671" t="n">
+        <v>7.4937</v>
+      </c>
+      <c r="D3671" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3671" t="inlineStr">
+        <is>
+          <t>2026-10-08 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3672">
+      <c r="A3672" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B3672" t="inlineStr">
+        <is>
+          <t>EUR/COP</t>
+        </is>
+      </c>
+      <c r="C3672" t="n">
+        <v>3599.147884</v>
+      </c>
+      <c r="D3672" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3672" t="inlineStr">
+        <is>
+          <t>2026-10-08 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3673">
+      <c r="A3673" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B3673" t="inlineStr">
+        <is>
+          <t>EUR/DKK</t>
+        </is>
+      </c>
+      <c r="C3673" t="n">
+        <v>7.4745</v>
+      </c>
+      <c r="D3673" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3673" t="inlineStr">
+        <is>
+          <t>2026-10-08 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3674">
+      <c r="A3674" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B3674" t="inlineStr">
+        <is>
+          <t>EUR/GBP</t>
+        </is>
+      </c>
+      <c r="C3674" t="n">
+        <v>0.84645</v>
+      </c>
+      <c r="D3674" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3674" t="inlineStr">
+        <is>
+          <t>2026-10-08 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3675">
+      <c r="A3675" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B3675" t="inlineStr">
+        <is>
+          <t>EUR/HKD</t>
+        </is>
+      </c>
+      <c r="C3675" t="n">
+        <v>8.7722</v>
+      </c>
+      <c r="D3675" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3675" t="inlineStr">
+        <is>
+          <t>2026-10-08 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3676">
+      <c r="A3676" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B3676" t="inlineStr">
+        <is>
+          <t>EUR/IDR</t>
+        </is>
+      </c>
+      <c r="C3676" t="n">
+        <v>19974.25</v>
+      </c>
+      <c r="D3676" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3676" t="inlineStr">
+        <is>
+          <t>2026-10-08 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3677">
+      <c r="A3677" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B3677" t="inlineStr">
+        <is>
+          <t>EUR/ILS</t>
+        </is>
+      </c>
+      <c r="C3677" t="n">
+        <v>3.429</v>
+      </c>
+      <c r="D3677" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3677" t="inlineStr">
+        <is>
+          <t>2026-10-08 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3678">
+      <c r="A3678" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B3678" t="inlineStr">
+        <is>
+          <t>EUR/JPY</t>
+        </is>
+      </c>
+      <c r="C3678" t="n">
+        <v>176.85</v>
+      </c>
+      <c r="D3678" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3678" t="inlineStr">
+        <is>
+          <t>2026-10-08 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3679">
+      <c r="A3679" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B3679" t="inlineStr">
+        <is>
+          <t>EUR/KRW</t>
+        </is>
+      </c>
+      <c r="C3679" t="n">
+        <v>1496.25</v>
+      </c>
+      <c r="D3679" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3679" t="inlineStr">
+        <is>
+          <t>2026-10-08 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3680">
+      <c r="A3680" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B3680" t="inlineStr">
+        <is>
+          <t>EUR/MAD</t>
+        </is>
+      </c>
+      <c r="C3680" t="n">
+        <v>11.215596</v>
+      </c>
+      <c r="D3680" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3680" t="inlineStr">
+        <is>
+          <t>2026-10-08 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3681">
+      <c r="A3681" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B3681" t="inlineStr">
+        <is>
+          <t>EUR/PEN</t>
+        </is>
+      </c>
+      <c r="C3681" t="n">
+        <v>3.868971</v>
+      </c>
+      <c r="D3681" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3681" t="inlineStr">
+        <is>
+          <t>2026-10-08 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3682">
+      <c r="A3682" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B3682" t="inlineStr">
+        <is>
+          <t>EUR/PHP</t>
+        </is>
+      </c>
+      <c r="C3682" t="n">
+        <v>70.203</v>
+      </c>
+      <c r="D3682" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3682" t="inlineStr">
+        <is>
+          <t>2026-10-08 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3683">
+      <c r="A3683" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B3683" t="inlineStr">
+        <is>
+          <t>EUR/RUB</t>
+        </is>
+      </c>
+      <c r="C3683" t="n">
+        <v>96.53019999999999</v>
+      </c>
+      <c r="D3683" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3683" t="inlineStr">
+        <is>
+          <t>2026-10-08 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3684">
+      <c r="A3684" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B3684" t="inlineStr">
+        <is>
+          <t>EUR/SAR</t>
+        </is>
+      </c>
+      <c r="C3684" t="n">
+        <v>4.219421</v>
+      </c>
+      <c r="D3684" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3684" t="inlineStr">
+        <is>
+          <t>2026-10-08 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3685">
+      <c r="A3685" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B3685" t="inlineStr">
+        <is>
+          <t>EUR/SEK</t>
+        </is>
+      </c>
+      <c r="C3685" t="n">
+        <v>11.224</v>
+      </c>
+      <c r="D3685" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3685" t="inlineStr">
+        <is>
+          <t>2026-10-08 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3686">
+      <c r="A3686" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B3686" t="inlineStr">
+        <is>
+          <t>EUR/SGD</t>
+        </is>
+      </c>
+      <c r="C3686" t="n">
+        <v>1.4311</v>
+      </c>
+      <c r="D3686" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3686" t="inlineStr">
+        <is>
+          <t>2026-10-08 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3687">
+      <c r="A3687" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B3687" t="inlineStr">
+        <is>
+          <t>EUR/THB</t>
+        </is>
+      </c>
+      <c r="C3687" t="n">
+        <v>37.661</v>
+      </c>
+      <c r="D3687" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3687" t="inlineStr">
+        <is>
+          <t>2026-10-08 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3688">
+      <c r="A3688" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B3688" t="inlineStr">
+        <is>
+          <t>EUR/TRY</t>
+        </is>
+      </c>
+      <c r="C3688" t="n">
+        <v>54.9822</v>
+      </c>
+      <c r="D3688" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3688" t="inlineStr">
+        <is>
+          <t>2026-10-08 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3689">
+      <c r="A3689" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B3689" t="inlineStr">
+        <is>
+          <t>EUR/USD</t>
+        </is>
+      </c>
+      <c r="C3689" t="n">
+        <v>1.1177</v>
+      </c>
+      <c r="D3689" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3689" t="inlineStr">
+        <is>
+          <t>2026-10-08 07:30 CET</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update currency rates for 2026-10-08
</commit_message>
<xml_diff>
--- a/data/rates.xlsx
+++ b/data/rates.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3689"/>
+  <dimension ref="A1:E3715"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -92643,6 +92643,656 @@
         </is>
       </c>
     </row>
+    <row r="3690">
+      <c r="A3690" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B3690" t="inlineStr">
+        <is>
+          <t>CNY/SGD</t>
+        </is>
+      </c>
+      <c r="C3690" t="n">
+        <v>0.191271</v>
+      </c>
+      <c r="D3690" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3690" t="inlineStr">
+        <is>
+          <t>2026-10-09 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3691">
+      <c r="A3691" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B3691" t="inlineStr">
+        <is>
+          <t>CNY/USD</t>
+        </is>
+      </c>
+      <c r="C3691" t="n">
+        <v>0.149202</v>
+      </c>
+      <c r="D3691" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3691" t="inlineStr">
+        <is>
+          <t>2026-10-09 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3692">
+      <c r="A3692" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B3692" t="inlineStr">
+        <is>
+          <t>EUR/AED</t>
+        </is>
+      </c>
+      <c r="C3692" t="n">
+        <v>4.112197</v>
+      </c>
+      <c r="D3692" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3692" t="inlineStr">
+        <is>
+          <t>2026-10-09 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3693">
+      <c r="A3693" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B3693" t="inlineStr">
+        <is>
+          <t>EUR/ARS</t>
+        </is>
+      </c>
+      <c r="C3693" t="n">
+        <v>1702.783981</v>
+      </c>
+      <c r="D3693" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3693" t="inlineStr">
+        <is>
+          <t>2026-10-09 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3694">
+      <c r="A3694" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B3694" t="inlineStr">
+        <is>
+          <t>EUR/BRL</t>
+        </is>
+      </c>
+      <c r="C3694" t="n">
+        <v>5.6118</v>
+      </c>
+      <c r="D3694" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3694" t="inlineStr">
+        <is>
+          <t>2026-10-09 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3695">
+      <c r="A3695" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B3695" t="inlineStr">
+        <is>
+          <t>EUR/CHF</t>
+        </is>
+      </c>
+      <c r="C3695" t="n">
+        <v>0.9326</v>
+      </c>
+      <c r="D3695" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3695" t="inlineStr">
+        <is>
+          <t>2026-10-09 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3696">
+      <c r="A3696" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B3696" t="inlineStr">
+        <is>
+          <t>EUR/CLP</t>
+        </is>
+      </c>
+      <c r="C3696" t="n">
+        <v>1091.048532</v>
+      </c>
+      <c r="D3696" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3696" t="inlineStr">
+        <is>
+          <t>2026-10-09 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3697">
+      <c r="A3697" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B3697" t="inlineStr">
+        <is>
+          <t>EUR/CNY</t>
+        </is>
+      </c>
+      <c r="C3697" t="n">
+        <v>7.4972</v>
+      </c>
+      <c r="D3697" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3697" t="inlineStr">
+        <is>
+          <t>2026-10-09 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3698">
+      <c r="A3698" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B3698" t="inlineStr">
+        <is>
+          <t>EUR/COP</t>
+        </is>
+      </c>
+      <c r="C3698" t="n">
+        <v>3630.734063</v>
+      </c>
+      <c r="D3698" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3698" t="inlineStr">
+        <is>
+          <t>2026-10-09 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3699">
+      <c r="A3699" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B3699" t="inlineStr">
+        <is>
+          <t>EUR/DKK</t>
+        </is>
+      </c>
+      <c r="C3699" t="n">
+        <v>7.4739</v>
+      </c>
+      <c r="D3699" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3699" t="inlineStr">
+        <is>
+          <t>2026-10-09 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3700">
+      <c r="A3700" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B3700" t="inlineStr">
+        <is>
+          <t>EUR/GBP</t>
+        </is>
+      </c>
+      <c r="C3700" t="n">
+        <v>0.84698</v>
+      </c>
+      <c r="D3700" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3700" t="inlineStr">
+        <is>
+          <t>2026-10-09 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3701">
+      <c r="A3701" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B3701" t="inlineStr">
+        <is>
+          <t>EUR/HKD</t>
+        </is>
+      </c>
+      <c r="C3701" t="n">
+        <v>8.7783</v>
+      </c>
+      <c r="D3701" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3701" t="inlineStr">
+        <is>
+          <t>2026-10-09 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3702">
+      <c r="A3702" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B3702" t="inlineStr">
+        <is>
+          <t>EUR/IDR</t>
+        </is>
+      </c>
+      <c r="C3702" t="n">
+        <v>20045.31</v>
+      </c>
+      <c r="D3702" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3702" t="inlineStr">
+        <is>
+          <t>2026-10-09 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3703">
+      <c r="A3703" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B3703" t="inlineStr">
+        <is>
+          <t>EUR/ILS</t>
+        </is>
+      </c>
+      <c r="C3703" t="n">
+        <v>3.4423</v>
+      </c>
+      <c r="D3703" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3703" t="inlineStr">
+        <is>
+          <t>2026-10-09 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3704">
+      <c r="A3704" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B3704" t="inlineStr">
+        <is>
+          <t>EUR/JPY</t>
+        </is>
+      </c>
+      <c r="C3704" t="n">
+        <v>177.05</v>
+      </c>
+      <c r="D3704" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3704" t="inlineStr">
+        <is>
+          <t>2026-10-09 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3705">
+      <c r="A3705" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B3705" t="inlineStr">
+        <is>
+          <t>EUR/KRW</t>
+        </is>
+      </c>
+      <c r="C3705" t="n">
+        <v>1502.79</v>
+      </c>
+      <c r="D3705" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3705" t="inlineStr">
+        <is>
+          <t>2026-10-09 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3706">
+      <c r="A3706" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B3706" t="inlineStr">
+        <is>
+          <t>EUR/MAD</t>
+        </is>
+      </c>
+      <c r="C3706" t="n">
+        <v>11.168629</v>
+      </c>
+      <c r="D3706" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3706" t="inlineStr">
+        <is>
+          <t>2026-10-09 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3707">
+      <c r="A3707" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B3707" t="inlineStr">
+        <is>
+          <t>EUR/PEN</t>
+        </is>
+      </c>
+      <c r="C3707" t="n">
+        <v>3.855958</v>
+      </c>
+      <c r="D3707" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3707" t="inlineStr">
+        <is>
+          <t>2026-10-09 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3708">
+      <c r="A3708" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B3708" t="inlineStr">
+        <is>
+          <t>EUR/PHP</t>
+        </is>
+      </c>
+      <c r="C3708" t="n">
+        <v>70.47499999999999</v>
+      </c>
+      <c r="D3708" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3708" t="inlineStr">
+        <is>
+          <t>2026-10-09 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3709">
+      <c r="A3709" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B3709" t="inlineStr">
+        <is>
+          <t>EUR/RUB</t>
+        </is>
+      </c>
+      <c r="C3709" t="n">
+        <v>95.763255</v>
+      </c>
+      <c r="D3709" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3709" t="inlineStr">
+        <is>
+          <t>2026-10-09 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3710">
+      <c r="A3710" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B3710" t="inlineStr">
+        <is>
+          <t>EUR/SAR</t>
+        </is>
+      </c>
+      <c r="C3710" t="n">
+        <v>4.198976</v>
+      </c>
+      <c r="D3710" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3710" t="inlineStr">
+        <is>
+          <t>2026-10-09 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3711">
+      <c r="A3711" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B3711" t="inlineStr">
+        <is>
+          <t>EUR/SEK</t>
+        </is>
+      </c>
+      <c r="C3711" t="n">
+        <v>11.194</v>
+      </c>
+      <c r="D3711" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3711" t="inlineStr">
+        <is>
+          <t>2026-10-09 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3712">
+      <c r="A3712" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B3712" t="inlineStr">
+        <is>
+          <t>EUR/SGD</t>
+        </is>
+      </c>
+      <c r="C3712" t="n">
+        <v>1.434</v>
+      </c>
+      <c r="D3712" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3712" t="inlineStr">
+        <is>
+          <t>2026-10-09 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3713">
+      <c r="A3713" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B3713" t="inlineStr">
+        <is>
+          <t>EUR/THB</t>
+        </is>
+      </c>
+      <c r="C3713" t="n">
+        <v>37.68</v>
+      </c>
+      <c r="D3713" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3713" t="inlineStr">
+        <is>
+          <t>2026-10-09 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3714">
+      <c r="A3714" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B3714" t="inlineStr">
+        <is>
+          <t>EUR/TRY</t>
+        </is>
+      </c>
+      <c r="C3714" t="n">
+        <v>55.0523</v>
+      </c>
+      <c r="D3714" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3714" t="inlineStr">
+        <is>
+          <t>2026-10-09 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3715">
+      <c r="A3715" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B3715" t="inlineStr">
+        <is>
+          <t>EUR/USD</t>
+        </is>
+      </c>
+      <c r="C3715" t="n">
+        <v>1.1186</v>
+      </c>
+      <c r="D3715" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3715" t="inlineStr">
+        <is>
+          <t>2026-10-09 07:30 CET</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update currency rates for 2026-10-09
</commit_message>
<xml_diff>
--- a/data/rates.xlsx
+++ b/data/rates.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3715"/>
+  <dimension ref="A1:E3741"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -93293,6 +93293,656 @@
         </is>
       </c>
     </row>
+    <row r="3716">
+      <c r="A3716" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B3716" t="inlineStr">
+        <is>
+          <t>CNY/SGD</t>
+        </is>
+      </c>
+      <c r="C3716" t="n">
+        <v>0.191327</v>
+      </c>
+      <c r="D3716" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3716" t="inlineStr">
+        <is>
+          <t>2026-10-09 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3717">
+      <c r="A3717" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B3717" t="inlineStr">
+        <is>
+          <t>CNY/USD</t>
+        </is>
+      </c>
+      <c r="C3717" t="n">
+        <v>0.149429</v>
+      </c>
+      <c r="D3717" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3717" t="inlineStr">
+        <is>
+          <t>2026-10-09 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3718">
+      <c r="A3718" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B3718" t="inlineStr">
+        <is>
+          <t>EUR/AED</t>
+        </is>
+      </c>
+      <c r="C3718" t="n">
+        <v>4.115995</v>
+      </c>
+      <c r="D3718" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3718" t="inlineStr">
+        <is>
+          <t>2026-10-09 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3719">
+      <c r="A3719" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B3719" t="inlineStr">
+        <is>
+          <t>EUR/ARS</t>
+        </is>
+      </c>
+      <c r="C3719" t="n">
+        <v>1701.804276</v>
+      </c>
+      <c r="D3719" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3719" t="inlineStr">
+        <is>
+          <t>2026-10-09 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3720">
+      <c r="A3720" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B3720" t="inlineStr">
+        <is>
+          <t>EUR/BRL</t>
+        </is>
+      </c>
+      <c r="C3720" t="n">
+        <v>5.6086</v>
+      </c>
+      <c r="D3720" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3720" t="inlineStr">
+        <is>
+          <t>2026-10-09 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3721">
+      <c r="A3721" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B3721" t="inlineStr">
+        <is>
+          <t>EUR/CHF</t>
+        </is>
+      </c>
+      <c r="C3721" t="n">
+        <v>0.9313</v>
+      </c>
+      <c r="D3721" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3721" t="inlineStr">
+        <is>
+          <t>2026-10-09 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3722">
+      <c r="A3722" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B3722" t="inlineStr">
+        <is>
+          <t>EUR/CLP</t>
+        </is>
+      </c>
+      <c r="C3722" t="n">
+        <v>1094.009208</v>
+      </c>
+      <c r="D3722" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3722" t="inlineStr">
+        <is>
+          <t>2026-10-09 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3723">
+      <c r="A3723" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B3723" t="inlineStr">
+        <is>
+          <t>EUR/CNY</t>
+        </is>
+      </c>
+      <c r="C3723" t="n">
+        <v>7.4992</v>
+      </c>
+      <c r="D3723" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3723" t="inlineStr">
+        <is>
+          <t>2026-10-09 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3724">
+      <c r="A3724" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B3724" t="inlineStr">
+        <is>
+          <t>EUR/COP</t>
+        </is>
+      </c>
+      <c r="C3724" t="n">
+        <v>3625.104297</v>
+      </c>
+      <c r="D3724" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3724" t="inlineStr">
+        <is>
+          <t>2026-10-09 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3725">
+      <c r="A3725" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B3725" t="inlineStr">
+        <is>
+          <t>EUR/DKK</t>
+        </is>
+      </c>
+      <c r="C3725" t="n">
+        <v>7.4751</v>
+      </c>
+      <c r="D3725" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3725" t="inlineStr">
+        <is>
+          <t>2026-10-09 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3726">
+      <c r="A3726" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B3726" t="inlineStr">
+        <is>
+          <t>EUR/GBP</t>
+        </is>
+      </c>
+      <c r="C3726" t="n">
+        <v>0.84763</v>
+      </c>
+      <c r="D3726" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3726" t="inlineStr">
+        <is>
+          <t>2026-10-09 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3727">
+      <c r="A3727" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B3727" t="inlineStr">
+        <is>
+          <t>EUR/HKD</t>
+        </is>
+      </c>
+      <c r="C3727" t="n">
+        <v>8.794</v>
+      </c>
+      <c r="D3727" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3727" t="inlineStr">
+        <is>
+          <t>2026-10-09 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3728">
+      <c r="A3728" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B3728" t="inlineStr">
+        <is>
+          <t>EUR/IDR</t>
+        </is>
+      </c>
+      <c r="C3728" t="n">
+        <v>20036.94</v>
+      </c>
+      <c r="D3728" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3728" t="inlineStr">
+        <is>
+          <t>2026-10-09 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3729">
+      <c r="A3729" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B3729" t="inlineStr">
+        <is>
+          <t>EUR/ILS</t>
+        </is>
+      </c>
+      <c r="C3729" t="n">
+        <v>3.426</v>
+      </c>
+      <c r="D3729" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3729" t="inlineStr">
+        <is>
+          <t>2026-10-09 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3730">
+      <c r="A3730" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B3730" t="inlineStr">
+        <is>
+          <t>EUR/JPY</t>
+        </is>
+      </c>
+      <c r="C3730" t="n">
+        <v>177.34</v>
+      </c>
+      <c r="D3730" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3730" t="inlineStr">
+        <is>
+          <t>2026-10-09 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3731">
+      <c r="A3731" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B3731" t="inlineStr">
+        <is>
+          <t>EUR/KRW</t>
+        </is>
+      </c>
+      <c r="C3731" t="n">
+        <v>1503.27</v>
+      </c>
+      <c r="D3731" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3731" t="inlineStr">
+        <is>
+          <t>2026-10-09 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3732">
+      <c r="A3732" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B3732" t="inlineStr">
+        <is>
+          <t>EUR/MAD</t>
+        </is>
+      </c>
+      <c r="C3732" t="n">
+        <v>11.122126</v>
+      </c>
+      <c r="D3732" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3732" t="inlineStr">
+        <is>
+          <t>2026-10-09 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3733">
+      <c r="A3733" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B3733" t="inlineStr">
+        <is>
+          <t>EUR/PEN</t>
+        </is>
+      </c>
+      <c r="C3733" t="n">
+        <v>3.852743</v>
+      </c>
+      <c r="D3733" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3733" t="inlineStr">
+        <is>
+          <t>2026-10-09 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3734">
+      <c r="A3734" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B3734" t="inlineStr">
+        <is>
+          <t>EUR/PHP</t>
+        </is>
+      </c>
+      <c r="C3734" t="n">
+        <v>70.39700000000001</v>
+      </c>
+      <c r="D3734" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3734" t="inlineStr">
+        <is>
+          <t>2026-10-09 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3735">
+      <c r="A3735" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B3735" t="inlineStr">
+        <is>
+          <t>EUR/RUB</t>
+        </is>
+      </c>
+      <c r="C3735" t="n">
+        <v>95.73107899999999</v>
+      </c>
+      <c r="D3735" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3735" t="inlineStr">
+        <is>
+          <t>2026-10-09 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3736">
+      <c r="A3736" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B3736" t="inlineStr">
+        <is>
+          <t>EUR/SAR</t>
+        </is>
+      </c>
+      <c r="C3736" t="n">
+        <v>4.202854</v>
+      </c>
+      <c r="D3736" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3736" t="inlineStr">
+        <is>
+          <t>2026-10-09 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3737">
+      <c r="A3737" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B3737" t="inlineStr">
+        <is>
+          <t>EUR/SEK</t>
+        </is>
+      </c>
+      <c r="C3737" t="n">
+        <v>11.1675</v>
+      </c>
+      <c r="D3737" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3737" t="inlineStr">
+        <is>
+          <t>2026-10-09 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3738">
+      <c r="A3738" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B3738" t="inlineStr">
+        <is>
+          <t>EUR/SGD</t>
+        </is>
+      </c>
+      <c r="C3738" t="n">
+        <v>1.4348</v>
+      </c>
+      <c r="D3738" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3738" t="inlineStr">
+        <is>
+          <t>2026-10-09 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3739">
+      <c r="A3739" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B3739" t="inlineStr">
+        <is>
+          <t>EUR/THB</t>
+        </is>
+      </c>
+      <c r="C3739" t="n">
+        <v>37.574</v>
+      </c>
+      <c r="D3739" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3739" t="inlineStr">
+        <is>
+          <t>2026-10-09 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3740">
+      <c r="A3740" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B3740" t="inlineStr">
+        <is>
+          <t>EUR/TRY</t>
+        </is>
+      </c>
+      <c r="C3740" t="n">
+        <v>55.1033</v>
+      </c>
+      <c r="D3740" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3740" t="inlineStr">
+        <is>
+          <t>2026-10-09 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3741">
+      <c r="A3741" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B3741" t="inlineStr">
+        <is>
+          <t>EUR/USD</t>
+        </is>
+      </c>
+      <c r="C3741" t="n">
+        <v>1.1206</v>
+      </c>
+      <c r="D3741" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3741" t="inlineStr">
+        <is>
+          <t>2026-10-09 07:30 CET</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update currency rates for 2026-10-12
</commit_message>
<xml_diff>
--- a/data/rates.xlsx
+++ b/data/rates.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3741"/>
+  <dimension ref="A1:E3767"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -93943,6 +93943,656 @@
         </is>
       </c>
     </row>
+    <row r="3742">
+      <c r="A3742" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B3742" t="inlineStr">
+        <is>
+          <t>CNY/SGD</t>
+        </is>
+      </c>
+      <c r="C3742" t="n">
+        <v>0.191282</v>
+      </c>
+      <c r="D3742" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3742" t="inlineStr">
+        <is>
+          <t>2026-10-13 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3743">
+      <c r="A3743" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B3743" t="inlineStr">
+        <is>
+          <t>CNY/USD</t>
+        </is>
+      </c>
+      <c r="C3743" t="n">
+        <v>0.149415</v>
+      </c>
+      <c r="D3743" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3743" t="inlineStr">
+        <is>
+          <t>2026-10-13 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3744">
+      <c r="A3744" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B3744" t="inlineStr">
+        <is>
+          <t>EUR/AED</t>
+        </is>
+      </c>
+      <c r="C3744" t="n">
+        <v>4.114252</v>
+      </c>
+      <c r="D3744" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3744" t="inlineStr">
+        <is>
+          <t>2026-10-13 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3745">
+      <c r="A3745" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B3745" t="inlineStr">
+        <is>
+          <t>EUR/ARS</t>
+        </is>
+      </c>
+      <c r="C3745" t="n">
+        <v>1698.215903</v>
+      </c>
+      <c r="D3745" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3745" t="inlineStr">
+        <is>
+          <t>2026-10-13 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3746">
+      <c r="A3746" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B3746" t="inlineStr">
+        <is>
+          <t>EUR/BRL</t>
+        </is>
+      </c>
+      <c r="C3746" t="n">
+        <v>5.5819</v>
+      </c>
+      <c r="D3746" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3746" t="inlineStr">
+        <is>
+          <t>2026-10-13 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3747">
+      <c r="A3747" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B3747" t="inlineStr">
+        <is>
+          <t>EUR/CHF</t>
+        </is>
+      </c>
+      <c r="C3747" t="n">
+        <v>0.9312</v>
+      </c>
+      <c r="D3747" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3747" t="inlineStr">
+        <is>
+          <t>2026-10-13 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3748">
+      <c r="A3748" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B3748" t="inlineStr">
+        <is>
+          <t>EUR/CLP</t>
+        </is>
+      </c>
+      <c r="C3748" t="n">
+        <v>1097.086572</v>
+      </c>
+      <c r="D3748" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3748" t="inlineStr">
+        <is>
+          <t>2026-10-13 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3749">
+      <c r="A3749" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B3749" t="inlineStr">
+        <is>
+          <t>EUR/CNY</t>
+        </is>
+      </c>
+      <c r="C3749" t="n">
+        <v>7.4832</v>
+      </c>
+      <c r="D3749" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3749" t="inlineStr">
+        <is>
+          <t>2026-10-13 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3750">
+      <c r="A3750" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B3750" t="inlineStr">
+        <is>
+          <t>EUR/COP</t>
+        </is>
+      </c>
+      <c r="C3750" t="n">
+        <v>3592.588649</v>
+      </c>
+      <c r="D3750" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3750" t="inlineStr">
+        <is>
+          <t>2026-10-13 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3751">
+      <c r="A3751" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B3751" t="inlineStr">
+        <is>
+          <t>EUR/DKK</t>
+        </is>
+      </c>
+      <c r="C3751" t="n">
+        <v>7.4748</v>
+      </c>
+      <c r="D3751" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3751" t="inlineStr">
+        <is>
+          <t>2026-10-13 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3752">
+      <c r="A3752" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B3752" t="inlineStr">
+        <is>
+          <t>EUR/GBP</t>
+        </is>
+      </c>
+      <c r="C3752" t="n">
+        <v>0.84478</v>
+      </c>
+      <c r="D3752" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3752" t="inlineStr">
+        <is>
+          <t>2026-10-13 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3753">
+      <c r="A3753" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B3753" t="inlineStr">
+        <is>
+          <t>EUR/HKD</t>
+        </is>
+      </c>
+      <c r="C3753" t="n">
+        <v>8.7743</v>
+      </c>
+      <c r="D3753" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3753" t="inlineStr">
+        <is>
+          <t>2026-10-13 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3754">
+      <c r="A3754" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B3754" t="inlineStr">
+        <is>
+          <t>EUR/IDR</t>
+        </is>
+      </c>
+      <c r="C3754" t="n">
+        <v>20036.18</v>
+      </c>
+      <c r="D3754" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3754" t="inlineStr">
+        <is>
+          <t>2026-10-13 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3755">
+      <c r="A3755" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B3755" t="inlineStr">
+        <is>
+          <t>EUR/ILS</t>
+        </is>
+      </c>
+      <c r="C3755" t="n">
+        <v>3.432</v>
+      </c>
+      <c r="D3755" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3755" t="inlineStr">
+        <is>
+          <t>2026-10-13 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3756">
+      <c r="A3756" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B3756" t="inlineStr">
+        <is>
+          <t>EUR/JPY</t>
+        </is>
+      </c>
+      <c r="C3756" t="n">
+        <v>177.33</v>
+      </c>
+      <c r="D3756" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3756" t="inlineStr">
+        <is>
+          <t>2026-10-13 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3757">
+      <c r="A3757" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B3757" t="inlineStr">
+        <is>
+          <t>EUR/KRW</t>
+        </is>
+      </c>
+      <c r="C3757" t="n">
+        <v>1490.53</v>
+      </c>
+      <c r="D3757" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3757" t="inlineStr">
+        <is>
+          <t>2026-10-13 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3758">
+      <c r="A3758" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B3758" t="inlineStr">
+        <is>
+          <t>EUR/MAD</t>
+        </is>
+      </c>
+      <c r="C3758" t="n">
+        <v>10.996951</v>
+      </c>
+      <c r="D3758" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3758" t="inlineStr">
+        <is>
+          <t>2026-10-13 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3759">
+      <c r="A3759" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B3759" t="inlineStr">
+        <is>
+          <t>EUR/PEN</t>
+        </is>
+      </c>
+      <c r="C3759" t="n">
+        <v>3.846819</v>
+      </c>
+      <c r="D3759" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3759" t="inlineStr">
+        <is>
+          <t>2026-10-13 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3760">
+      <c r="A3760" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B3760" t="inlineStr">
+        <is>
+          <t>EUR/PHP</t>
+        </is>
+      </c>
+      <c r="C3760" t="n">
+        <v>70.169</v>
+      </c>
+      <c r="D3760" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3760" t="inlineStr">
+        <is>
+          <t>2026-10-13 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3761">
+      <c r="A3761" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B3761" t="inlineStr">
+        <is>
+          <t>EUR/RUB</t>
+        </is>
+      </c>
+      <c r="C3761" t="n">
+        <v>95.26558300000001</v>
+      </c>
+      <c r="D3761" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3761" t="inlineStr">
+        <is>
+          <t>2026-10-13 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3762">
+      <c r="A3762" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B3762" t="inlineStr">
+        <is>
+          <t>EUR/SAR</t>
+        </is>
+      </c>
+      <c r="C3762" t="n">
+        <v>4.201074</v>
+      </c>
+      <c r="D3762" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3762" t="inlineStr">
+        <is>
+          <t>2026-10-13 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3763">
+      <c r="A3763" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B3763" t="inlineStr">
+        <is>
+          <t>EUR/SEK</t>
+        </is>
+      </c>
+      <c r="C3763" t="n">
+        <v>11.1965</v>
+      </c>
+      <c r="D3763" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3763" t="inlineStr">
+        <is>
+          <t>2026-10-13 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3764">
+      <c r="A3764" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B3764" t="inlineStr">
+        <is>
+          <t>EUR/SGD</t>
+        </is>
+      </c>
+      <c r="C3764" t="n">
+        <v>1.4314</v>
+      </c>
+      <c r="D3764" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3764" t="inlineStr">
+        <is>
+          <t>2026-10-13 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3765">
+      <c r="A3765" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B3765" t="inlineStr">
+        <is>
+          <t>EUR/THB</t>
+        </is>
+      </c>
+      <c r="C3765" t="n">
+        <v>37.585</v>
+      </c>
+      <c r="D3765" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3765" t="inlineStr">
+        <is>
+          <t>2026-10-13 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3766">
+      <c r="A3766" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B3766" t="inlineStr">
+        <is>
+          <t>EUR/TRY</t>
+        </is>
+      </c>
+      <c r="C3766" t="n">
+        <v>55.1635</v>
+      </c>
+      <c r="D3766" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3766" t="inlineStr">
+        <is>
+          <t>2026-10-13 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3767">
+      <c r="A3767" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B3767" t="inlineStr">
+        <is>
+          <t>EUR/USD</t>
+        </is>
+      </c>
+      <c r="C3767" t="n">
+        <v>1.1181</v>
+      </c>
+      <c r="D3767" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3767" t="inlineStr">
+        <is>
+          <t>2026-10-13 07:30 CET</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update currency rates for 2026-10-13
</commit_message>
<xml_diff>
--- a/data/rates.xlsx
+++ b/data/rates.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3767"/>
+  <dimension ref="A1:E3793"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -94593,6 +94593,656 @@
         </is>
       </c>
     </row>
+    <row r="3768">
+      <c r="A3768" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B3768" t="inlineStr">
+        <is>
+          <t>CNY/SGD</t>
+        </is>
+      </c>
+      <c r="C3768" t="n">
+        <v>0.1912</v>
+      </c>
+      <c r="D3768" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3768" t="inlineStr">
+        <is>
+          <t>2026-10-13 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3769">
+      <c r="A3769" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B3769" t="inlineStr">
+        <is>
+          <t>CNY/USD</t>
+        </is>
+      </c>
+      <c r="C3769" t="n">
+        <v>0.149392</v>
+      </c>
+      <c r="D3769" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3769" t="inlineStr">
+        <is>
+          <t>2026-10-13 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3770">
+      <c r="A3770" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B3770" t="inlineStr">
+        <is>
+          <t>EUR/AED</t>
+        </is>
+      </c>
+      <c r="C3770" t="n">
+        <v>4.102503</v>
+      </c>
+      <c r="D3770" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3770" t="inlineStr">
+        <is>
+          <t>2026-10-13 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3771">
+      <c r="A3771" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B3771" t="inlineStr">
+        <is>
+          <t>EUR/ARS</t>
+        </is>
+      </c>
+      <c r="C3771" t="n">
+        <v>1693.366275</v>
+      </c>
+      <c r="D3771" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3771" t="inlineStr">
+        <is>
+          <t>2026-10-13 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3772">
+      <c r="A3772" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B3772" t="inlineStr">
+        <is>
+          <t>EUR/BRL</t>
+        </is>
+      </c>
+      <c r="C3772" t="n">
+        <v>5.6125</v>
+      </c>
+      <c r="D3772" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3772" t="inlineStr">
+        <is>
+          <t>2026-10-13 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3773">
+      <c r="A3773" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B3773" t="inlineStr">
+        <is>
+          <t>EUR/CHF</t>
+        </is>
+      </c>
+      <c r="C3773" t="n">
+        <v>0.9312</v>
+      </c>
+      <c r="D3773" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3773" t="inlineStr">
+        <is>
+          <t>2026-10-13 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3774">
+      <c r="A3774" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B3774" t="inlineStr">
+        <is>
+          <t>EUR/CLP</t>
+        </is>
+      </c>
+      <c r="C3774" t="n">
+        <v>1093.521562</v>
+      </c>
+      <c r="D3774" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3774" t="inlineStr">
+        <is>
+          <t>2026-10-13 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3775">
+      <c r="A3775" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B3775" t="inlineStr">
+        <is>
+          <t>EUR/CNY</t>
+        </is>
+      </c>
+      <c r="C3775" t="n">
+        <v>7.489</v>
+      </c>
+      <c r="D3775" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3775" t="inlineStr">
+        <is>
+          <t>2026-10-13 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3776">
+      <c r="A3776" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B3776" t="inlineStr">
+        <is>
+          <t>EUR/COP</t>
+        </is>
+      </c>
+      <c r="C3776" t="n">
+        <v>3578.670508</v>
+      </c>
+      <c r="D3776" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3776" t="inlineStr">
+        <is>
+          <t>2026-10-13 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3777">
+      <c r="A3777" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B3777" t="inlineStr">
+        <is>
+          <t>EUR/DKK</t>
+        </is>
+      </c>
+      <c r="C3777" t="n">
+        <v>7.4753</v>
+      </c>
+      <c r="D3777" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3777" t="inlineStr">
+        <is>
+          <t>2026-10-13 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3778">
+      <c r="A3778" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B3778" t="inlineStr">
+        <is>
+          <t>EUR/GBP</t>
+        </is>
+      </c>
+      <c r="C3778" t="n">
+        <v>0.8446</v>
+      </c>
+      <c r="D3778" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3778" t="inlineStr">
+        <is>
+          <t>2026-10-13 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3779">
+      <c r="A3779" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B3779" t="inlineStr">
+        <is>
+          <t>EUR/HKD</t>
+        </is>
+      </c>
+      <c r="C3779" t="n">
+        <v>8.780200000000001</v>
+      </c>
+      <c r="D3779" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3779" t="inlineStr">
+        <is>
+          <t>2026-10-13 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3780">
+      <c r="A3780" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B3780" t="inlineStr">
+        <is>
+          <t>EUR/IDR</t>
+        </is>
+      </c>
+      <c r="C3780" t="n">
+        <v>20004.87</v>
+      </c>
+      <c r="D3780" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3780" t="inlineStr">
+        <is>
+          <t>2026-10-13 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3781">
+      <c r="A3781" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B3781" t="inlineStr">
+        <is>
+          <t>EUR/ILS</t>
+        </is>
+      </c>
+      <c r="C3781" t="n">
+        <v>3.4404</v>
+      </c>
+      <c r="D3781" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3781" t="inlineStr">
+        <is>
+          <t>2026-10-13 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3782">
+      <c r="A3782" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B3782" t="inlineStr">
+        <is>
+          <t>EUR/JPY</t>
+        </is>
+      </c>
+      <c r="C3782" t="n">
+        <v>176.91</v>
+      </c>
+      <c r="D3782" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3782" t="inlineStr">
+        <is>
+          <t>2026-10-13 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3783">
+      <c r="A3783" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B3783" t="inlineStr">
+        <is>
+          <t>EUR/KRW</t>
+        </is>
+      </c>
+      <c r="C3783" t="n">
+        <v>1500.81</v>
+      </c>
+      <c r="D3783" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3783" t="inlineStr">
+        <is>
+          <t>2026-10-13 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3784">
+      <c r="A3784" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B3784" t="inlineStr">
+        <is>
+          <t>EUR/MAD</t>
+        </is>
+      </c>
+      <c r="C3784" t="n">
+        <v>10.85672</v>
+      </c>
+      <c r="D3784" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3784" t="inlineStr">
+        <is>
+          <t>2026-10-13 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3785">
+      <c r="A3785" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B3785" t="inlineStr">
+        <is>
+          <t>EUR/PEN</t>
+        </is>
+      </c>
+      <c r="C3785" t="n">
+        <v>3.843892</v>
+      </c>
+      <c r="D3785" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3785" t="inlineStr">
+        <is>
+          <t>2026-10-13 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3786">
+      <c r="A3786" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B3786" t="inlineStr">
+        <is>
+          <t>EUR/PHP</t>
+        </is>
+      </c>
+      <c r="C3786" t="n">
+        <v>70.22499999999999</v>
+      </c>
+      <c r="D3786" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3786" t="inlineStr">
+        <is>
+          <t>2026-10-13 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3787">
+      <c r="A3787" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B3787" t="inlineStr">
+        <is>
+          <t>EUR/RUB</t>
+        </is>
+      </c>
+      <c r="C3787" t="n">
+        <v>93.867199</v>
+      </c>
+      <c r="D3787" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3787" t="inlineStr">
+        <is>
+          <t>2026-10-13 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3788">
+      <c r="A3788" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B3788" t="inlineStr">
+        <is>
+          <t>EUR/SAR</t>
+        </is>
+      </c>
+      <c r="C3788" t="n">
+        <v>4.189077</v>
+      </c>
+      <c r="D3788" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3788" t="inlineStr">
+        <is>
+          <t>2026-10-13 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3789">
+      <c r="A3789" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B3789" t="inlineStr">
+        <is>
+          <t>EUR/SEK</t>
+        </is>
+      </c>
+      <c r="C3789" t="n">
+        <v>11.1698</v>
+      </c>
+      <c r="D3789" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3789" t="inlineStr">
+        <is>
+          <t>2026-10-13 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3790">
+      <c r="A3790" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B3790" t="inlineStr">
+        <is>
+          <t>EUR/SGD</t>
+        </is>
+      </c>
+      <c r="C3790" t="n">
+        <v>1.4319</v>
+      </c>
+      <c r="D3790" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3790" t="inlineStr">
+        <is>
+          <t>2026-10-13 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3791">
+      <c r="A3791" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B3791" t="inlineStr">
+        <is>
+          <t>EUR/THB</t>
+        </is>
+      </c>
+      <c r="C3791" t="n">
+        <v>37.58</v>
+      </c>
+      <c r="D3791" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3791" t="inlineStr">
+        <is>
+          <t>2026-10-13 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3792">
+      <c r="A3792" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B3792" t="inlineStr">
+        <is>
+          <t>EUR/TRY</t>
+        </is>
+      </c>
+      <c r="C3792" t="n">
+        <v>55.2325</v>
+      </c>
+      <c r="D3792" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3792" t="inlineStr">
+        <is>
+          <t>2026-10-13 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3793">
+      <c r="A3793" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B3793" t="inlineStr">
+        <is>
+          <t>EUR/USD</t>
+        </is>
+      </c>
+      <c r="C3793" t="n">
+        <v>1.1188</v>
+      </c>
+      <c r="D3793" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3793" t="inlineStr">
+        <is>
+          <t>2026-10-13 07:30 CET</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update currency rates for 2026-10-14
</commit_message>
<xml_diff>
--- a/data/rates.xlsx
+++ b/data/rates.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3793"/>
+  <dimension ref="A1:E3819"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -95243,6 +95243,656 @@
         </is>
       </c>
     </row>
+    <row r="3794">
+      <c r="A3794" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B3794" t="inlineStr">
+        <is>
+          <t>CNY/SGD</t>
+        </is>
+      </c>
+      <c r="C3794" t="n">
+        <v>0.191645</v>
+      </c>
+      <c r="D3794" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3794" t="inlineStr">
+        <is>
+          <t>2026-10-14 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3795">
+      <c r="A3795" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B3795" t="inlineStr">
+        <is>
+          <t>CNY/USD</t>
+        </is>
+      </c>
+      <c r="C3795" t="n">
+        <v>0.149416</v>
+      </c>
+      <c r="D3795" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3795" t="inlineStr">
+        <is>
+          <t>2026-10-14 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3796">
+      <c r="A3796" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B3796" t="inlineStr">
+        <is>
+          <t>EUR/AED</t>
+        </is>
+      </c>
+      <c r="C3796" t="n">
+        <v>4.110604</v>
+      </c>
+      <c r="D3796" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3796" t="inlineStr">
+        <is>
+          <t>2026-10-14 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3797">
+      <c r="A3797" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B3797" t="inlineStr">
+        <is>
+          <t>EUR/ARS</t>
+        </is>
+      </c>
+      <c r="C3797" t="n">
+        <v>1696.685224</v>
+      </c>
+      <c r="D3797" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3797" t="inlineStr">
+        <is>
+          <t>2026-10-14 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3798">
+      <c r="A3798" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B3798" t="inlineStr">
+        <is>
+          <t>EUR/BRL</t>
+        </is>
+      </c>
+      <c r="C3798" t="n">
+        <v>5.6246</v>
+      </c>
+      <c r="D3798" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3798" t="inlineStr">
+        <is>
+          <t>2026-10-14 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3799">
+      <c r="A3799" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B3799" t="inlineStr">
+        <is>
+          <t>EUR/CHF</t>
+        </is>
+      </c>
+      <c r="C3799" t="n">
+        <v>0.9330000000000001</v>
+      </c>
+      <c r="D3799" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3799" t="inlineStr">
+        <is>
+          <t>2026-10-14 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3800">
+      <c r="A3800" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B3800" t="inlineStr">
+        <is>
+          <t>EUR/CLP</t>
+        </is>
+      </c>
+      <c r="C3800" t="n">
+        <v>1091.45477</v>
+      </c>
+      <c r="D3800" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3800" t="inlineStr">
+        <is>
+          <t>2026-10-14 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3801">
+      <c r="A3801" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B3801" t="inlineStr">
+        <is>
+          <t>EUR/CNY</t>
+        </is>
+      </c>
+      <c r="C3801" t="n">
+        <v>7.4925</v>
+      </c>
+      <c r="D3801" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3801" t="inlineStr">
+        <is>
+          <t>2026-10-14 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3802">
+      <c r="A3802" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B3802" t="inlineStr">
+        <is>
+          <t>EUR/COP</t>
+        </is>
+      </c>
+      <c r="C3802" t="n">
+        <v>3561.555737</v>
+      </c>
+      <c r="D3802" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3802" t="inlineStr">
+        <is>
+          <t>2026-10-14 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3803">
+      <c r="A3803" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B3803" t="inlineStr">
+        <is>
+          <t>EUR/DKK</t>
+        </is>
+      </c>
+      <c r="C3803" t="n">
+        <v>7.4754</v>
+      </c>
+      <c r="D3803" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3803" t="inlineStr">
+        <is>
+          <t>2026-10-14 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3804">
+      <c r="A3804" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B3804" t="inlineStr">
+        <is>
+          <t>EUR/GBP</t>
+        </is>
+      </c>
+      <c r="C3804" t="n">
+        <v>0.84385</v>
+      </c>
+      <c r="D3804" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3804" t="inlineStr">
+        <is>
+          <t>2026-10-14 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3805">
+      <c r="A3805" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B3805" t="inlineStr">
+        <is>
+          <t>EUR/HKD</t>
+        </is>
+      </c>
+      <c r="C3805" t="n">
+        <v>8.7859</v>
+      </c>
+      <c r="D3805" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3805" t="inlineStr">
+        <is>
+          <t>2026-10-14 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3806">
+      <c r="A3806" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B3806" t="inlineStr">
+        <is>
+          <t>EUR/IDR</t>
+        </is>
+      </c>
+      <c r="C3806" t="n">
+        <v>20062.67</v>
+      </c>
+      <c r="D3806" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3806" t="inlineStr">
+        <is>
+          <t>2026-10-14 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3807">
+      <c r="A3807" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B3807" t="inlineStr">
+        <is>
+          <t>EUR/ILS</t>
+        </is>
+      </c>
+      <c r="C3807" t="n">
+        <v>3.4443</v>
+      </c>
+      <c r="D3807" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3807" t="inlineStr">
+        <is>
+          <t>2026-10-14 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3808">
+      <c r="A3808" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B3808" t="inlineStr">
+        <is>
+          <t>EUR/JPY</t>
+        </is>
+      </c>
+      <c r="C3808" t="n">
+        <v>177.39</v>
+      </c>
+      <c r="D3808" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3808" t="inlineStr">
+        <is>
+          <t>2026-10-14 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3809">
+      <c r="A3809" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B3809" t="inlineStr">
+        <is>
+          <t>EUR/KRW</t>
+        </is>
+      </c>
+      <c r="C3809" t="n">
+        <v>1496.54</v>
+      </c>
+      <c r="D3809" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3809" t="inlineStr">
+        <is>
+          <t>2026-10-14 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3810">
+      <c r="A3810" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B3810" t="inlineStr">
+        <is>
+          <t>EUR/MAD</t>
+        </is>
+      </c>
+      <c r="C3810" t="n">
+        <v>10.936762</v>
+      </c>
+      <c r="D3810" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3810" t="inlineStr">
+        <is>
+          <t>2026-10-14 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3811">
+      <c r="A3811" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B3811" t="inlineStr">
+        <is>
+          <t>EUR/PEN</t>
+        </is>
+      </c>
+      <c r="C3811" t="n">
+        <v>3.849658</v>
+      </c>
+      <c r="D3811" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3811" t="inlineStr">
+        <is>
+          <t>2026-10-14 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3812">
+      <c r="A3812" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B3812" t="inlineStr">
+        <is>
+          <t>EUR/PHP</t>
+        </is>
+      </c>
+      <c r="C3812" t="n">
+        <v>70.393</v>
+      </c>
+      <c r="D3812" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3812" t="inlineStr">
+        <is>
+          <t>2026-10-14 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3813">
+      <c r="A3813" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B3813" t="inlineStr">
+        <is>
+          <t>EUR/RUB</t>
+        </is>
+      </c>
+      <c r="C3813" t="n">
+        <v>93.70523</v>
+      </c>
+      <c r="D3813" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3813" t="inlineStr">
+        <is>
+          <t>2026-10-14 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3814">
+      <c r="A3814" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B3814" t="inlineStr">
+        <is>
+          <t>EUR/SAR</t>
+        </is>
+      </c>
+      <c r="C3814" t="n">
+        <v>4.197349</v>
+      </c>
+      <c r="D3814" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3814" t="inlineStr">
+        <is>
+          <t>2026-10-14 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3815">
+      <c r="A3815" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B3815" t="inlineStr">
+        <is>
+          <t>EUR/SEK</t>
+        </is>
+      </c>
+      <c r="C3815" t="n">
+        <v>11.158</v>
+      </c>
+      <c r="D3815" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3815" t="inlineStr">
+        <is>
+          <t>2026-10-14 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3816">
+      <c r="A3816" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B3816" t="inlineStr">
+        <is>
+          <t>EUR/SGD</t>
+        </is>
+      </c>
+      <c r="C3816" t="n">
+        <v>1.4359</v>
+      </c>
+      <c r="D3816" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3816" t="inlineStr">
+        <is>
+          <t>2026-10-14 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3817">
+      <c r="A3817" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B3817" t="inlineStr">
+        <is>
+          <t>EUR/THB</t>
+        </is>
+      </c>
+      <c r="C3817" t="n">
+        <v>37.587</v>
+      </c>
+      <c r="D3817" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3817" t="inlineStr">
+        <is>
+          <t>2026-10-14 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3818">
+      <c r="A3818" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B3818" t="inlineStr">
+        <is>
+          <t>EUR/TRY</t>
+        </is>
+      </c>
+      <c r="C3818" t="n">
+        <v>55.2921</v>
+      </c>
+      <c r="D3818" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3818" t="inlineStr">
+        <is>
+          <t>2026-10-14 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3819">
+      <c r="A3819" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B3819" t="inlineStr">
+        <is>
+          <t>EUR/USD</t>
+        </is>
+      </c>
+      <c r="C3819" t="n">
+        <v>1.1195</v>
+      </c>
+      <c r="D3819" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3819" t="inlineStr">
+        <is>
+          <t>2026-10-14 07:30 CET</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update currency rates for 2026-10-15
</commit_message>
<xml_diff>
--- a/data/rates.xlsx
+++ b/data/rates.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3819"/>
+  <dimension ref="A1:E3845"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -95893,6 +95893,656 @@
         </is>
       </c>
     </row>
+    <row r="3820">
+      <c r="A3820" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B3820" t="inlineStr">
+        <is>
+          <t>CNY/SGD</t>
+        </is>
+      </c>
+      <c r="C3820" t="n">
+        <v>0.191738</v>
+      </c>
+      <c r="D3820" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3820" t="inlineStr">
+        <is>
+          <t>2026-10-15 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3821">
+      <c r="A3821" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B3821" t="inlineStr">
+        <is>
+          <t>CNY/USD</t>
+        </is>
+      </c>
+      <c r="C3821" t="n">
+        <v>0.149454</v>
+      </c>
+      <c r="D3821" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3821" t="inlineStr">
+        <is>
+          <t>2026-10-15 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3822">
+      <c r="A3822" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B3822" t="inlineStr">
+        <is>
+          <t>EUR/AED</t>
+        </is>
+      </c>
+      <c r="C3822" t="n">
+        <v>4.105759</v>
+      </c>
+      <c r="D3822" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3822" t="inlineStr">
+        <is>
+          <t>2026-10-15 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3823">
+      <c r="A3823" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B3823" t="inlineStr">
+        <is>
+          <t>EUR/ARS</t>
+        </is>
+      </c>
+      <c r="C3823" t="n">
+        <v>1693.244601</v>
+      </c>
+      <c r="D3823" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3823" t="inlineStr">
+        <is>
+          <t>2026-10-15 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3824">
+      <c r="A3824" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B3824" t="inlineStr">
+        <is>
+          <t>EUR/BRL</t>
+        </is>
+      </c>
+      <c r="C3824" t="n">
+        <v>5.6679</v>
+      </c>
+      <c r="D3824" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3824" t="inlineStr">
+        <is>
+          <t>2026-10-15 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3825">
+      <c r="A3825" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B3825" t="inlineStr">
+        <is>
+          <t>EUR/CHF</t>
+        </is>
+      </c>
+      <c r="C3825" t="n">
+        <v>0.9305</v>
+      </c>
+      <c r="D3825" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3825" t="inlineStr">
+        <is>
+          <t>2026-10-15 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3826">
+      <c r="A3826" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B3826" t="inlineStr">
+        <is>
+          <t>EUR/CLP</t>
+        </is>
+      </c>
+      <c r="C3826" t="n">
+        <v>1099.419986</v>
+      </c>
+      <c r="D3826" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3826" t="inlineStr">
+        <is>
+          <t>2026-10-15 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3827">
+      <c r="A3827" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B3827" t="inlineStr">
+        <is>
+          <t>EUR/CNY</t>
+        </is>
+      </c>
+      <c r="C3827" t="n">
+        <v>7.4993</v>
+      </c>
+      <c r="D3827" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3827" t="inlineStr">
+        <is>
+          <t>2026-10-15 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3828">
+      <c r="A3828" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B3828" t="inlineStr">
+        <is>
+          <t>EUR/COP</t>
+        </is>
+      </c>
+      <c r="C3828" t="n">
+        <v>3563.768771</v>
+      </c>
+      <c r="D3828" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3828" t="inlineStr">
+        <is>
+          <t>2026-10-15 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3829">
+      <c r="A3829" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B3829" t="inlineStr">
+        <is>
+          <t>EUR/DKK</t>
+        </is>
+      </c>
+      <c r="C3829" t="n">
+        <v>7.475</v>
+      </c>
+      <c r="D3829" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3829" t="inlineStr">
+        <is>
+          <t>2026-10-15 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3830">
+      <c r="A3830" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B3830" t="inlineStr">
+        <is>
+          <t>EUR/GBP</t>
+        </is>
+      </c>
+      <c r="C3830" t="n">
+        <v>0.8461</v>
+      </c>
+      <c r="D3830" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3830" t="inlineStr">
+        <is>
+          <t>2026-10-15 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3831">
+      <c r="A3831" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B3831" t="inlineStr">
+        <is>
+          <t>EUR/HKD</t>
+        </is>
+      </c>
+      <c r="C3831" t="n">
+        <v>8.795299999999999</v>
+      </c>
+      <c r="D3831" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3831" t="inlineStr">
+        <is>
+          <t>2026-10-15 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3832">
+      <c r="A3832" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B3832" t="inlineStr">
+        <is>
+          <t>EUR/IDR</t>
+        </is>
+      </c>
+      <c r="C3832" t="n">
+        <v>20112.25</v>
+      </c>
+      <c r="D3832" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3832" t="inlineStr">
+        <is>
+          <t>2026-10-15 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3833">
+      <c r="A3833" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B3833" t="inlineStr">
+        <is>
+          <t>EUR/ILS</t>
+        </is>
+      </c>
+      <c r="C3833" t="n">
+        <v>3.4769</v>
+      </c>
+      <c r="D3833" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3833" t="inlineStr">
+        <is>
+          <t>2026-10-15 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3834">
+      <c r="A3834" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B3834" t="inlineStr">
+        <is>
+          <t>EUR/JPY</t>
+        </is>
+      </c>
+      <c r="C3834" t="n">
+        <v>177.06</v>
+      </c>
+      <c r="D3834" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3834" t="inlineStr">
+        <is>
+          <t>2026-10-15 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3835">
+      <c r="A3835" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B3835" t="inlineStr">
+        <is>
+          <t>EUR/KRW</t>
+        </is>
+      </c>
+      <c r="C3835" t="n">
+        <v>1508.48</v>
+      </c>
+      <c r="D3835" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3835" t="inlineStr">
+        <is>
+          <t>2026-10-15 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3836">
+      <c r="A3836" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B3836" t="inlineStr">
+        <is>
+          <t>EUR/MAD</t>
+        </is>
+      </c>
+      <c r="C3836" t="n">
+        <v>10.998032</v>
+      </c>
+      <c r="D3836" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3836" t="inlineStr">
+        <is>
+          <t>2026-10-15 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3837">
+      <c r="A3837" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B3837" t="inlineStr">
+        <is>
+          <t>EUR/PEN</t>
+        </is>
+      </c>
+      <c r="C3837" t="n">
+        <v>3.837254</v>
+      </c>
+      <c r="D3837" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3837" t="inlineStr">
+        <is>
+          <t>2026-10-15 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3838">
+      <c r="A3838" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B3838" t="inlineStr">
+        <is>
+          <t>EUR/PHP</t>
+        </is>
+      </c>
+      <c r="C3838" t="n">
+        <v>70.693</v>
+      </c>
+      <c r="D3838" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3838" t="inlineStr">
+        <is>
+          <t>2026-10-15 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3839">
+      <c r="A3839" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B3839" t="inlineStr">
+        <is>
+          <t>EUR/RUB</t>
+        </is>
+      </c>
+      <c r="C3839" t="n">
+        <v>93.820031</v>
+      </c>
+      <c r="D3839" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3839" t="inlineStr">
+        <is>
+          <t>2026-10-15 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3840">
+      <c r="A3840" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B3840" t="inlineStr">
+        <is>
+          <t>EUR/SAR</t>
+        </is>
+      </c>
+      <c r="C3840" t="n">
+        <v>4.192402</v>
+      </c>
+      <c r="D3840" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3840" t="inlineStr">
+        <is>
+          <t>2026-10-15 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3841">
+      <c r="A3841" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B3841" t="inlineStr">
+        <is>
+          <t>EUR/SEK</t>
+        </is>
+      </c>
+      <c r="C3841" t="n">
+        <v>11.1765</v>
+      </c>
+      <c r="D3841" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3841" t="inlineStr">
+        <is>
+          <t>2026-10-15 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3842">
+      <c r="A3842" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B3842" t="inlineStr">
+        <is>
+          <t>EUR/SGD</t>
+        </is>
+      </c>
+      <c r="C3842" t="n">
+        <v>1.4379</v>
+      </c>
+      <c r="D3842" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3842" t="inlineStr">
+        <is>
+          <t>2026-10-15 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3843">
+      <c r="A3843" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B3843" t="inlineStr">
+        <is>
+          <t>EUR/THB</t>
+        </is>
+      </c>
+      <c r="C3843" t="n">
+        <v>37.592</v>
+      </c>
+      <c r="D3843" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3843" t="inlineStr">
+        <is>
+          <t>2026-10-15 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3844">
+      <c r="A3844" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B3844" t="inlineStr">
+        <is>
+          <t>EUR/TRY</t>
+        </is>
+      </c>
+      <c r="C3844" t="n">
+        <v>55.3873</v>
+      </c>
+      <c r="D3844" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3844" t="inlineStr">
+        <is>
+          <t>2026-10-15 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3845">
+      <c r="A3845" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B3845" t="inlineStr">
+        <is>
+          <t>EUR/USD</t>
+        </is>
+      </c>
+      <c r="C3845" t="n">
+        <v>1.1208</v>
+      </c>
+      <c r="D3845" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3845" t="inlineStr">
+        <is>
+          <t>2026-10-15 07:30 CET</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update currency rates for 2026-10-16
</commit_message>
<xml_diff>
--- a/data/rates.xlsx
+++ b/data/rates.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3845"/>
+  <dimension ref="A1:E3871"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -96543,6 +96543,656 @@
         </is>
       </c>
     </row>
+    <row r="3846">
+      <c r="A3846" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B3846" t="inlineStr">
+        <is>
+          <t>CNY/SGD</t>
+        </is>
+      </c>
+      <c r="C3846" t="n">
+        <v>0.191321</v>
+      </c>
+      <c r="D3846" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3846" t="inlineStr">
+        <is>
+          <t>2026-10-16 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3847">
+      <c r="A3847" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B3847" t="inlineStr">
+        <is>
+          <t>CNY/USD</t>
+        </is>
+      </c>
+      <c r="C3847" t="n">
+        <v>0.149561</v>
+      </c>
+      <c r="D3847" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3847" t="inlineStr">
+        <is>
+          <t>2026-10-16 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3848">
+      <c r="A3848" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B3848" t="inlineStr">
+        <is>
+          <t>EUR/AED</t>
+        </is>
+      </c>
+      <c r="C3848" t="n">
+        <v>4.118738</v>
+      </c>
+      <c r="D3848" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3848" t="inlineStr">
+        <is>
+          <t>2026-10-16 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3849">
+      <c r="A3849" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B3849" t="inlineStr">
+        <is>
+          <t>EUR/ARS</t>
+        </is>
+      </c>
+      <c r="C3849" t="n">
+        <v>1697.885281</v>
+      </c>
+      <c r="D3849" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3849" t="inlineStr">
+        <is>
+          <t>2026-10-16 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3850">
+      <c r="A3850" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B3850" t="inlineStr">
+        <is>
+          <t>EUR/BRL</t>
+        </is>
+      </c>
+      <c r="C3850" t="n">
+        <v>5.7197</v>
+      </c>
+      <c r="D3850" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3850" t="inlineStr">
+        <is>
+          <t>2026-10-16 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3851">
+      <c r="A3851" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B3851" t="inlineStr">
+        <is>
+          <t>EUR/CHF</t>
+        </is>
+      </c>
+      <c r="C3851" t="n">
+        <v>0.9272</v>
+      </c>
+      <c r="D3851" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3851" t="inlineStr">
+        <is>
+          <t>2026-10-16 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3852">
+      <c r="A3852" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B3852" t="inlineStr">
+        <is>
+          <t>EUR/CLP</t>
+        </is>
+      </c>
+      <c r="C3852" t="n">
+        <v>1105.122474</v>
+      </c>
+      <c r="D3852" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3852" t="inlineStr">
+        <is>
+          <t>2026-10-16 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3853">
+      <c r="A3853" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B3853" t="inlineStr">
+        <is>
+          <t>EUR/CNY</t>
+        </is>
+      </c>
+      <c r="C3853" t="n">
+        <v>7.524</v>
+      </c>
+      <c r="D3853" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3853" t="inlineStr">
+        <is>
+          <t>2026-10-16 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3854">
+      <c r="A3854" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B3854" t="inlineStr">
+        <is>
+          <t>EUR/COP</t>
+        </is>
+      </c>
+      <c r="C3854" t="n">
+        <v>3570.390226</v>
+      </c>
+      <c r="D3854" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3854" t="inlineStr">
+        <is>
+          <t>2026-10-16 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3855">
+      <c r="A3855" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B3855" t="inlineStr">
+        <is>
+          <t>EUR/DKK</t>
+        </is>
+      </c>
+      <c r="C3855" t="n">
+        <v>7.4748</v>
+      </c>
+      <c r="D3855" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3855" t="inlineStr">
+        <is>
+          <t>2026-10-16 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3856">
+      <c r="A3856" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B3856" t="inlineStr">
+        <is>
+          <t>EUR/GBP</t>
+        </is>
+      </c>
+      <c r="C3856" t="n">
+        <v>0.84385</v>
+      </c>
+      <c r="D3856" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3856" t="inlineStr">
+        <is>
+          <t>2026-10-16 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3857">
+      <c r="A3857" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B3857" t="inlineStr">
+        <is>
+          <t>EUR/HKD</t>
+        </is>
+      </c>
+      <c r="C3857" t="n">
+        <v>8.8316</v>
+      </c>
+      <c r="D3857" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3857" t="inlineStr">
+        <is>
+          <t>2026-10-16 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3858">
+      <c r="A3858" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B3858" t="inlineStr">
+        <is>
+          <t>EUR/IDR</t>
+        </is>
+      </c>
+      <c r="C3858" t="n">
+        <v>20290.28</v>
+      </c>
+      <c r="D3858" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3858" t="inlineStr">
+        <is>
+          <t>2026-10-16 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3859">
+      <c r="A3859" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B3859" t="inlineStr">
+        <is>
+          <t>EUR/ILS</t>
+        </is>
+      </c>
+      <c r="C3859" t="n">
+        <v>3.4822</v>
+      </c>
+      <c r="D3859" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3859" t="inlineStr">
+        <is>
+          <t>2026-10-16 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3860">
+      <c r="A3860" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B3860" t="inlineStr">
+        <is>
+          <t>EUR/JPY</t>
+        </is>
+      </c>
+      <c r="C3860" t="n">
+        <v>177.82</v>
+      </c>
+      <c r="D3860" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3860" t="inlineStr">
+        <is>
+          <t>2026-10-16 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3861">
+      <c r="A3861" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B3861" t="inlineStr">
+        <is>
+          <t>EUR/KRW</t>
+        </is>
+      </c>
+      <c r="C3861" t="n">
+        <v>1499.01</v>
+      </c>
+      <c r="D3861" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3861" t="inlineStr">
+        <is>
+          <t>2026-10-16 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3862">
+      <c r="A3862" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B3862" t="inlineStr">
+        <is>
+          <t>EUR/MAD</t>
+        </is>
+      </c>
+      <c r="C3862" t="n">
+        <v>10.972393</v>
+      </c>
+      <c r="D3862" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3862" t="inlineStr">
+        <is>
+          <t>2026-10-16 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3863">
+      <c r="A3863" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B3863" t="inlineStr">
+        <is>
+          <t>EUR/PEN</t>
+        </is>
+      </c>
+      <c r="C3863" t="n">
+        <v>3.849911</v>
+      </c>
+      <c r="D3863" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3863" t="inlineStr">
+        <is>
+          <t>2026-10-16 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3864">
+      <c r="A3864" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B3864" t="inlineStr">
+        <is>
+          <t>EUR/PHP</t>
+        </is>
+      </c>
+      <c r="C3864" t="n">
+        <v>70.858</v>
+      </c>
+      <c r="D3864" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3864" t="inlineStr">
+        <is>
+          <t>2026-10-16 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3865">
+      <c r="A3865" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B3865" t="inlineStr">
+        <is>
+          <t>EUR/RUB</t>
+        </is>
+      </c>
+      <c r="C3865" t="n">
+        <v>94.01792</v>
+      </c>
+      <c r="D3865" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3865" t="inlineStr">
+        <is>
+          <t>2026-10-16 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3866">
+      <c r="A3866" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B3866" t="inlineStr">
+        <is>
+          <t>EUR/SAR</t>
+        </is>
+      </c>
+      <c r="C3866" t="n">
+        <v>4.205654</v>
+      </c>
+      <c r="D3866" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3866" t="inlineStr">
+        <is>
+          <t>2026-10-16 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3867">
+      <c r="A3867" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B3867" t="inlineStr">
+        <is>
+          <t>EUR/SEK</t>
+        </is>
+      </c>
+      <c r="C3867" t="n">
+        <v>11.145</v>
+      </c>
+      <c r="D3867" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3867" t="inlineStr">
+        <is>
+          <t>2026-10-16 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3868">
+      <c r="A3868" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B3868" t="inlineStr">
+        <is>
+          <t>EUR/SGD</t>
+        </is>
+      </c>
+      <c r="C3868" t="n">
+        <v>1.4395</v>
+      </c>
+      <c r="D3868" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3868" t="inlineStr">
+        <is>
+          <t>2026-10-16 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3869">
+      <c r="A3869" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B3869" t="inlineStr">
+        <is>
+          <t>EUR/THB</t>
+        </is>
+      </c>
+      <c r="C3869" t="n">
+        <v>37.602</v>
+      </c>
+      <c r="D3869" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3869" t="inlineStr">
+        <is>
+          <t>2026-10-16 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3870">
+      <c r="A3870" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B3870" t="inlineStr">
+        <is>
+          <t>EUR/TRY</t>
+        </is>
+      </c>
+      <c r="C3870" t="n">
+        <v>55.7328</v>
+      </c>
+      <c r="D3870" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3870" t="inlineStr">
+        <is>
+          <t>2026-10-16 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3871">
+      <c r="A3871" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B3871" t="inlineStr">
+        <is>
+          <t>EUR/USD</t>
+        </is>
+      </c>
+      <c r="C3871" t="n">
+        <v>1.1253</v>
+      </c>
+      <c r="D3871" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3871" t="inlineStr">
+        <is>
+          <t>2026-10-16 07:30 CET</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update currency rates for 2026-10-19
</commit_message>
<xml_diff>
--- a/data/rates.xlsx
+++ b/data/rates.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3871"/>
+  <dimension ref="A1:E3897"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -97193,6 +97193,656 @@
         </is>
       </c>
     </row>
+    <row r="3872">
+      <c r="A3872" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B3872" t="inlineStr">
+        <is>
+          <t>CNY/SGD</t>
+        </is>
+      </c>
+      <c r="C3872" t="n">
+        <v>0.19145</v>
+      </c>
+      <c r="D3872" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3872" t="inlineStr">
+        <is>
+          <t>2026-10-19 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3873">
+      <c r="A3873" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B3873" t="inlineStr">
+        <is>
+          <t>CNY/USD</t>
+        </is>
+      </c>
+      <c r="C3873" t="n">
+        <v>0.149685</v>
+      </c>
+      <c r="D3873" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3873" t="inlineStr">
+        <is>
+          <t>2026-10-19 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3874">
+      <c r="A3874" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B3874" t="inlineStr">
+        <is>
+          <t>EUR/AED</t>
+        </is>
+      </c>
+      <c r="C3874" t="n">
+        <v>4.122418</v>
+      </c>
+      <c r="D3874" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3874" t="inlineStr">
+        <is>
+          <t>2026-10-19 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3875">
+      <c r="A3875" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B3875" t="inlineStr">
+        <is>
+          <t>EUR/ARS</t>
+        </is>
+      </c>
+      <c r="C3875" t="n">
+        <v>1700.11481</v>
+      </c>
+      <c r="D3875" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3875" t="inlineStr">
+        <is>
+          <t>2026-10-19 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3876">
+      <c r="A3876" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B3876" t="inlineStr">
+        <is>
+          <t>EUR/BRL</t>
+        </is>
+      </c>
+      <c r="C3876" t="n">
+        <v>5.6633</v>
+      </c>
+      <c r="D3876" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3876" t="inlineStr">
+        <is>
+          <t>2026-10-19 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3877">
+      <c r="A3877" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B3877" t="inlineStr">
+        <is>
+          <t>EUR/CHF</t>
+        </is>
+      </c>
+      <c r="C3877" t="n">
+        <v>0.9261</v>
+      </c>
+      <c r="D3877" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3877" t="inlineStr">
+        <is>
+          <t>2026-10-19 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3878">
+      <c r="A3878" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B3878" t="inlineStr">
+        <is>
+          <t>EUR/CLP</t>
+        </is>
+      </c>
+      <c r="C3878" t="n">
+        <v>1104.15988</v>
+      </c>
+      <c r="D3878" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3878" t="inlineStr">
+        <is>
+          <t>2026-10-19 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3879">
+      <c r="A3879" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B3879" t="inlineStr">
+        <is>
+          <t>EUR/CNY</t>
+        </is>
+      </c>
+      <c r="C3879" t="n">
+        <v>7.4991</v>
+      </c>
+      <c r="D3879" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3879" t="inlineStr">
+        <is>
+          <t>2026-10-19 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3880">
+      <c r="A3880" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B3880" t="inlineStr">
+        <is>
+          <t>EUR/COP</t>
+        </is>
+      </c>
+      <c r="C3880" t="n">
+        <v>3570.384787</v>
+      </c>
+      <c r="D3880" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3880" t="inlineStr">
+        <is>
+          <t>2026-10-19 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3881">
+      <c r="A3881" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B3881" t="inlineStr">
+        <is>
+          <t>EUR/DKK</t>
+        </is>
+      </c>
+      <c r="C3881" t="n">
+        <v>7.4747</v>
+      </c>
+      <c r="D3881" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3881" t="inlineStr">
+        <is>
+          <t>2026-10-19 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3882">
+      <c r="A3882" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B3882" t="inlineStr">
+        <is>
+          <t>EUR/GBP</t>
+        </is>
+      </c>
+      <c r="C3882" t="n">
+        <v>0.84205</v>
+      </c>
+      <c r="D3882" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3882" t="inlineStr">
+        <is>
+          <t>2026-10-19 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3883">
+      <c r="A3883" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B3883" t="inlineStr">
+        <is>
+          <t>EUR/HKD</t>
+        </is>
+      </c>
+      <c r="C3883" t="n">
+        <v>8.809699999999999</v>
+      </c>
+      <c r="D3883" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3883" t="inlineStr">
+        <is>
+          <t>2026-10-19 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3884">
+      <c r="A3884" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B3884" t="inlineStr">
+        <is>
+          <t>EUR/IDR</t>
+        </is>
+      </c>
+      <c r="C3884" t="n">
+        <v>20253.16</v>
+      </c>
+      <c r="D3884" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3884" t="inlineStr">
+        <is>
+          <t>2026-10-19 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3885">
+      <c r="A3885" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B3885" t="inlineStr">
+        <is>
+          <t>EUR/ILS</t>
+        </is>
+      </c>
+      <c r="C3885" t="n">
+        <v>3.489</v>
+      </c>
+      <c r="D3885" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3885" t="inlineStr">
+        <is>
+          <t>2026-10-19 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3886">
+      <c r="A3886" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B3886" t="inlineStr">
+        <is>
+          <t>EUR/JPY</t>
+        </is>
+      </c>
+      <c r="C3886" t="n">
+        <v>177.63</v>
+      </c>
+      <c r="D3886" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3886" t="inlineStr">
+        <is>
+          <t>2026-10-19 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3887">
+      <c r="A3887" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B3887" t="inlineStr">
+        <is>
+          <t>EUR/KRW</t>
+        </is>
+      </c>
+      <c r="C3887" t="n">
+        <v>1492.35</v>
+      </c>
+      <c r="D3887" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3887" t="inlineStr">
+        <is>
+          <t>2026-10-19 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3888">
+      <c r="A3888" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B3888" t="inlineStr">
+        <is>
+          <t>EUR/MAD</t>
+        </is>
+      </c>
+      <c r="C3888" t="n">
+        <v>10.939609</v>
+      </c>
+      <c r="D3888" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3888" t="inlineStr">
+        <is>
+          <t>2026-10-19 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3889">
+      <c r="A3889" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B3889" t="inlineStr">
+        <is>
+          <t>EUR/PEN</t>
+        </is>
+      </c>
+      <c r="C3889" t="n">
+        <v>3.864523</v>
+      </c>
+      <c r="D3889" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3889" t="inlineStr">
+        <is>
+          <t>2026-10-19 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3890">
+      <c r="A3890" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B3890" t="inlineStr">
+        <is>
+          <t>EUR/PHP</t>
+        </is>
+      </c>
+      <c r="C3890" t="n">
+        <v>70.715</v>
+      </c>
+      <c r="D3890" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3890" t="inlineStr">
+        <is>
+          <t>2026-10-19 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3891">
+      <c r="A3891" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B3891" t="inlineStr">
+        <is>
+          <t>EUR/RUB</t>
+        </is>
+      </c>
+      <c r="C3891" t="n">
+        <v>93.876993</v>
+      </c>
+      <c r="D3891" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3891" t="inlineStr">
+        <is>
+          <t>2026-10-19 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3892">
+      <c r="A3892" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B3892" t="inlineStr">
+        <is>
+          <t>EUR/SAR</t>
+        </is>
+      </c>
+      <c r="C3892" t="n">
+        <v>4.209412</v>
+      </c>
+      <c r="D3892" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3892" t="inlineStr">
+        <is>
+          <t>2026-10-19 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3893">
+      <c r="A3893" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B3893" t="inlineStr">
+        <is>
+          <t>EUR/SEK</t>
+        </is>
+      </c>
+      <c r="C3893" t="n">
+        <v>11.104</v>
+      </c>
+      <c r="D3893" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3893" t="inlineStr">
+        <is>
+          <t>2026-10-19 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3894">
+      <c r="A3894" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B3894" t="inlineStr">
+        <is>
+          <t>EUR/SGD</t>
+        </is>
+      </c>
+      <c r="C3894" t="n">
+        <v>1.4357</v>
+      </c>
+      <c r="D3894" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3894" t="inlineStr">
+        <is>
+          <t>2026-10-19 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3895">
+      <c r="A3895" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B3895" t="inlineStr">
+        <is>
+          <t>EUR/THB</t>
+        </is>
+      </c>
+      <c r="C3895" t="n">
+        <v>37.665</v>
+      </c>
+      <c r="D3895" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3895" t="inlineStr">
+        <is>
+          <t>2026-10-19 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3896">
+      <c r="A3896" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B3896" t="inlineStr">
+        <is>
+          <t>EUR/TRY</t>
+        </is>
+      </c>
+      <c r="C3896" t="n">
+        <v>55.6227</v>
+      </c>
+      <c r="D3896" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3896" t="inlineStr">
+        <is>
+          <t>2026-10-19 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3897">
+      <c r="A3897" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B3897" t="inlineStr">
+        <is>
+          <t>EUR/USD</t>
+        </is>
+      </c>
+      <c r="C3897" t="n">
+        <v>1.1225</v>
+      </c>
+      <c r="D3897" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3897" t="inlineStr">
+        <is>
+          <t>2026-10-19 07:30 CET</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update currency rates for 2026-10-20
</commit_message>
<xml_diff>
--- a/data/rates.xlsx
+++ b/data/rates.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3897"/>
+  <dimension ref="A1:E3923"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -97843,6 +97843,656 @@
         </is>
       </c>
     </row>
+    <row r="3898">
+      <c r="A3898" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B3898" t="inlineStr">
+        <is>
+          <t>CNY/SGD</t>
+        </is>
+      </c>
+      <c r="C3898" t="n">
+        <v>0.191444</v>
+      </c>
+      <c r="D3898" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3898" t="inlineStr">
+        <is>
+          <t>2026-10-20 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3899">
+      <c r="A3899" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B3899" t="inlineStr">
+        <is>
+          <t>CNY/USD</t>
+        </is>
+      </c>
+      <c r="C3899" t="n">
+        <v>0.149745</v>
+      </c>
+      <c r="D3899" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3899" t="inlineStr">
+        <is>
+          <t>2026-10-20 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3900">
+      <c r="A3900" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B3900" t="inlineStr">
+        <is>
+          <t>EUR/AED</t>
+        </is>
+      </c>
+      <c r="C3900" t="n">
+        <v>4.119603</v>
+      </c>
+      <c r="D3900" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3900" t="inlineStr">
+        <is>
+          <t>2026-10-20 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3901">
+      <c r="A3901" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B3901" t="inlineStr">
+        <is>
+          <t>EUR/ARS</t>
+        </is>
+      </c>
+      <c r="C3901" t="n">
+        <v>1708.804296</v>
+      </c>
+      <c r="D3901" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3901" t="inlineStr">
+        <is>
+          <t>2026-10-20 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3902">
+      <c r="A3902" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B3902" t="inlineStr">
+        <is>
+          <t>EUR/BRL</t>
+        </is>
+      </c>
+      <c r="C3902" t="n">
+        <v>5.6339</v>
+      </c>
+      <c r="D3902" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3902" t="inlineStr">
+        <is>
+          <t>2026-10-20 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3903">
+      <c r="A3903" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B3903" t="inlineStr">
+        <is>
+          <t>EUR/CHF</t>
+        </is>
+      </c>
+      <c r="C3903" t="n">
+        <v>0.9237</v>
+      </c>
+      <c r="D3903" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3903" t="inlineStr">
+        <is>
+          <t>2026-10-20 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3904">
+      <c r="A3904" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B3904" t="inlineStr">
+        <is>
+          <t>EUR/CLP</t>
+        </is>
+      </c>
+      <c r="C3904" t="n">
+        <v>1102.699854</v>
+      </c>
+      <c r="D3904" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3904" t="inlineStr">
+        <is>
+          <t>2026-10-20 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3905">
+      <c r="A3905" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B3905" t="inlineStr">
+        <is>
+          <t>EUR/CNY</t>
+        </is>
+      </c>
+      <c r="C3905" t="n">
+        <v>7.4894</v>
+      </c>
+      <c r="D3905" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3905" t="inlineStr">
+        <is>
+          <t>2026-10-20 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3906">
+      <c r="A3906" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B3906" t="inlineStr">
+        <is>
+          <t>EUR/COP</t>
+        </is>
+      </c>
+      <c r="C3906" t="n">
+        <v>3563.59579</v>
+      </c>
+      <c r="D3906" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3906" t="inlineStr">
+        <is>
+          <t>2026-10-20 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3907">
+      <c r="A3907" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B3907" t="inlineStr">
+        <is>
+          <t>EUR/DKK</t>
+        </is>
+      </c>
+      <c r="C3907" t="n">
+        <v>7.4746</v>
+      </c>
+      <c r="D3907" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3907" t="inlineStr">
+        <is>
+          <t>2026-10-20 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3908">
+      <c r="A3908" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B3908" t="inlineStr">
+        <is>
+          <t>EUR/GBP</t>
+        </is>
+      </c>
+      <c r="C3908" t="n">
+        <v>0.84028</v>
+      </c>
+      <c r="D3908" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3908" t="inlineStr">
+        <is>
+          <t>2026-10-20 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3909">
+      <c r="A3909" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B3909" t="inlineStr">
+        <is>
+          <t>EUR/HKD</t>
+        </is>
+      </c>
+      <c r="C3909" t="n">
+        <v>8.802300000000001</v>
+      </c>
+      <c r="D3909" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3909" t="inlineStr">
+        <is>
+          <t>2026-10-20 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3910">
+      <c r="A3910" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B3910" t="inlineStr">
+        <is>
+          <t>EUR/IDR</t>
+        </is>
+      </c>
+      <c r="C3910" t="n">
+        <v>20170.57</v>
+      </c>
+      <c r="D3910" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3910" t="inlineStr">
+        <is>
+          <t>2026-10-20 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3911">
+      <c r="A3911" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B3911" t="inlineStr">
+        <is>
+          <t>EUR/ILS</t>
+        </is>
+      </c>
+      <c r="C3911" t="n">
+        <v>3.4853</v>
+      </c>
+      <c r="D3911" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3911" t="inlineStr">
+        <is>
+          <t>2026-10-20 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3912">
+      <c r="A3912" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B3912" t="inlineStr">
+        <is>
+          <t>EUR/JPY</t>
+        </is>
+      </c>
+      <c r="C3912" t="n">
+        <v>177.34</v>
+      </c>
+      <c r="D3912" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3912" t="inlineStr">
+        <is>
+          <t>2026-10-20 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3913">
+      <c r="A3913" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B3913" t="inlineStr">
+        <is>
+          <t>EUR/KRW</t>
+        </is>
+      </c>
+      <c r="C3913" t="n">
+        <v>1489.17</v>
+      </c>
+      <c r="D3913" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3913" t="inlineStr">
+        <is>
+          <t>2026-10-20 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3914">
+      <c r="A3914" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B3914" t="inlineStr">
+        <is>
+          <t>EUR/MAD</t>
+        </is>
+      </c>
+      <c r="C3914" t="n">
+        <v>10.97921</v>
+      </c>
+      <c r="D3914" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3914" t="inlineStr">
+        <is>
+          <t>2026-10-20 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3915">
+      <c r="A3915" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B3915" t="inlineStr">
+        <is>
+          <t>EUR/PEN</t>
+        </is>
+      </c>
+      <c r="C3915" t="n">
+        <v>3.861736</v>
+      </c>
+      <c r="D3915" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3915" t="inlineStr">
+        <is>
+          <t>2026-10-20 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3916">
+      <c r="A3916" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B3916" t="inlineStr">
+        <is>
+          <t>EUR/PHP</t>
+        </is>
+      </c>
+      <c r="C3916" t="n">
+        <v>70.804</v>
+      </c>
+      <c r="D3916" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3916" t="inlineStr">
+        <is>
+          <t>2026-10-20 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3917">
+      <c r="A3917" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B3917" t="inlineStr">
+        <is>
+          <t>EUR/RUB</t>
+        </is>
+      </c>
+      <c r="C3917" t="n">
+        <v>92.86007499999999</v>
+      </c>
+      <c r="D3917" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3917" t="inlineStr">
+        <is>
+          <t>2026-10-20 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3918">
+      <c r="A3918" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B3918" t="inlineStr">
+        <is>
+          <t>EUR/SAR</t>
+        </is>
+      </c>
+      <c r="C3918" t="n">
+        <v>4.206538</v>
+      </c>
+      <c r="D3918" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3918" t="inlineStr">
+        <is>
+          <t>2026-10-20 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3919">
+      <c r="A3919" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B3919" t="inlineStr">
+        <is>
+          <t>EUR/SEK</t>
+        </is>
+      </c>
+      <c r="C3919" t="n">
+        <v>11.123</v>
+      </c>
+      <c r="D3919" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3919" t="inlineStr">
+        <is>
+          <t>2026-10-20 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3920">
+      <c r="A3920" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B3920" t="inlineStr">
+        <is>
+          <t>EUR/SGD</t>
+        </is>
+      </c>
+      <c r="C3920" t="n">
+        <v>1.4338</v>
+      </c>
+      <c r="D3920" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3920" t="inlineStr">
+        <is>
+          <t>2026-10-20 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3921">
+      <c r="A3921" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B3921" t="inlineStr">
+        <is>
+          <t>EUR/THB</t>
+        </is>
+      </c>
+      <c r="C3921" t="n">
+        <v>37.738</v>
+      </c>
+      <c r="D3921" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3921" t="inlineStr">
+        <is>
+          <t>2026-10-20 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3922">
+      <c r="A3922" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B3922" t="inlineStr">
+        <is>
+          <t>EUR/TRY</t>
+        </is>
+      </c>
+      <c r="C3922" t="n">
+        <v>55.6009</v>
+      </c>
+      <c r="D3922" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3922" t="inlineStr">
+        <is>
+          <t>2026-10-20 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3923">
+      <c r="A3923" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B3923" t="inlineStr">
+        <is>
+          <t>EUR/USD</t>
+        </is>
+      </c>
+      <c r="C3923" t="n">
+        <v>1.1215</v>
+      </c>
+      <c r="D3923" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3923" t="inlineStr">
+        <is>
+          <t>2026-10-20 07:30 CET</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update currency rates for 2026-10-21
</commit_message>
<xml_diff>
--- a/data/rates.xlsx
+++ b/data/rates.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3923"/>
+  <dimension ref="A1:E3949"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -98493,6 +98493,656 @@
         </is>
       </c>
     </row>
+    <row r="3924">
+      <c r="A3924" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B3924" t="inlineStr">
+        <is>
+          <t>CNY/SGD</t>
+        </is>
+      </c>
+      <c r="C3924" t="n">
+        <v>0.191309</v>
+      </c>
+      <c r="D3924" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3924" t="inlineStr">
+        <is>
+          <t>2026-10-21 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3925">
+      <c r="A3925" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B3925" t="inlineStr">
+        <is>
+          <t>CNY/USD</t>
+        </is>
+      </c>
+      <c r="C3925" t="n">
+        <v>0.149789</v>
+      </c>
+      <c r="D3925" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3925" t="inlineStr">
+        <is>
+          <t>2026-10-21 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3926">
+      <c r="A3926" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B3926" t="inlineStr">
+        <is>
+          <t>EUR/AED</t>
+        </is>
+      </c>
+      <c r="C3926" t="n">
+        <v>4.123061</v>
+      </c>
+      <c r="D3926" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3926" t="inlineStr">
+        <is>
+          <t>2026-10-21 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3927">
+      <c r="A3927" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B3927" t="inlineStr">
+        <is>
+          <t>EUR/ARS</t>
+        </is>
+      </c>
+      <c r="C3927" t="n">
+        <v>1711.915115</v>
+      </c>
+      <c r="D3927" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3927" t="inlineStr">
+        <is>
+          <t>2026-10-21 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3928">
+      <c r="A3928" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B3928" t="inlineStr">
+        <is>
+          <t>EUR/BRL</t>
+        </is>
+      </c>
+      <c r="C3928" t="n">
+        <v>5.6432</v>
+      </c>
+      <c r="D3928" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3928" t="inlineStr">
+        <is>
+          <t>2026-10-21 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3929">
+      <c r="A3929" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B3929" t="inlineStr">
+        <is>
+          <t>EUR/CHF</t>
+        </is>
+      </c>
+      <c r="C3929" t="n">
+        <v>0.9256</v>
+      </c>
+      <c r="D3929" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3929" t="inlineStr">
+        <is>
+          <t>2026-10-21 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3930">
+      <c r="A3930" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B3930" t="inlineStr">
+        <is>
+          <t>EUR/CLP</t>
+        </is>
+      </c>
+      <c r="C3930" t="n">
+        <v>1101.066353</v>
+      </c>
+      <c r="D3930" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3930" t="inlineStr">
+        <is>
+          <t>2026-10-21 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3931">
+      <c r="A3931" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B3931" t="inlineStr">
+        <is>
+          <t>EUR/CNY</t>
+        </is>
+      </c>
+      <c r="C3931" t="n">
+        <v>7.4999</v>
+      </c>
+      <c r="D3931" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3931" t="inlineStr">
+        <is>
+          <t>2026-10-21 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3932">
+      <c r="A3932" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B3932" t="inlineStr">
+        <is>
+          <t>EUR/COP</t>
+        </is>
+      </c>
+      <c r="C3932" t="n">
+        <v>3538.679762</v>
+      </c>
+      <c r="D3932" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3932" t="inlineStr">
+        <is>
+          <t>2026-10-21 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3933">
+      <c r="A3933" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B3933" t="inlineStr">
+        <is>
+          <t>EUR/DKK</t>
+        </is>
+      </c>
+      <c r="C3933" t="n">
+        <v>7.4746</v>
+      </c>
+      <c r="D3933" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3933" t="inlineStr">
+        <is>
+          <t>2026-10-21 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3934">
+      <c r="A3934" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B3934" t="inlineStr">
+        <is>
+          <t>EUR/GBP</t>
+        </is>
+      </c>
+      <c r="C3934" t="n">
+        <v>0.8382500000000001</v>
+      </c>
+      <c r="D3934" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3934" t="inlineStr">
+        <is>
+          <t>2026-10-21 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3935">
+      <c r="A3935" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B3935" t="inlineStr">
+        <is>
+          <t>EUR/HKD</t>
+        </is>
+      </c>
+      <c r="C3935" t="n">
+        <v>8.8155</v>
+      </c>
+      <c r="D3935" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3935" t="inlineStr">
+        <is>
+          <t>2026-10-21 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3936">
+      <c r="A3936" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B3936" t="inlineStr">
+        <is>
+          <t>EUR/IDR</t>
+        </is>
+      </c>
+      <c r="C3936" t="n">
+        <v>20269.17</v>
+      </c>
+      <c r="D3936" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3936" t="inlineStr">
+        <is>
+          <t>2026-10-21 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3937">
+      <c r="A3937" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B3937" t="inlineStr">
+        <is>
+          <t>EUR/ILS</t>
+        </is>
+      </c>
+      <c r="C3937" t="n">
+        <v>3.4726</v>
+      </c>
+      <c r="D3937" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3937" t="inlineStr">
+        <is>
+          <t>2026-10-21 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3938">
+      <c r="A3938" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B3938" t="inlineStr">
+        <is>
+          <t>EUR/JPY</t>
+        </is>
+      </c>
+      <c r="C3938" t="n">
+        <v>177.36</v>
+      </c>
+      <c r="D3938" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3938" t="inlineStr">
+        <is>
+          <t>2026-10-21 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3939">
+      <c r="A3939" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B3939" t="inlineStr">
+        <is>
+          <t>EUR/KRW</t>
+        </is>
+      </c>
+      <c r="C3939" t="n">
+        <v>1489.15</v>
+      </c>
+      <c r="D3939" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3939" t="inlineStr">
+        <is>
+          <t>2026-10-21 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3940">
+      <c r="A3940" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B3940" t="inlineStr">
+        <is>
+          <t>EUR/MAD</t>
+        </is>
+      </c>
+      <c r="C3940" t="n">
+        <v>11.001327</v>
+      </c>
+      <c r="D3940" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3940" t="inlineStr">
+        <is>
+          <t>2026-10-21 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3941">
+      <c r="A3941" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B3941" t="inlineStr">
+        <is>
+          <t>EUR/PEN</t>
+        </is>
+      </c>
+      <c r="C3941" t="n">
+        <v>3.859877</v>
+      </c>
+      <c r="D3941" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3941" t="inlineStr">
+        <is>
+          <t>2026-10-21 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3942">
+      <c r="A3942" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B3942" t="inlineStr">
+        <is>
+          <t>EUR/PHP</t>
+        </is>
+      </c>
+      <c r="C3942" t="n">
+        <v>71.121</v>
+      </c>
+      <c r="D3942" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3942" t="inlineStr">
+        <is>
+          <t>2026-10-21 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3943">
+      <c r="A3943" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B3943" t="inlineStr">
+        <is>
+          <t>EUR/RUB</t>
+        </is>
+      </c>
+      <c r="C3943" t="n">
+        <v>92.667991</v>
+      </c>
+      <c r="D3943" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3943" t="inlineStr">
+        <is>
+          <t>2026-10-21 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3944">
+      <c r="A3944" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B3944" t="inlineStr">
+        <is>
+          <t>EUR/SAR</t>
+        </is>
+      </c>
+      <c r="C3944" t="n">
+        <v>4.210069</v>
+      </c>
+      <c r="D3944" t="inlineStr">
+        <is>
+          <t>ExchangeRate-API</t>
+        </is>
+      </c>
+      <c r="E3944" t="inlineStr">
+        <is>
+          <t>2026-10-21 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3945">
+      <c r="A3945" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B3945" t="inlineStr">
+        <is>
+          <t>EUR/SEK</t>
+        </is>
+      </c>
+      <c r="C3945" t="n">
+        <v>11.0975</v>
+      </c>
+      <c r="D3945" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3945" t="inlineStr">
+        <is>
+          <t>2026-10-21 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3946">
+      <c r="A3946" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B3946" t="inlineStr">
+        <is>
+          <t>EUR/SGD</t>
+        </is>
+      </c>
+      <c r="C3946" t="n">
+        <v>1.4348</v>
+      </c>
+      <c r="D3946" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3946" t="inlineStr">
+        <is>
+          <t>2026-10-21 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3947">
+      <c r="A3947" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B3947" t="inlineStr">
+        <is>
+          <t>EUR/THB</t>
+        </is>
+      </c>
+      <c r="C3947" t="n">
+        <v>37.718</v>
+      </c>
+      <c r="D3947" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3947" t="inlineStr">
+        <is>
+          <t>2026-10-21 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3948">
+      <c r="A3948" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B3948" t="inlineStr">
+        <is>
+          <t>EUR/TRY</t>
+        </is>
+      </c>
+      <c r="C3948" t="n">
+        <v>55.7233</v>
+      </c>
+      <c r="D3948" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3948" t="inlineStr">
+        <is>
+          <t>2026-10-21 07:30 CET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3949">
+      <c r="A3949" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B3949" t="inlineStr">
+        <is>
+          <t>EUR/USD</t>
+        </is>
+      </c>
+      <c r="C3949" t="n">
+        <v>1.1234</v>
+      </c>
+      <c r="D3949" t="inlineStr">
+        <is>
+          <t>Frankfurter/ECB</t>
+        </is>
+      </c>
+      <c r="E3949" t="inlineStr">
+        <is>
+          <t>2026-10-21 07:30 CET</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>